<commit_message>
#900 Added generated property constants for i18n strings and validations
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3178" uniqueCount="1120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3178" uniqueCount="1117">
   <si>
     <t>Field</t>
   </si>
@@ -341,7 +341,7 @@
     <t>DEAD</t>
   </si>
   <si>
-    <t xml:space="preserve">Dead </t>
+    <t>Dead</t>
   </si>
   <si>
     <t>BURIED</t>
@@ -491,7 +491,7 @@
     <t>RELIGIOUS_LEADER</t>
   </si>
   <si>
-    <t xml:space="preserve">Religious leader </t>
+    <t>Religious leader</t>
   </si>
   <si>
     <t>HOUSEWIFE</t>
@@ -1007,7 +1007,7 @@
     <t>admittedToHealthFacility</t>
   </si>
   <si>
-    <t>Was patient admitted at the health facility?</t>
+    <t>Was patient admitted at the health facility as an inpatient?</t>
   </si>
   <si>
     <t>admissionDate</t>
@@ -1451,7 +1451,7 @@
     <t>Pain behind eyes/Sensitivity to light</t>
   </si>
   <si>
-    <t>Pain behind eyes or eyes sensitive to light</t>
+    <t>ain behind eyes or eyes sensitive to light</t>
   </si>
   <si>
     <t>EVD, Lassa, New flu, CSM, Measles, Dengue, Monkeypox, Other</t>
@@ -1736,9 +1736,6 @@
     <t>patientIllLocation</t>
   </si>
   <si>
-    <t>Name of the village (and country) where the patient got ill</t>
-  </si>
-  <si>
     <t>AXILLARY</t>
   </si>
   <si>
@@ -1757,9 +1754,6 @@
     <t>rectal</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes </t>
-  </si>
-  <si>
     <t>burialAttended</t>
   </si>
   <si>
@@ -2102,9 +2096,6 @@
     <t>Stream</t>
   </si>
   <si>
-    <t>Dead</t>
-  </si>
-  <si>
     <t>PROCESSED</t>
   </si>
   <si>
@@ -3389,7 +3380,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.10.0-SNAPSHOT</t>
+    <t>1.11.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -5824,10 +5815,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
@@ -5845,13 +5836,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="C3" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>17</v>
@@ -5866,13 +5857,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>17</v>
@@ -5885,16 +5876,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -5906,13 +5897,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>17</v>
@@ -5927,13 +5918,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>17</v>
@@ -5946,7 +5937,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>206</v>
@@ -5967,13 +5958,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="C9" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>17</v>
@@ -5988,13 +5979,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>921</v>
+        <v>918</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>17</v>
@@ -6009,13 +6000,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>341</v>
       </c>
       <c r="C11" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>17</v>
@@ -6028,16 +6019,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>341</v>
       </c>
       <c r="C12" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="E12"/>
       <c r="F12" s="10" t="s">
@@ -6064,13 +6055,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B15" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="C15" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -6082,10 +6073,10 @@
     <row r="16">
       <c r="A16"/>
       <c r="B16" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="C16" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -6097,10 +6088,10 @@
     <row r="17">
       <c r="A17"/>
       <c r="B17" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="C17" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="D17" t="s">
         <v>17</v>
@@ -6112,10 +6103,10 @@
     <row r="18">
       <c r="A18"/>
       <c r="B18" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="C18" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="D18" t="s">
         <v>17</v>
@@ -6127,10 +6118,10 @@
     <row r="19">
       <c r="A19"/>
       <c r="B19" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="C19" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="D19" t="s">
         <v>17</v>
@@ -6142,10 +6133,10 @@
     <row r="20">
       <c r="A20"/>
       <c r="B20" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="C20" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="D20" t="s">
         <v>17</v>
@@ -6157,7 +6148,7 @@
     <row r="21">
       <c r="A21"/>
       <c r="B21" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="C21" t="s">
         <v>332</v>
@@ -6172,10 +6163,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="C22" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="D22" t="s">
         <v>17</v>
@@ -6187,10 +6178,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="C23" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -6202,10 +6193,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="C24" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
@@ -6217,10 +6208,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="C25" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="D25" t="s">
         <v>17</v>
@@ -6232,10 +6223,10 @@
     <row r="26">
       <c r="A26"/>
       <c r="B26" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="C26" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="D26" t="s">
         <v>17</v>
@@ -6247,10 +6238,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="C27" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="D27" t="s">
         <v>17</v>
@@ -6262,10 +6253,10 @@
     <row r="28">
       <c r="A28"/>
       <c r="B28" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="C28" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
@@ -6277,10 +6268,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="C29" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="D29" t="s">
         <v>17</v>
@@ -6292,10 +6283,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="C30" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
@@ -6307,10 +6298,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="C31" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
@@ -6353,13 +6344,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="B35" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C35" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
@@ -6386,10 +6377,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="C37" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
@@ -6401,10 +6392,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="C38" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
@@ -6462,13 +6453,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="C2" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>17</v>
@@ -6483,13 +6474,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C3" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>17</v>
@@ -6502,13 +6493,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="C4" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>17</v>
@@ -6521,13 +6512,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>940</v>
+        <v>937</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>941</v>
+        <v>938</v>
       </c>
       <c r="C5" t="s">
-        <v>942</v>
+        <v>939</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>17</v>
@@ -6540,16 +6531,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>940</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>941</v>
+      </c>
+      <c r="C6" t="s">
+        <v>942</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>943</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>944</v>
-      </c>
-      <c r="C6" t="s">
-        <v>945</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>946</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -6561,13 +6552,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C7" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>17</v>
@@ -6580,13 +6571,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>17</v>
@@ -6601,13 +6592,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>17</v>
@@ -6620,13 +6611,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="C10" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>17</v>
@@ -6639,13 +6630,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>17</v>
@@ -6658,13 +6649,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>960</v>
+        <v>957</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>17</v>
@@ -6677,13 +6668,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>961</v>
+        <v>958</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>206</v>
       </c>
       <c r="C13" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>17</v>
@@ -6696,13 +6687,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>17</v>
@@ -6715,13 +6706,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>17</v>
@@ -6736,13 +6727,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>17</v>
@@ -6755,7 +6746,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>25</v>
@@ -6774,7 +6765,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>25</v>
@@ -6793,7 +6784,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>25</v>
@@ -6829,13 +6820,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="B22" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="C22" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="D22" t="s">
         <v>17</v>
@@ -6847,10 +6838,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="C23" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -6862,10 +6853,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
       <c r="C24" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
@@ -6877,10 +6868,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>978</v>
+        <v>975</v>
       </c>
       <c r="C25" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
       <c r="D25" t="s">
         <v>17</v>
@@ -6908,13 +6899,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="B28" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="C28" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
@@ -6926,10 +6917,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="C29" t="s">
-        <v>983</v>
+        <v>980</v>
       </c>
       <c r="D29" t="s">
         <v>17</v>
@@ -6941,10 +6932,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>984</v>
+        <v>981</v>
       </c>
       <c r="C30" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
@@ -6956,10 +6947,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="C31" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
@@ -6971,10 +6962,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>988</v>
+        <v>985</v>
       </c>
       <c r="C32" t="s">
-        <v>989</v>
+        <v>986</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
@@ -6986,10 +6977,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="C33" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
@@ -7001,10 +6992,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="C34" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="D34" t="s">
         <v>17</v>
@@ -7016,10 +7007,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>994</v>
+        <v>991</v>
       </c>
       <c r="C35" t="s">
-        <v>995</v>
+        <v>992</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
@@ -7031,10 +7022,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="C36" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
@@ -7046,10 +7037,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>998</v>
+        <v>995</v>
       </c>
       <c r="C37" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
@@ -7061,10 +7052,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>1000</v>
+        <v>997</v>
       </c>
       <c r="C38" t="s">
-        <v>1001</v>
+        <v>998</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
@@ -7076,10 +7067,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="C39" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
@@ -7091,10 +7082,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>1004</v>
+        <v>1001</v>
       </c>
       <c r="C40" t="s">
-        <v>1005</v>
+        <v>1002</v>
       </c>
       <c r="D40" t="s">
         <v>17</v>
@@ -7106,10 +7097,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>1006</v>
+        <v>1003</v>
       </c>
       <c r="C41" t="s">
-        <v>1007</v>
+        <v>1004</v>
       </c>
       <c r="D41" t="s">
         <v>17</v>
@@ -7121,10 +7112,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>1008</v>
+        <v>1005</v>
       </c>
       <c r="C42" t="s">
-        <v>1009</v>
+        <v>1006</v>
       </c>
       <c r="D42" t="s">
         <v>17</v>
@@ -7136,10 +7127,10 @@
     <row r="43">
       <c r="A43"/>
       <c r="B43" t="s">
-        <v>1010</v>
+        <v>1007</v>
       </c>
       <c r="C43" t="s">
-        <v>1011</v>
+        <v>1008</v>
       </c>
       <c r="D43" t="s">
         <v>17</v>
@@ -7151,10 +7142,10 @@
     <row r="44">
       <c r="A44"/>
       <c r="B44" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="C44" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
@@ -7169,7 +7160,7 @@
         <v>133</v>
       </c>
       <c r="C45" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="D45" t="s">
         <v>17</v>
@@ -7181,10 +7172,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="C46" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
       <c r="D46" t="s">
         <v>17</v>
@@ -7196,10 +7187,10 @@
     <row r="47">
       <c r="A47"/>
       <c r="B47" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="C47" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="D47" t="s">
         <v>17</v>
@@ -7211,10 +7202,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>1019</v>
+        <v>1016</v>
       </c>
       <c r="C48" t="s">
-        <v>1020</v>
+        <v>1017</v>
       </c>
       <c r="D48" t="s">
         <v>17</v>
@@ -7242,13 +7233,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="B51" t="s">
-        <v>1021</v>
+        <v>1018</v>
       </c>
       <c r="C51" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="D51" t="s">
         <v>17</v>
@@ -7260,10 +7251,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="C52" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
       <c r="D52" t="s">
         <v>17</v>
@@ -7275,10 +7266,10 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>1025</v>
+        <v>1022</v>
       </c>
       <c r="C53" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="D53" t="s">
         <v>17</v>
@@ -7306,13 +7297,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="B56" t="s">
         <v>295</v>
       </c>
       <c r="C56" t="s">
-        <v>1027</v>
+        <v>1024</v>
       </c>
       <c r="D56" t="s">
         <v>17</v>
@@ -7327,7 +7318,7 @@
         <v>298</v>
       </c>
       <c r="C57" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
       <c r="D57" t="s">
         <v>17</v>
@@ -7339,10 +7330,10 @@
     <row r="58">
       <c r="A58"/>
       <c r="B58" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="C58" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
       <c r="D58" t="s">
         <v>17</v>
@@ -7354,10 +7345,10 @@
     <row r="59">
       <c r="A59"/>
       <c r="B59" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
       <c r="C59" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="D59" t="s">
         <v>17</v>
@@ -7417,13 +7408,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="C2" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>17</v>
@@ -7438,16 +7429,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D3" s="12" t="s">
         <v>1036</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>1037</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1038</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>1039</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -7459,16 +7450,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -7480,16 +7471,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="E5"/>
       <c r="F5" s="12" t="s">
@@ -7499,7 +7490,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>39</v>
@@ -7541,13 +7532,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1046</v>
+        <v>1043</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>17</v>
@@ -7560,16 +7551,16 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>1048</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>1049</v>
-      </c>
-      <c r="C9" t="s">
-        <v>1050</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>1051</v>
       </c>
       <c r="E9"/>
       <c r="F9" s="12" t="s">
@@ -7579,16 +7570,16 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="E10"/>
       <c r="F10" s="12" t="s">
@@ -7598,16 +7589,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="E11"/>
       <c r="F11" s="12" t="s">
@@ -7617,16 +7608,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="E12"/>
       <c r="F12" s="12" t="s">
@@ -7636,16 +7627,16 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="E13"/>
       <c r="F13" s="12" t="s">
@@ -7712,13 +7703,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>1064</v>
+        <v>1061</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>17</v>
@@ -7805,13 +7796,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="B23" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="C23" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -7823,10 +7814,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="C24" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
@@ -7854,19 +7845,19 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="B27" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="C27" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="D27" t="s">
         <v>17</v>
       </c>
       <c r="E27" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="28">
@@ -7875,7 +7866,7 @@
         <v>289</v>
       </c>
       <c r="C28" t="s">
-        <v>1073</v>
+        <v>1070</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
@@ -7887,16 +7878,16 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>1074</v>
+        <v>1071</v>
       </c>
       <c r="C29" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="D29" t="s">
         <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="31">
@@ -7918,13 +7909,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="B32" t="s">
-        <v>1077</v>
+        <v>1074</v>
       </c>
       <c r="C32" t="s">
-        <v>1078</v>
+        <v>1075</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
@@ -7936,10 +7927,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>1079</v>
+        <v>1076</v>
       </c>
       <c r="C33" t="s">
-        <v>1080</v>
+        <v>1077</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
@@ -7966,10 +7957,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="C35" t="s">
-        <v>1082</v>
+        <v>1079</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
@@ -7981,10 +7972,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="C36" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
@@ -8258,13 +8249,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="C2" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>17</v>
@@ -8282,10 +8273,10 @@
         <v>198</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>1085</v>
+        <v>1082</v>
       </c>
       <c r="C3" t="s">
-        <v>1085</v>
+        <v>1082</v>
       </c>
       <c r="D3" s="13" t="s">
         <v>17</v>
@@ -8300,13 +8291,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>17</v>
@@ -8319,10 +8310,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
@@ -8383,13 +8374,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>17</v>
@@ -8484,7 +8475,7 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>1090</v>
+        <v>1087</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>17</v>
@@ -8503,7 +8494,7 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>1091</v>
+        <v>1088</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>17</v>
@@ -8516,10 +8507,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1093</v>
+        <v>1090</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
@@ -8535,7 +8526,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>341</v>
@@ -8571,13 +8562,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C13" t="s">
         <v>1093</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C13" t="s">
-        <v>1096</v>
       </c>
       <c r="D13" t="s">
         <v>17</v>
@@ -8589,10 +8580,10 @@
     <row r="14">
       <c r="A14"/>
       <c r="B14" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
       <c r="C14" t="s">
-        <v>1098</v>
+        <v>1095</v>
       </c>
       <c r="D14" t="s">
         <v>17</v>
@@ -8604,10 +8595,10 @@
     <row r="15">
       <c r="A15"/>
       <c r="B15" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
       <c r="C15" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -8619,10 +8610,10 @@
     <row r="16">
       <c r="A16"/>
       <c r="B16" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="C16" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -8679,13 +8670,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>17</v>
@@ -8698,13 +8689,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>17</v>
@@ -8717,13 +8708,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>17</v>
@@ -8736,13 +8727,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>17</v>
@@ -8800,13 +8791,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="D2" s="16" t="s">
         <v>17</v>
@@ -8819,13 +8810,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="B3" s="16" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>17</v>
@@ -8838,13 +8829,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>17</v>
@@ -8857,13 +8848,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>17</v>
@@ -8940,13 +8931,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>17</v>
@@ -9023,13 +9014,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>341</v>
       </c>
       <c r="C2" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>17</v>
@@ -9042,13 +9033,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>17</v>
@@ -9099,13 +9090,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1112</v>
+        <v>1109</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>17</v>
@@ -9156,11 +9147,11 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="D9" s="18" t="s">
         <v>17</v>
@@ -9249,13 +9240,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1115</v>
+        <v>1112</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>86</v>
       </c>
       <c r="C14" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>17</v>
@@ -9268,13 +9259,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1116</v>
+        <v>1113</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>1117</v>
+        <v>1114</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>17</v>
@@ -9300,12 +9291,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>1118</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1119</v>
+        <v>1116</v>
       </c>
     </row>
   </sheetData>
@@ -13096,7 +13087,7 @@
         <v>8</v>
       </c>
       <c r="C90" t="s">
-        <v>568</v>
+        <v>17</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>17</v>
@@ -13129,10 +13120,10 @@
         <v>355</v>
       </c>
       <c r="B93" t="s">
+        <v>568</v>
+      </c>
+      <c r="C93" t="s">
         <v>569</v>
-      </c>
-      <c r="C93" t="s">
-        <v>570</v>
       </c>
       <c r="D93" t="s">
         <v>17</v>
@@ -13144,10 +13135,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
+        <v>570</v>
+      </c>
+      <c r="C94" t="s">
         <v>571</v>
-      </c>
-      <c r="C94" t="s">
-        <v>572</v>
       </c>
       <c r="D94" t="s">
         <v>17</v>
@@ -13159,10 +13150,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
+        <v>572</v>
+      </c>
+      <c r="C95" t="s">
         <v>573</v>
-      </c>
-      <c r="C95" t="s">
-        <v>574</v>
       </c>
       <c r="D95" t="s">
         <v>17</v>
@@ -13196,7 +13187,7 @@
         <v>312</v>
       </c>
       <c r="C98" t="s">
-        <v>575</v>
+        <v>313</v>
       </c>
       <c r="D98" t="s">
         <v>17</v>
@@ -13284,16 +13275,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E2"/>
       <c r="F2" s="6" t="s">
@@ -13303,35 +13294,35 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E3"/>
       <c r="F3" s="6" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="G3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E4"/>
       <c r="F4" s="6" t="s">
@@ -13341,11 +13332,11 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>17</v>
@@ -13358,11 +13349,11 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>17</v>
@@ -13375,11 +13366,11 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>17</v>
@@ -13392,89 +13383,89 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C8" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E8"/>
       <c r="F8" s="6" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="G8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C9" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E9"/>
       <c r="F9" s="6" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C10" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E10"/>
       <c r="F10" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C11" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E11"/>
       <c r="F11" s="6" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="G11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C12" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>17</v>
@@ -13487,13 +13478,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C13" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>17</v>
@@ -13506,13 +13497,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C14" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>17</v>
@@ -13525,206 +13516,206 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C15" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E15"/>
       <c r="F15" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C16" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E16"/>
       <c r="F16" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C17" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E17"/>
       <c r="F17" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E18"/>
       <c r="F18" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E19"/>
       <c r="F19" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E20"/>
       <c r="F20" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C21" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E21"/>
       <c r="F21" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C22" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E22"/>
       <c r="F22" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E23"/>
       <c r="F23" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C24" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="E24"/>
       <c r="F24" s="6" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="G24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C25" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="E25"/>
       <c r="F25" s="6" t="s">
@@ -13734,35 +13725,35 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C26" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="E26"/>
       <c r="F26" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="G26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C27" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="E27"/>
       <c r="F27" s="6" t="s">
@@ -13772,35 +13763,35 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C28" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="E28"/>
       <c r="F28" s="6" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="G28"/>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C29" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="E29"/>
       <c r="F29" s="6" t="s">
@@ -13810,130 +13801,130 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C30" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E30"/>
       <c r="F30" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="G30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="E31"/>
       <c r="F31" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="G31"/>
     </row>
     <row r="32">
       <c r="A32" t="s">
+        <v>653</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="C32" t="s">
         <v>655</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="D32" s="6" t="s">
         <v>656</v>
-      </c>
-      <c r="C32" t="s">
-        <v>657</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>658</v>
       </c>
       <c r="E32"/>
       <c r="F32" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G32"/>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E33"/>
       <c r="F33" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C34" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E34"/>
       <c r="F34" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C35" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="E35"/>
       <c r="F35" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G35"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C36" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="E36"/>
       <c r="F36" s="6" t="s">
@@ -13943,16 +13934,16 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>235</v>
       </c>
       <c r="C37" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E37"/>
       <c r="F37" s="6" t="s">
@@ -13962,13 +13953,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>17</v>
@@ -13981,13 +13972,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C39" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>17</v>
@@ -14000,13 +13991,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>677</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="C40" t="s">
         <v>679</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>680</v>
-      </c>
-      <c r="C40" t="s">
-        <v>681</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>17</v>
@@ -14100,13 +14091,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B48" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C48" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="D48" t="s">
         <v>17</v>
@@ -14118,10 +14109,10 @@
     <row r="49">
       <c r="A49"/>
       <c r="B49" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C49" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="D49" t="s">
         <v>17</v>
@@ -14133,10 +14124,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C50" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="D50" t="s">
         <v>17</v>
@@ -14148,10 +14139,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C51" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D51" t="s">
         <v>17</v>
@@ -14194,7 +14185,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B55" t="s">
         <v>100</v>
@@ -14215,7 +14206,7 @@
         <v>102</v>
       </c>
       <c r="C56" t="s">
-        <v>690</v>
+        <v>103</v>
       </c>
       <c r="D56" t="s">
         <v>17</v>
@@ -14227,10 +14218,10 @@
     <row r="57">
       <c r="A57"/>
       <c r="B57" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="C57" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="D57" t="s">
         <v>17</v>
@@ -14304,13 +14295,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>17</v>
@@ -14409,7 +14400,7 @@
         <v>199</v>
       </c>
       <c r="C7" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>17</v>
@@ -14424,13 +14415,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C8" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>17</v>
@@ -14445,13 +14436,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>17</v>
@@ -14464,13 +14455,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>17</v>
@@ -14483,16 +14474,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>700</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="C11" t="s">
+        <v>702</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>703</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>704</v>
-      </c>
-      <c r="C11" t="s">
-        <v>705</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>706</v>
       </c>
       <c r="E11"/>
       <c r="F11" s="7" t="s">
@@ -14502,13 +14493,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C12" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>17</v>
@@ -14521,13 +14512,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C13" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>17</v>
@@ -14540,89 +14531,89 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>710</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>711</v>
+      </c>
+      <c r="C14" t="s">
+        <v>712</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>713</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>714</v>
-      </c>
-      <c r="C14" t="s">
-        <v>715</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>716</v>
       </c>
       <c r="E14"/>
       <c r="F14" s="7" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E15"/>
       <c r="F15" s="7" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E16"/>
       <c r="F16" s="7" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>206</v>
       </c>
       <c r="C17" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E17"/>
       <c r="F17" s="7" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>17</v>
@@ -14635,16 +14626,16 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>723</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="C19" t="s">
+        <v>725</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>726</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>727</v>
-      </c>
-      <c r="C19" t="s">
-        <v>728</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>729</v>
       </c>
       <c r="E19"/>
       <c r="F19" s="7" t="s">
@@ -14654,13 +14645,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C20" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>17</v>
@@ -14673,13 +14664,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>206</v>
       </c>
       <c r="C21" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>17</v>
@@ -14893,13 +14884,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="B37" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="C37" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
@@ -14911,10 +14902,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="C38" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
@@ -14926,10 +14917,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="C39" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
@@ -14941,10 +14932,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="C40" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="D40" t="s">
         <v>17</v>
@@ -14956,10 +14947,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="C41" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="D41" t="s">
         <v>17</v>
@@ -14987,19 +14978,19 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="B44" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="C44" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
       </c>
       <c r="E44" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
     </row>
     <row r="45">
@@ -15008,7 +14999,7 @@
         <v>289</v>
       </c>
       <c r="C45" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="D45" t="s">
         <v>17</v>
@@ -15020,16 +15011,16 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="C46" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="D46" t="s">
         <v>17</v>
       </c>
       <c r="E46" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
     </row>
     <row r="48">
@@ -15051,13 +15042,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="B49" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="C49" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="D49" t="s">
         <v>17</v>
@@ -15069,10 +15060,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="C50" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="D50" t="s">
         <v>17</v>
@@ -15084,10 +15075,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="C51" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="D51" t="s">
         <v>17</v>
@@ -15115,76 +15106,76 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="B54" t="s">
+        <v>754</v>
+      </c>
+      <c r="C54" t="s">
+        <v>755</v>
+      </c>
+      <c r="D54" t="s">
+        <v>756</v>
+      </c>
+      <c r="E54" t="s">
         <v>757</v>
-      </c>
-      <c r="C54" t="s">
-        <v>758</v>
-      </c>
-      <c r="D54" t="s">
-        <v>759</v>
-      </c>
-      <c r="E54" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="55">
       <c r="A55"/>
       <c r="B55" t="s">
+        <v>758</v>
+      </c>
+      <c r="C55" t="s">
+        <v>759</v>
+      </c>
+      <c r="D55" t="s">
+        <v>760</v>
+      </c>
+      <c r="E55" t="s">
         <v>761</v>
-      </c>
-      <c r="C55" t="s">
-        <v>762</v>
-      </c>
-      <c r="D55" t="s">
-        <v>763</v>
-      </c>
-      <c r="E55" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="56">
       <c r="A56"/>
       <c r="B56" t="s">
+        <v>762</v>
+      </c>
+      <c r="C56" t="s">
+        <v>763</v>
+      </c>
+      <c r="D56" t="s">
+        <v>764</v>
+      </c>
+      <c r="E56" t="s">
         <v>765</v>
-      </c>
-      <c r="C56" t="s">
-        <v>766</v>
-      </c>
-      <c r="D56" t="s">
-        <v>767</v>
-      </c>
-      <c r="E56" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="57">
       <c r="A57"/>
       <c r="B57" t="s">
+        <v>766</v>
+      </c>
+      <c r="C57" t="s">
+        <v>767</v>
+      </c>
+      <c r="D57" t="s">
+        <v>768</v>
+      </c>
+      <c r="E57" t="s">
         <v>769</v>
-      </c>
-      <c r="C57" t="s">
-        <v>770</v>
-      </c>
-      <c r="D57" t="s">
-        <v>771</v>
-      </c>
-      <c r="E57" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="58">
       <c r="A58"/>
       <c r="B58" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C58" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="D58" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="E58" t="s">
         <v>17</v>
@@ -15209,13 +15200,13 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="B61" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="C61" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="D61" t="s">
         <v>17</v>
@@ -15227,10 +15218,10 @@
     <row r="62">
       <c r="A62"/>
       <c r="B62" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="C62" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="D62" t="s">
         <v>17</v>
@@ -15242,10 +15233,10 @@
     <row r="63">
       <c r="A63"/>
       <c r="B63" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="C63" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="D63" t="s">
         <v>17</v>
@@ -15257,10 +15248,10 @@
     <row r="64">
       <c r="A64"/>
       <c r="B64" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="C64" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="D64" t="s">
         <v>17</v>
@@ -15343,7 +15334,7 @@
         <v>199</v>
       </c>
       <c r="C2" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>17</v>
@@ -15377,16 +15368,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -15398,13 +15389,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>206</v>
       </c>
       <c r="C5" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>17</v>
@@ -15419,16 +15410,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>787</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>788</v>
+      </c>
+      <c r="C6" t="s">
+        <v>789</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>790</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>791</v>
-      </c>
-      <c r="C6" t="s">
-        <v>792</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>793</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -15440,16 +15431,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="E7"/>
       <c r="F7" s="8" t="s">
@@ -15736,13 +15727,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B27" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="C27" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="D27" t="s">
         <v>17</v>
@@ -15754,31 +15745,31 @@
     <row r="28">
       <c r="A28"/>
       <c r="B28" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C28" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
       </c>
       <c r="E28" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="C29" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="D29" t="s">
         <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
     </row>
   </sheetData>
@@ -15830,13 +15821,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C2" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>17</v>
@@ -15851,13 +15842,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>17</v>
@@ -15870,13 +15861,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>17</v>
@@ -15889,16 +15880,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -15910,7 +15901,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>39</v>
@@ -16009,13 +16000,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="C11" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>17</v>
@@ -16030,13 +16021,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>17</v>
@@ -16049,13 +16040,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>17</v>
@@ -16070,13 +16061,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>17</v>
@@ -16089,13 +16080,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>17</v>
@@ -16108,13 +16099,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>17</v>
@@ -16127,13 +16118,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>17</v>
@@ -16146,13 +16137,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="C18" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>17</v>
@@ -16165,13 +16156,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>17</v>
@@ -16184,13 +16175,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>17</v>
@@ -16203,13 +16194,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="C21" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>17</v>
@@ -16222,13 +16213,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="C22" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>17</v>
@@ -16241,10 +16232,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="C23" t="s">
         <v>17</v>
@@ -16260,13 +16251,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>341</v>
       </c>
       <c r="C24" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>17</v>
@@ -16279,13 +16270,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>341</v>
       </c>
       <c r="C25" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>17</v>
@@ -16315,13 +16306,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="B28" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="C28" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
@@ -16333,10 +16324,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="C29" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="D29" t="s">
         <v>17</v>
@@ -16348,10 +16339,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="C30" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
@@ -16363,10 +16354,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="C31" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
@@ -16378,10 +16369,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="C32" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
@@ -16393,10 +16384,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="C33" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
@@ -16408,10 +16399,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="C34" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="D34" t="s">
         <v>17</v>
@@ -16423,10 +16414,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="C35" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
@@ -16438,10 +16429,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="C36" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
@@ -16484,13 +16475,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="B40" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="C40" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="D40" t="s">
         <v>17</v>
@@ -16502,10 +16493,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="C41" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="D41" t="s">
         <v>17</v>
@@ -16533,13 +16524,13 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="B44" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="C44" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
@@ -16551,10 +16542,10 @@
     <row r="45">
       <c r="A45"/>
       <c r="B45" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="C45" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
       <c r="D45" t="s">
         <v>17</v>
@@ -16566,10 +16557,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="C46" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="D46" t="s">
         <v>17</v>
@@ -16597,13 +16588,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B49" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="C49" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="D49" t="s">
         <v>17</v>
@@ -16615,10 +16606,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="C50" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="D50" t="s">
         <v>17</v>
@@ -16630,10 +16621,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="C51" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="D51" t="s">
         <v>17</v>
@@ -16645,10 +16636,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="C52" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="D52" t="s">
         <v>17</v>
@@ -16660,10 +16651,10 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="C53" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="D53" t="s">
         <v>17</v>
@@ -16675,10 +16666,10 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="C54" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="D54" t="s">
         <v>17</v>
@@ -16690,7 +16681,7 @@
     <row r="55">
       <c r="A55"/>
       <c r="B55" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="C55" t="s">
         <v>332</v>
@@ -16705,10 +16696,10 @@
     <row r="56">
       <c r="A56"/>
       <c r="B56" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="C56" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="D56" t="s">
         <v>17</v>
@@ -16720,10 +16711,10 @@
     <row r="57">
       <c r="A57"/>
       <c r="B57" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="C57" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="D57" t="s">
         <v>17</v>
@@ -16735,10 +16726,10 @@
     <row r="58">
       <c r="A58"/>
       <c r="B58" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="C58" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="D58" t="s">
         <v>17</v>
@@ -16750,10 +16741,10 @@
     <row r="59">
       <c r="A59"/>
       <c r="B59" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="C59" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="D59" t="s">
         <v>17</v>
@@ -16765,10 +16756,10 @@
     <row r="60">
       <c r="A60"/>
       <c r="B60" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="C60" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="D60" t="s">
         <v>17</v>
@@ -16780,10 +16771,10 @@
     <row r="61">
       <c r="A61"/>
       <c r="B61" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="C61" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="D61" t="s">
         <v>17</v>
@@ -16795,10 +16786,10 @@
     <row r="62">
       <c r="A62"/>
       <c r="B62" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="C62" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="D62" t="s">
         <v>17</v>
@@ -16810,10 +16801,10 @@
     <row r="63">
       <c r="A63"/>
       <c r="B63" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="C63" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="D63" t="s">
         <v>17</v>
@@ -16825,10 +16816,10 @@
     <row r="64">
       <c r="A64"/>
       <c r="B64" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="C64" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="D64" t="s">
         <v>17</v>
@@ -16840,10 +16831,10 @@
     <row r="65">
       <c r="A65"/>
       <c r="B65" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="C65" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="D65" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
#1774 Separated address fields on Case and Contact detailed export
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -3787,6 +3787,30 @@
     <t>Attending clinician</t>
   </si>
   <si>
+    <t>caze</t>
+  </si>
+  <si>
+    <t>CaseReference</t>
+  </si>
+  <si>
+    <t>Source case</t>
+  </si>
+  <si>
+    <t>caseIdExternalSystem</t>
+  </si>
+  <si>
+    <t>Case ID in external system</t>
+  </si>
+  <si>
+    <t>caseOrEventInformation</t>
+  </si>
+  <si>
+    <t>Case or event information</t>
+  </si>
+  <si>
+    <t>Disease of source case</t>
+  </si>
+  <si>
     <t>reportDateTime</t>
   </si>
   <si>
@@ -3802,117 +3826,141 @@
     <t>Responsible district</t>
   </si>
   <si>
+    <t>lastContactDate</t>
+  </si>
+  <si>
+    <t>Date of last contact</t>
+  </si>
+  <si>
+    <t>contactProximity</t>
+  </si>
+  <si>
+    <t>ContactProximity</t>
+  </si>
+  <si>
+    <t>Type of contact - if multiple pick the closest contact proximity</t>
+  </si>
+  <si>
+    <t>Select the type of contact with the case</t>
+  </si>
+  <si>
+    <t>contactProximityDetails</t>
+  </si>
+  <si>
+    <t>Additional information on the type of contact</t>
+  </si>
+  <si>
+    <t>contactCategory</t>
+  </si>
+  <si>
+    <t>ContactCategory</t>
+  </si>
+  <si>
+    <t>Contact Category</t>
+  </si>
+  <si>
+    <t>contactClassification</t>
+  </si>
+  <si>
+    <t>ContactClassification</t>
+  </si>
+  <si>
+    <t>Contact classification</t>
+  </si>
+  <si>
+    <t>contactStatus</t>
+  </si>
+  <si>
+    <t>ContactStatus</t>
+  </si>
+  <si>
+    <t>Contact status</t>
+  </si>
+  <si>
+    <t>followUpStatus</t>
+  </si>
+  <si>
+    <t>FollowUpStatus</t>
+  </si>
+  <si>
+    <t>Follow-up status</t>
+  </si>
+  <si>
+    <t>&lt;ul&gt;&lt;li&gt;Under follow-up: The follow-up process is running.&lt;/li&gt;&lt;li&gt;Follow-up completed: The follow-up has been completed.&lt;/li&gt;&lt;li&gt;Follow-up canceled: The follow-up process has been canceled, e.g. because the person died or the contact became irrelevant.&lt;/li&gt;&lt;li&gt;Lost to follow-up: The follow-up process could not be continued, e.g. because the person could not be found.&lt;/li&gt;&lt;li&gt;No follow-up: No contact follow-up is being done.&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t>followUpComment</t>
+  </si>
+  <si>
+    <t>Follow-up status comment</t>
+  </si>
+  <si>
+    <t>followUpUntil</t>
+  </si>
+  <si>
+    <t>Follow-up until</t>
+  </si>
+  <si>
+    <t>overwriteFollowUpUntil</t>
+  </si>
+  <si>
+    <t>Overwrite follow-up until date</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Description of how contact took place</t>
+  </si>
+  <si>
+    <t>relationToCase</t>
+  </si>
+  <si>
+    <t>ContactRelation</t>
+  </si>
+  <si>
+    <t>Relationship with case</t>
+  </si>
+  <si>
+    <t>Select the person's relation to the case</t>
+  </si>
+  <si>
+    <t>relationDescription</t>
+  </si>
+  <si>
+    <t>Relationship description</t>
+  </si>
+  <si>
+    <t>highPriority</t>
+  </si>
+  <si>
+    <t>High priority contact</t>
+  </si>
+  <si>
+    <t>immunosuppressiveTherapyBasicDisease</t>
+  </si>
+  <si>
+    <t>Immunosuppressive therapy or basic disease is present</t>
+  </si>
+  <si>
+    <t>immunosuppressiveTherapyBasicDiseaseDetails</t>
+  </si>
+  <si>
+    <t>careForPeopleOver60</t>
+  </si>
+  <si>
+    <t>Is the person medically/nursingly active in the care of patients or people over 60 years of age?</t>
+  </si>
+  <si>
     <t>Contact person</t>
   </si>
   <si>
-    <t>caze</t>
-  </si>
-  <si>
-    <t>CaseReference</t>
-  </si>
-  <si>
-    <t>Source case</t>
-  </si>
-  <si>
-    <t>Disease of source case</t>
-  </si>
-  <si>
-    <t>lastContactDate</t>
-  </si>
-  <si>
-    <t>Date of last contact</t>
-  </si>
-  <si>
-    <t>contactProximity</t>
-  </si>
-  <si>
-    <t>ContactProximity</t>
-  </si>
-  <si>
-    <t>Type of contact - if multiple pick the closest contact proximity</t>
-  </si>
-  <si>
-    <t>Select the type of contact with the case</t>
-  </si>
-  <si>
-    <t>contactClassification</t>
-  </si>
-  <si>
-    <t>ContactClassification</t>
-  </si>
-  <si>
-    <t>Contact classification</t>
-  </si>
-  <si>
-    <t>contactStatus</t>
-  </si>
-  <si>
-    <t>ContactStatus</t>
-  </si>
-  <si>
-    <t>Contact status</t>
-  </si>
-  <si>
-    <t>followUpStatus</t>
-  </si>
-  <si>
-    <t>FollowUpStatus</t>
-  </si>
-  <si>
-    <t>Follow-up status</t>
-  </si>
-  <si>
-    <t>&lt;ul&gt;&lt;li&gt;Under follow-up: The follow-up process is running.&lt;/li&gt;&lt;li&gt;Follow-up completed: The follow-up has been completed.&lt;/li&gt;&lt;li&gt;Follow-up canceled: The follow-up process has been canceled, e.g. because the person died or the contact became irrelevant.&lt;/li&gt;&lt;li&gt;Lost to follow-up: The follow-up process could not be continued, e.g. because the person could not be found.&lt;/li&gt;&lt;li&gt;No follow-up: No contact follow-up is being done.&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t>followUpComment</t>
-  </si>
-  <si>
-    <t>Follow-up status comment</t>
-  </si>
-  <si>
-    <t>followUpUntil</t>
-  </si>
-  <si>
-    <t>Follow-up until</t>
-  </si>
-  <si>
-    <t>overwriteFollowUpUntil</t>
-  </si>
-  <si>
-    <t>Overwrite follow-up until date</t>
-  </si>
-  <si>
     <t>contactOfficer</t>
   </si>
   <si>
     <t>Responsible contact officer</t>
   </si>
   <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>Description of how contact took place</t>
-  </si>
-  <si>
-    <t>relationToCase</t>
-  </si>
-  <si>
-    <t>ContactRelation</t>
-  </si>
-  <si>
-    <t>Relationship with case</t>
-  </si>
-  <si>
-    <t>Select the person's relation to the case</t>
-  </si>
-  <si>
-    <t>relationDescription</t>
-  </si>
-  <si>
-    <t>Relationship description</t>
-  </si>
-  <si>
     <t>resultingCase</t>
   </si>
   <si>
@@ -3925,54 +3973,6 @@
     <t>Resulting case assigned by</t>
   </si>
   <si>
-    <t>highPriority</t>
-  </si>
-  <si>
-    <t>High priority contact</t>
-  </si>
-  <si>
-    <t>immunosuppressiveTherapyBasicDisease</t>
-  </si>
-  <si>
-    <t>Immunosuppressive therapy or basic disease is present</t>
-  </si>
-  <si>
-    <t>immunosuppressiveTherapyBasicDiseaseDetails</t>
-  </si>
-  <si>
-    <t>careForPeopleOver60</t>
-  </si>
-  <si>
-    <t>Is the person medically/nursingly active in the care of patients or people over 60 years of age?</t>
-  </si>
-  <si>
-    <t>caseIdExternalSystem</t>
-  </si>
-  <si>
-    <t>Case ID in external system</t>
-  </si>
-  <si>
-    <t>caseOrEventInformation</t>
-  </si>
-  <si>
-    <t>Case or event information</t>
-  </si>
-  <si>
-    <t>contactProximityDetails</t>
-  </si>
-  <si>
-    <t>Additional information on the type of contact</t>
-  </si>
-  <si>
-    <t>contactCategory</t>
-  </si>
-  <si>
-    <t>ContactCategory</t>
-  </si>
-  <si>
-    <t>Contact Category</t>
-  </si>
-  <si>
     <t>TOUCHED_FLUID</t>
   </si>
   <si>
@@ -4051,6 +4051,24 @@
     <t>Medical personnel at save proximity (&gt; 2 meter), without direct contact with secretions or excretions of the patient and without aerosol exposure</t>
   </si>
   <si>
+    <t>HIGH_RISK</t>
+  </si>
+  <si>
+    <t>High risk contact</t>
+  </si>
+  <si>
+    <t>LOW_RISK</t>
+  </si>
+  <si>
+    <t>Low risk contact</t>
+  </si>
+  <si>
+    <t>NO_RISK</t>
+  </si>
+  <si>
+    <t>No risk contact</t>
+  </si>
+  <si>
     <t>UNCONFIRMED</t>
   </si>
   <si>
@@ -4171,24 +4189,6 @@
     <t>Provided medical care for the case</t>
   </si>
   <si>
-    <t>HIGH_RISK</t>
-  </si>
-  <si>
-    <t>High risk contact</t>
-  </si>
-  <si>
-    <t>LOW_RISK</t>
-  </si>
-  <si>
-    <t>Low risk contact</t>
-  </si>
-  <si>
-    <t>NO_RISK</t>
-  </si>
-  <si>
-    <t>No risk contact</t>
-  </si>
-  <si>
     <t>Visited person</t>
   </si>
   <si>
@@ -5473,7 +5473,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.37.0-SNAPSHOT</t>
+    <t>1.38.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -6319,7 +6319,7 @@
 </file>
 
 <file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="ContactContactClassification" displayName="ContactContactClassification" ref="A113:E116">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="ContactContactCategory" displayName="ContactContactCategory" ref="A113:E116">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6333,7 +6333,7 @@
 </file>
 
 <file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="ContactContactStatus" displayName="ContactContactStatus" ref="A118:E121">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="ContactContactClassification" displayName="ContactContactClassification" ref="A118:E121">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6347,7 +6347,7 @@
 </file>
 
 <file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="ContactFollowUpStatus" displayName="ContactFollowUpStatus" ref="A123:E128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="ContactContactStatus" displayName="ContactContactStatus" ref="A123:E126">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6361,7 +6361,7 @@
 </file>
 
 <file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="ContactContactRelation" displayName="ContactContactRelation" ref="A130:E135">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="ContactFollowUpStatus" displayName="ContactFollowUpStatus" ref="A128:E133">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6375,7 +6375,7 @@
 </file>
 
 <file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ContactYesNoUnknown" displayName="ContactYesNoUnknown" ref="A137:E140">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ContactContactRelation" displayName="ContactContactRelation" ref="A135:E140">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6403,7 +6403,7 @@
 </file>
 
 <file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ContactQuarantineType" displayName="ContactQuarantineType" ref="A142:E146">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ContactYesNoUnknown" displayName="ContactYesNoUnknown" ref="A142:E145">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6417,7 +6417,7 @@
 </file>
 
 <file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ContactContactCategory" displayName="ContactContactCategory" ref="A148:E151">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ContactQuarantineType" displayName="ContactQuarantineType" ref="A147:E151">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -10546,17 +10546,15 @@
         <v>1250</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>39</v>
+        <v>1251</v>
       </c>
       <c r="C2" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
+      <c r="E2"/>
       <c r="G2" s="11" t="s">
         <v>12</v>
       </c>
@@ -10564,20 +10562,18 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>363</v>
+        <v>1253</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>364</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>365</v>
+        <v>1254</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
+      <c r="E3"/>
       <c r="G3" s="11" t="s">
         <v>12</v>
       </c>
@@ -10585,13 +10581,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>439</v>
+        <v>1255</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>1256</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>18</v>
@@ -10604,13 +10600,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>442</v>
+        <v>343</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>1257</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>18</v>
@@ -10623,13 +10619,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>445</v>
+        <v>345</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>346</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>18</v>
@@ -10642,18 +10638,20 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>312</v>
+        <v>1258</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>1252</v>
+        <v>1259</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>1253</v>
-      </c>
-      <c r="E7"/>
+        <v>18</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
       <c r="G7" s="11" t="s">
         <v>12</v>
       </c>
@@ -10661,18 +10659,20 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>314</v>
+        <v>363</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>46</v>
+        <v>364</v>
       </c>
       <c r="C8" t="s">
-        <v>1254</v>
+        <v>365</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>1253</v>
-      </c>
-      <c r="E8"/>
+        <v>18</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
       <c r="G8" s="11" t="s">
         <v>12</v>
       </c>
@@ -10680,20 +10680,18 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>356</v>
+        <v>439</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>357</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>1255</v>
+        <v>18</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E9" t="b">
-        <v>1</v>
-      </c>
+      <c r="E9"/>
       <c r="G9" s="11" t="s">
         <v>12</v>
       </c>
@@ -10701,20 +10699,18 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1256</v>
+        <v>442</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1257</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>1258</v>
+        <v>18</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
+      <c r="E10"/>
       <c r="G10" s="11" t="s">
         <v>12</v>
       </c>
@@ -10722,13 +10718,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>343</v>
+        <v>445</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>1259</v>
+        <v>18</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>18</v>
@@ -10741,16 +10737,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>345</v>
+        <v>312</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>346</v>
+        <v>1260</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>18</v>
+        <v>1261</v>
       </c>
       <c r="E12"/>
       <c r="G12" s="11" t="s">
@@ -10760,16 +10756,16 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1260</v>
+        <v>314</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
+        <v>1262</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>1261</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="E13"/>
       <c r="G13" s="11" t="s">
@@ -10779,18 +10775,20 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1263</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>1264</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>1265</v>
-      </c>
-      <c r="E14"/>
+        <v>18</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
       <c r="G14" s="11" t="s">
         <v>12</v>
       </c>
@@ -10798,16 +10796,16 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>1266</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="C15" t="s">
         <v>1267</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="11" t="s">
         <v>1268</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="E15"/>
       <c r="G15" s="11" t="s">
@@ -10820,10 +10818,10 @@
         <v>1269</v>
       </c>
       <c r="B16" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
         <v>1270</v>
-      </c>
-      <c r="C16" t="s">
-        <v>1271</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>18</v>
@@ -10836,16 +10834,16 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B17" s="11" t="s">
         <v>1272</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="C17" t="s">
         <v>1273</v>
       </c>
-      <c r="C17" t="s">
-        <v>1274</v>
-      </c>
       <c r="D17" s="11" t="s">
-        <v>1275</v>
+        <v>18</v>
       </c>
       <c r="E17"/>
       <c r="G17" s="11" t="s">
@@ -10855,13 +10853,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C18" t="s">
         <v>1276</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
-        <v>1277</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>18</v>
@@ -10874,10 +10872,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>1278</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="C19" t="s">
         <v>1279</v>
@@ -10896,13 +10894,13 @@
         <v>1280</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>480</v>
+        <v>1281</v>
       </c>
       <c r="C20" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>18</v>
+        <v>1283</v>
       </c>
       <c r="E20"/>
       <c r="G20" s="11" t="s">
@@ -10912,13 +10910,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>1282</v>
+        <v>1284</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>364</v>
+        <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>1283</v>
+        <v>1285</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>18</v>
@@ -10931,13 +10929,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>1284</v>
+        <v>1286</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>1285</v>
+        <v>1287</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>18</v>
@@ -10950,16 +10948,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>1286</v>
+        <v>1288</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>1287</v>
+        <v>480</v>
       </c>
       <c r="C23" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>1289</v>
+        <v>18</v>
       </c>
       <c r="E23"/>
       <c r="G23" s="11" t="s">
@@ -10988,16 +10986,16 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>477</v>
+        <v>1292</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>9</v>
+        <v>1293</v>
       </c>
       <c r="C25" t="s">
-        <v>478</v>
+        <v>1294</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>18</v>
+        <v>1295</v>
       </c>
       <c r="E25"/>
       <c r="G25" s="11" t="s">
@@ -11007,13 +11005,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>1292</v>
+        <v>1296</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>1257</v>
+        <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>1293</v>
+        <v>1297</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>18</v>
@@ -11026,13 +11024,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>1294</v>
+        <v>477</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>364</v>
+        <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>1295</v>
+        <v>478</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>18</v>
@@ -11045,13 +11043,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>480</v>
       </c>
       <c r="C28" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>18</v>
@@ -11064,13 +11062,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>393</v>
       </c>
       <c r="C29" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>18</v>
@@ -11083,7 +11081,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>9</v>
@@ -11102,13 +11100,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>393</v>
       </c>
       <c r="C31" t="s">
-        <v>1302</v>
+        <v>1304</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>18</v>
@@ -11178,18 +11176,20 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>1303</v>
+        <v>356</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="C35" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E35"/>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
       <c r="G35" s="11" t="s">
         <v>12</v>
       </c>
@@ -11197,13 +11197,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>9</v>
+        <v>364</v>
       </c>
       <c r="C36" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>18</v>
@@ -11216,13 +11216,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>9</v>
+        <v>1251</v>
       </c>
       <c r="C37" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="D37" s="11" t="s">
         <v>18</v>
@@ -11235,10 +11235,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>1310</v>
+        <v>364</v>
       </c>
       <c r="C38" t="s">
         <v>1311</v>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="B99" t="s">
         <v>1312</v>
@@ -12344,7 +12344,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>1267</v>
+        <v>1272</v>
       </c>
       <c r="B114" t="s">
         <v>1338</v>
@@ -12356,13 +12356,13 @@
         <v>18</v>
       </c>
       <c r="E114" t="s">
-        <v>1340</v>
+        <v>18</v>
       </c>
     </row>
     <row r="115">
       <c r="A115"/>
       <c r="B115" t="s">
-        <v>513</v>
+        <v>1340</v>
       </c>
       <c r="C115" t="s">
         <v>1341</v>
@@ -12371,7 +12371,7 @@
         <v>18</v>
       </c>
       <c r="E115" t="s">
-        <v>515</v>
+        <v>18</v>
       </c>
     </row>
     <row r="116">
@@ -12386,7 +12386,7 @@
         <v>18</v>
       </c>
       <c r="E116" t="s">
-        <v>1344</v>
+        <v>18</v>
       </c>
     </row>
     <row r="118">
@@ -12408,49 +12408,49 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>1270</v>
+        <v>1275</v>
       </c>
       <c r="B119" t="s">
+        <v>1344</v>
+      </c>
+      <c r="C119" t="s">
         <v>1345</v>
       </c>
-      <c r="C119" t="s">
+      <c r="D119" t="s">
+        <v>18</v>
+      </c>
+      <c r="E119" t="s">
         <v>1346</v>
-      </c>
-      <c r="D119" t="s">
-        <v>18</v>
-      </c>
-      <c r="E119" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="120">
       <c r="A120"/>
       <c r="B120" t="s">
+        <v>513</v>
+      </c>
+      <c r="C120" t="s">
         <v>1347</v>
       </c>
-      <c r="C120" t="s">
-        <v>1348</v>
-      </c>
       <c r="D120" t="s">
         <v>18</v>
       </c>
       <c r="E120" t="s">
-        <v>18</v>
+        <v>515</v>
       </c>
     </row>
     <row r="121">
       <c r="A121"/>
       <c r="B121" t="s">
+        <v>1348</v>
+      </c>
+      <c r="C121" t="s">
         <v>1349</v>
       </c>
-      <c r="C121" t="s">
+      <c r="D121" t="s">
+        <v>18</v>
+      </c>
+      <c r="E121" t="s">
         <v>1350</v>
-      </c>
-      <c r="D121" t="s">
-        <v>18</v>
-      </c>
-      <c r="E121" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="123">
@@ -12472,7 +12472,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>1273</v>
+        <v>1278</v>
       </c>
       <c r="B124" t="s">
         <v>1351</v>
@@ -12481,192 +12481,192 @@
         <v>1352</v>
       </c>
       <c r="D124" t="s">
-        <v>1353</v>
+        <v>18</v>
       </c>
       <c r="E124" t="s">
-        <v>1354</v>
+        <v>18</v>
       </c>
     </row>
     <row r="125">
       <c r="A125"/>
       <c r="B125" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="C125" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="D125" t="s">
-        <v>1357</v>
+        <v>18</v>
       </c>
       <c r="E125" t="s">
-        <v>1358</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126">
       <c r="A126"/>
       <c r="B126" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C126" t="s">
+        <v>1356</v>
+      </c>
+      <c r="D126" t="s">
+        <v>18</v>
+      </c>
+      <c r="E126" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>1</v>
+      </c>
+      <c r="B128" t="s">
+        <v>123</v>
+      </c>
+      <c r="C128" t="s">
+        <v>2</v>
+      </c>
+      <c r="D128" t="s">
+        <v>3</v>
+      </c>
+      <c r="E128" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B129" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1358</v>
+      </c>
+      <c r="D129" t="s">
         <v>1359</v>
       </c>
-      <c r="C126" t="s">
+      <c r="E129" t="s">
         <v>1360</v>
       </c>
-      <c r="D126" t="s">
+    </row>
+    <row r="130">
+      <c r="A130"/>
+      <c r="B130" t="s">
         <v>1361</v>
       </c>
-      <c r="E126" t="s">
+      <c r="C130" t="s">
         <v>1362</v>
       </c>
-    </row>
-    <row r="127">
-      <c r="A127"/>
-      <c r="B127" t="s">
+      <c r="D130" t="s">
         <v>1363</v>
       </c>
-      <c r="C127" t="s">
+      <c r="E130" t="s">
         <v>1364</v>
       </c>
-      <c r="D127" t="s">
+    </row>
+    <row r="131">
+      <c r="A131"/>
+      <c r="B131" t="s">
         <v>1365</v>
       </c>
-      <c r="E127" t="s">
+      <c r="C131" t="s">
         <v>1366</v>
       </c>
-    </row>
-    <row r="128">
-      <c r="A128"/>
-      <c r="B128" t="s">
+      <c r="D131" t="s">
         <v>1367</v>
       </c>
-      <c r="C128" t="s">
+      <c r="E131" t="s">
         <v>1368</v>
-      </c>
-      <c r="D128" t="s">
-        <v>1369</v>
-      </c>
-      <c r="E128" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="s">
-        <v>1</v>
-      </c>
-      <c r="B130" t="s">
-        <v>123</v>
-      </c>
-      <c r="C130" t="s">
-        <v>2</v>
-      </c>
-      <c r="D130" t="s">
-        <v>3</v>
-      </c>
-      <c r="E130" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="s">
-        <v>1287</v>
-      </c>
-      <c r="B131" t="s">
-        <v>1370</v>
-      </c>
-      <c r="C131" t="s">
-        <v>1371</v>
-      </c>
-      <c r="D131" t="s">
-        <v>18</v>
-      </c>
-      <c r="E131" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="132">
       <c r="A132"/>
       <c r="B132" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C132" t="s">
+        <v>1370</v>
+      </c>
+      <c r="D132" t="s">
+        <v>1371</v>
+      </c>
+      <c r="E132" t="s">
         <v>1372</v>
-      </c>
-      <c r="C132" t="s">
-        <v>1373</v>
-      </c>
-      <c r="D132" t="s">
-        <v>18</v>
-      </c>
-      <c r="E132" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="133">
       <c r="A133"/>
       <c r="B133" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C133" t="s">
         <v>1374</v>
       </c>
-      <c r="C133" t="s">
+      <c r="D133" t="s">
         <v>1375</v>
       </c>
-      <c r="D133" t="s">
-        <v>18</v>
-      </c>
       <c r="E133" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134"/>
-      <c r="B134" t="s">
+    <row r="135">
+      <c r="A135" t="s">
+        <v>1</v>
+      </c>
+      <c r="B135" t="s">
+        <v>123</v>
+      </c>
+      <c r="C135" t="s">
+        <v>2</v>
+      </c>
+      <c r="D135" t="s">
+        <v>3</v>
+      </c>
+      <c r="E135" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B136" t="s">
         <v>1376</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C136" t="s">
         <v>1377</v>
       </c>
-      <c r="D134" t="s">
-        <v>18</v>
-      </c>
-      <c r="E134" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135"/>
-      <c r="B135" t="s">
-        <v>260</v>
-      </c>
-      <c r="C135" t="s">
-        <v>262</v>
-      </c>
-      <c r="D135" t="s">
-        <v>18</v>
-      </c>
-      <c r="E135" t="s">
+      <c r="D136" t="s">
+        <v>18</v>
+      </c>
+      <c r="E136" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="s">
-        <v>1</v>
-      </c>
+      <c r="A137"/>
       <c r="B137" t="s">
-        <v>123</v>
+        <v>1378</v>
       </c>
       <c r="C137" t="s">
-        <v>2</v>
+        <v>1379</v>
       </c>
       <c r="D137" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E137" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="s">
-        <v>393</v>
-      </c>
+      <c r="A138"/>
       <c r="B138" t="s">
-        <v>534</v>
+        <v>1380</v>
       </c>
       <c r="C138" t="s">
-        <v>535</v>
+        <v>1381</v>
       </c>
       <c r="D138" t="s">
         <v>18</v>
@@ -12678,10 +12678,10 @@
     <row r="139">
       <c r="A139"/>
       <c r="B139" t="s">
-        <v>536</v>
+        <v>1382</v>
       </c>
       <c r="C139" t="s">
-        <v>537</v>
+        <v>1383</v>
       </c>
       <c r="D139" t="s">
         <v>18</v>
@@ -12693,10 +12693,10 @@
     <row r="140">
       <c r="A140"/>
       <c r="B140" t="s">
-        <v>341</v>
+        <v>260</v>
       </c>
       <c r="C140" t="s">
-        <v>342</v>
+        <v>262</v>
       </c>
       <c r="D140" t="s">
         <v>18</v>
@@ -12724,13 +12724,13 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>483</v>
+        <v>393</v>
       </c>
       <c r="B143" t="s">
-        <v>560</v>
+        <v>534</v>
       </c>
       <c r="C143" t="s">
-        <v>561</v>
+        <v>535</v>
       </c>
       <c r="D143" t="s">
         <v>18</v>
@@ -12742,10 +12742,10 @@
     <row r="144">
       <c r="A144"/>
       <c r="B144" t="s">
-        <v>562</v>
+        <v>536</v>
       </c>
       <c r="C144" t="s">
-        <v>563</v>
+        <v>537</v>
       </c>
       <c r="D144" t="s">
         <v>18</v>
@@ -12757,10 +12757,10 @@
     <row r="145">
       <c r="A145"/>
       <c r="B145" t="s">
-        <v>274</v>
+        <v>341</v>
       </c>
       <c r="C145" t="s">
-        <v>564</v>
+        <v>342</v>
       </c>
       <c r="D145" t="s">
         <v>18</v>
@@ -12769,47 +12769,47 @@
         <v>18</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146"/>
-      <c r="B146" t="s">
-        <v>341</v>
-      </c>
-      <c r="C146" t="s">
-        <v>342</v>
-      </c>
-      <c r="D146" t="s">
-        <v>18</v>
-      </c>
-      <c r="E146" t="s">
-        <v>18</v>
+    <row r="147">
+      <c r="A147" t="s">
+        <v>1</v>
+      </c>
+      <c r="B147" t="s">
+        <v>123</v>
+      </c>
+      <c r="C147" t="s">
+        <v>2</v>
+      </c>
+      <c r="D147" t="s">
+        <v>3</v>
+      </c>
+      <c r="E147" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>1</v>
+        <v>483</v>
       </c>
       <c r="B148" t="s">
-        <v>123</v>
+        <v>560</v>
       </c>
       <c r="C148" t="s">
-        <v>2</v>
+        <v>561</v>
       </c>
       <c r="D148" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E148" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="s">
-        <v>1310</v>
-      </c>
+      <c r="A149"/>
       <c r="B149" t="s">
-        <v>1378</v>
+        <v>562</v>
       </c>
       <c r="C149" t="s">
-        <v>1379</v>
+        <v>563</v>
       </c>
       <c r="D149" t="s">
         <v>18</v>
@@ -12821,10 +12821,10 @@
     <row r="150">
       <c r="A150"/>
       <c r="B150" t="s">
-        <v>1380</v>
+        <v>274</v>
       </c>
       <c r="C150" t="s">
-        <v>1381</v>
+        <v>564</v>
       </c>
       <c r="D150" t="s">
         <v>18</v>
@@ -12836,10 +12836,10 @@
     <row r="151">
       <c r="A151"/>
       <c r="B151" t="s">
-        <v>1382</v>
+        <v>341</v>
       </c>
       <c r="C151" t="s">
-        <v>1383</v>
+        <v>342</v>
       </c>
       <c r="D151" t="s">
         <v>18</v>
@@ -14083,7 +14083,7 @@
         <v>1402</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="C2" t="s">
         <v>1403</v>
@@ -14141,7 +14141,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1250</v>
+        <v>1258</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>39</v>
@@ -17422,10 +17422,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1256</v>
+        <v>1250</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="C3" t="s">
         <v>1403</v>
@@ -18421,7 +18421,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1250</v>
+        <v>1258</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>39</v>
@@ -19870,10 +19870,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1292</v>
+        <v>1308</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
#2206: Code formatting with Eclipse 2020-03: sormas-api
- Added some missing serialVersionUID
- Added sometimes blank lines after method declaration
- @formatter:off for formatted query DTO constructors
- @formatter:off for HTML definitions
- Removed some empty blocks (usually from enum toString methods)
- Tests: throws Exception removed, method names changed to pattern
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6812" uniqueCount="1906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6824" uniqueCount="1912">
   <si>
     <t>Field</t>
   </si>
@@ -4264,10 +4264,10 @@
     <t>Face-to-face contact of at least 15 minutes</t>
   </si>
   <si>
-    <t>MEDICAL_UNSAVE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medical personal at close proximity (2 meter) without protective equipment		</t>
+    <t>MEDICAL_UNSAFE</t>
+  </si>
+  <si>
+    <t>Medical personnel with a high risk of exposure, e.g. unprotected relevant exposure to secretions, exposure to aerosols from COVID-19 cases</t>
   </si>
   <si>
     <t>SAME_ROOM</t>
@@ -4288,16 +4288,16 @@
     <t>Face-to-face contact of less than 15 minutes</t>
   </si>
   <si>
-    <t>MEDICAL_SAVE</t>
-  </si>
-  <si>
-    <t>Medical personal at save proximity (&gt; 2 meter) or with protective equipment</t>
+    <t>MEDICAL_SAFE</t>
+  </si>
+  <si>
+    <t>Medical personnel at save proximity (&gt; 2 meter) or with protective equipment</t>
   </si>
   <si>
     <t>MEDICAL_SAME_ROOM</t>
   </si>
   <si>
-    <t>Medical personal that was in same room or house with source case</t>
+    <t>Medical personnel that was in same room or house with source case</t>
   </si>
   <si>
     <t>AEROSOL</t>
@@ -4312,12 +4312,30 @@
     <t>Medical personnel at save proximity (&gt; 2 meter), without direct contact with secretions or excretions of the patient and without aerosol exposure</t>
   </si>
   <si>
+    <t>MEDICAL_LIMITED</t>
+  </si>
+  <si>
+    <t>Medical personnel with limited exposure, e.g. with contact &lt; 2m to COVID-19 cases without protective equipment, ≥ 15min face-to-face contact (without exposure as described under Ia)</t>
+  </si>
+  <si>
     <t>HIGH_RISK</t>
   </si>
   <si>
     <t>High risk contact</t>
   </si>
   <si>
+    <t>HIGH_RISK_MED</t>
+  </si>
+  <si>
+    <t>High risk medical contact</t>
+  </si>
+  <si>
+    <t>MEDIUM_RISK_MED</t>
+  </si>
+  <si>
+    <t>Medium risk medical contact</t>
+  </si>
+  <si>
     <t>LOW_RISK</t>
   </si>
   <si>
@@ -5752,7 +5770,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.41.0-SNAPSHOT</t>
+    <t>1.42.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -6598,7 +6616,7 @@
 </file>
 
 <file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="ContactContactProximity" displayName="ContactContactProximity" ref="A108:E121">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="ContactContactProximity" displayName="ContactContactProximity" ref="A108:E122">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6612,7 +6630,7 @@
 </file>
 
 <file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="ContactContactCategory" displayName="ContactContactCategory" ref="A123:E126">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="ContactContactCategory" displayName="ContactContactCategory" ref="A124:E129">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6626,7 +6644,7 @@
 </file>
 
 <file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="ContactContactClassification" displayName="ContactContactClassification" ref="A128:E131">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="ContactContactClassification" displayName="ContactContactClassification" ref="A131:E134">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6640,7 +6658,7 @@
 </file>
 
 <file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="ContactContactStatus" displayName="ContactContactStatus" ref="A133:E136">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="ContactContactStatus" displayName="ContactContactStatus" ref="A136:E139">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6654,7 +6672,7 @@
 </file>
 
 <file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ContactFollowUpStatus" displayName="ContactFollowUpStatus" ref="A138:E143">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ContactFollowUpStatus" displayName="ContactFollowUpStatus" ref="A141:E146">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6682,7 +6700,7 @@
 </file>
 
 <file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ContactContactRelation" displayName="ContactContactRelation" ref="A145:E150">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ContactContactRelation" displayName="ContactContactRelation" ref="A148:E153">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6696,7 +6714,7 @@
 </file>
 
 <file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ContactYesNoUnknown" displayName="ContactYesNoUnknown" ref="A152:E155">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ContactYesNoUnknown" displayName="ContactYesNoUnknown" ref="A155:E158">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6710,7 +6728,7 @@
 </file>
 
 <file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="ContactQuarantineType" displayName="ContactQuarantineType" ref="A157:E161">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="ContactQuarantineType" displayName="ContactQuarantineType" ref="A160:E164">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -10795,7 +10813,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I164"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -12808,42 +12826,42 @@
         <v>18</v>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" t="s">
-        <v>1</v>
-      </c>
-      <c r="B123" t="s">
-        <v>123</v>
-      </c>
-      <c r="C123" t="s">
-        <v>2</v>
-      </c>
-      <c r="D123" t="s">
-        <v>3</v>
-      </c>
-      <c r="E123" t="s">
-        <v>124</v>
+    <row r="122">
+      <c r="A122"/>
+      <c r="B122" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D122" t="s">
+        <v>18</v>
+      </c>
+      <c r="E122" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
+        <v>1</v>
+      </c>
+      <c r="B124" t="s">
+        <v>123</v>
+      </c>
+      <c r="C124" t="s">
+        <v>2</v>
+      </c>
+      <c r="D124" t="s">
+        <v>3</v>
+      </c>
+      <c r="E124" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
         <v>1359</v>
       </c>
-      <c r="B124" t="s">
-        <v>1425</v>
-      </c>
-      <c r="C124" t="s">
-        <v>1426</v>
-      </c>
-      <c r="D124" t="s">
-        <v>18</v>
-      </c>
-      <c r="E124" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125"/>
       <c r="B125" t="s">
         <v>1427</v>
       </c>
@@ -12872,294 +12890,294 @@
         <v>18</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127"/>
+      <c r="B127" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C127" t="s">
+        <v>1432</v>
+      </c>
+      <c r="D127" t="s">
+        <v>18</v>
+      </c>
+      <c r="E127" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="128">
-      <c r="A128" t="s">
+      <c r="A128"/>
+      <c r="B128" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C128" t="s">
+        <v>1434</v>
+      </c>
+      <c r="D128" t="s">
+        <v>18</v>
+      </c>
+      <c r="E128" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129"/>
+      <c r="B129" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1436</v>
+      </c>
+      <c r="D129" t="s">
+        <v>18</v>
+      </c>
+      <c r="E129" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
         <v>1</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B131" t="s">
         <v>123</v>
       </c>
-      <c r="C128" t="s">
+      <c r="C131" t="s">
         <v>2</v>
       </c>
-      <c r="D128" t="s">
+      <c r="D131" t="s">
         <v>3</v>
       </c>
-      <c r="E128" t="s">
+      <c r="E131" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="s">
+    <row r="132">
+      <c r="A132" t="s">
         <v>1362</v>
       </c>
-      <c r="B129" t="s">
-        <v>1431</v>
-      </c>
-      <c r="C129" t="s">
-        <v>1432</v>
-      </c>
-      <c r="D129" t="s">
-        <v>18</v>
-      </c>
-      <c r="E129" t="s">
-        <v>1433</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130"/>
-      <c r="B130" t="s">
+      <c r="B132" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C132" t="s">
+        <v>1438</v>
+      </c>
+      <c r="D132" t="s">
+        <v>18</v>
+      </c>
+      <c r="E132" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133"/>
+      <c r="B133" t="s">
         <v>536</v>
       </c>
-      <c r="C130" t="s">
-        <v>1434</v>
-      </c>
-      <c r="D130" t="s">
-        <v>18</v>
-      </c>
-      <c r="E130" t="s">
+      <c r="C133" t="s">
+        <v>1440</v>
+      </c>
+      <c r="D133" t="s">
+        <v>18</v>
+      </c>
+      <c r="E133" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131"/>
-      <c r="B131" t="s">
-        <v>1435</v>
-      </c>
-      <c r="C131" t="s">
-        <v>1436</v>
-      </c>
-      <c r="D131" t="s">
-        <v>18</v>
-      </c>
-      <c r="E131" t="s">
-        <v>1437</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="s">
+    <row r="134">
+      <c r="A134"/>
+      <c r="B134" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C134" t="s">
+        <v>1442</v>
+      </c>
+      <c r="D134" t="s">
+        <v>18</v>
+      </c>
+      <c r="E134" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
         <v>1</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B136" t="s">
         <v>123</v>
       </c>
-      <c r="C133" t="s">
+      <c r="C136" t="s">
         <v>2</v>
       </c>
-      <c r="D133" t="s">
+      <c r="D136" t="s">
         <v>3</v>
       </c>
-      <c r="E133" t="s">
+      <c r="E136" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="s">
+    <row r="137">
+      <c r="A137" t="s">
         <v>1365</v>
       </c>
-      <c r="B134" t="s">
-        <v>1438</v>
-      </c>
-      <c r="C134" t="s">
-        <v>1439</v>
-      </c>
-      <c r="D134" t="s">
-        <v>18</v>
-      </c>
-      <c r="E134" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135"/>
-      <c r="B135" t="s">
-        <v>1440</v>
-      </c>
-      <c r="C135" t="s">
-        <v>1441</v>
-      </c>
-      <c r="D135" t="s">
-        <v>18</v>
-      </c>
-      <c r="E135" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136"/>
-      <c r="B136" t="s">
-        <v>1442</v>
-      </c>
-      <c r="C136" t="s">
-        <v>1443</v>
-      </c>
-      <c r="D136" t="s">
-        <v>18</v>
-      </c>
-      <c r="E136" t="s">
+      <c r="B137" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C137" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D137" t="s">
+        <v>18</v>
+      </c>
+      <c r="E137" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="s">
+      <c r="A138"/>
+      <c r="B138" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C138" t="s">
+        <v>1447</v>
+      </c>
+      <c r="D138" t="s">
+        <v>18</v>
+      </c>
+      <c r="E138" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139"/>
+      <c r="B139" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C139" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D139" t="s">
+        <v>18</v>
+      </c>
+      <c r="E139" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
         <v>1</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B141" t="s">
         <v>123</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C141" t="s">
         <v>2</v>
       </c>
-      <c r="D138" t="s">
+      <c r="D141" t="s">
         <v>3</v>
       </c>
-      <c r="E138" t="s">
+      <c r="E141" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" t="s">
+    <row r="142">
+      <c r="A142" t="s">
         <v>1368</v>
       </c>
-      <c r="B139" t="s">
-        <v>1444</v>
-      </c>
-      <c r="C139" t="s">
-        <v>1445</v>
-      </c>
-      <c r="D139" t="s">
-        <v>1446</v>
-      </c>
-      <c r="E139" t="s">
-        <v>1447</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140"/>
-      <c r="B140" t="s">
-        <v>1448</v>
-      </c>
-      <c r="C140" t="s">
-        <v>1449</v>
-      </c>
-      <c r="D140" t="s">
+      <c r="B142" t="s">
         <v>1450</v>
       </c>
-      <c r="E140" t="s">
+      <c r="C142" t="s">
         <v>1451</v>
       </c>
-    </row>
-    <row r="141">
-      <c r="A141"/>
-      <c r="B141" t="s">
+      <c r="D142" t="s">
         <v>1452</v>
       </c>
-      <c r="C141" t="s">
+      <c r="E142" t="s">
         <v>1453</v>
-      </c>
-      <c r="D141" t="s">
-        <v>1454</v>
-      </c>
-      <c r="E141" t="s">
-        <v>1455</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142"/>
-      <c r="B142" t="s">
-        <v>1456</v>
-      </c>
-      <c r="C142" t="s">
-        <v>1457</v>
-      </c>
-      <c r="D142" t="s">
-        <v>1458</v>
-      </c>
-      <c r="E142" t="s">
-        <v>1459</v>
       </c>
     </row>
     <row r="143">
       <c r="A143"/>
       <c r="B143" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C143" t="s">
+        <v>1455</v>
+      </c>
+      <c r="D143" t="s">
+        <v>1456</v>
+      </c>
+      <c r="E143" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144"/>
+      <c r="B144" t="s">
+        <v>1458</v>
+      </c>
+      <c r="C144" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D144" t="s">
         <v>1460</v>
       </c>
-      <c r="C143" t="s">
+      <c r="E144" t="s">
         <v>1461</v>
       </c>
-      <c r="D143" t="s">
+    </row>
+    <row r="145">
+      <c r="A145"/>
+      <c r="B145" t="s">
         <v>1462</v>
       </c>
-      <c r="E143" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="s">
+      <c r="C145" t="s">
+        <v>1463</v>
+      </c>
+      <c r="D145" t="s">
+        <v>1464</v>
+      </c>
+      <c r="E145" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146"/>
+      <c r="B146" t="s">
+        <v>1466</v>
+      </c>
+      <c r="C146" t="s">
+        <v>1467</v>
+      </c>
+      <c r="D146" t="s">
+        <v>1468</v>
+      </c>
+      <c r="E146" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s">
         <v>1</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B148" t="s">
         <v>123</v>
       </c>
-      <c r="C145" t="s">
+      <c r="C148" t="s">
         <v>2</v>
       </c>
-      <c r="D145" t="s">
+      <c r="D148" t="s">
         <v>3</v>
       </c>
-      <c r="E145" t="s">
+      <c r="E148" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" t="s">
+    <row r="149">
+      <c r="A149" t="s">
         <v>1380</v>
       </c>
-      <c r="B146" t="s">
-        <v>1463</v>
-      </c>
-      <c r="C146" t="s">
-        <v>1464</v>
-      </c>
-      <c r="D146" t="s">
-        <v>18</v>
-      </c>
-      <c r="E146" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147"/>
-      <c r="B147" t="s">
-        <v>1465</v>
-      </c>
-      <c r="C147" t="s">
-        <v>1466</v>
-      </c>
-      <c r="D147" t="s">
-        <v>18</v>
-      </c>
-      <c r="E147" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148"/>
-      <c r="B148" t="s">
-        <v>1467</v>
-      </c>
-      <c r="C148" t="s">
-        <v>1468</v>
-      </c>
-      <c r="D148" t="s">
-        <v>18</v>
-      </c>
-      <c r="E148" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149"/>
       <c r="B149" t="s">
         <v>1469</v>
       </c>
@@ -13176,158 +13194,203 @@
     <row r="150">
       <c r="A150"/>
       <c r="B150" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C150" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D150" t="s">
+        <v>18</v>
+      </c>
+      <c r="E150" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151"/>
+      <c r="B151" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C151" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D151" t="s">
+        <v>18</v>
+      </c>
+      <c r="E151" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152"/>
+      <c r="B152" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C152" t="s">
+        <v>1476</v>
+      </c>
+      <c r="D152" t="s">
+        <v>18</v>
+      </c>
+      <c r="E152" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153"/>
+      <c r="B153" t="s">
         <v>260</v>
       </c>
-      <c r="C150" t="s">
+      <c r="C153" t="s">
         <v>262</v>
       </c>
-      <c r="D150" t="s">
-        <v>18</v>
-      </c>
-      <c r="E150" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="s">
+      <c r="D153" t="s">
+        <v>18</v>
+      </c>
+      <c r="E153" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s">
         <v>1</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B155" t="s">
         <v>123</v>
       </c>
-      <c r="C152" t="s">
+      <c r="C155" t="s">
         <v>2</v>
       </c>
-      <c r="D152" t="s">
+      <c r="D155" t="s">
         <v>3</v>
       </c>
-      <c r="E152" t="s">
+      <c r="E155" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" t="s">
+    <row r="156">
+      <c r="A156" t="s">
         <v>393</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B156" t="s">
         <v>557</v>
       </c>
-      <c r="C153" t="s">
+      <c r="C156" t="s">
         <v>558</v>
       </c>
-      <c r="D153" t="s">
-        <v>18</v>
-      </c>
-      <c r="E153" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154"/>
-      <c r="B154" t="s">
+      <c r="D156" t="s">
+        <v>18</v>
+      </c>
+      <c r="E156" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157"/>
+      <c r="B157" t="s">
         <v>559</v>
       </c>
-      <c r="C154" t="s">
+      <c r="C157" t="s">
         <v>560</v>
       </c>
-      <c r="D154" t="s">
-        <v>18</v>
-      </c>
-      <c r="E154" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155"/>
-      <c r="B155" t="s">
+      <c r="D157" t="s">
+        <v>18</v>
+      </c>
+      <c r="E157" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158"/>
+      <c r="B158" t="s">
         <v>341</v>
       </c>
-      <c r="C155" t="s">
+      <c r="C158" t="s">
         <v>342</v>
       </c>
-      <c r="D155" t="s">
-        <v>18</v>
-      </c>
-      <c r="E155" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="s">
+      <c r="D158" t="s">
+        <v>18</v>
+      </c>
+      <c r="E158" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s">
         <v>1</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B160" t="s">
         <v>123</v>
       </c>
-      <c r="C157" t="s">
+      <c r="C160" t="s">
         <v>2</v>
       </c>
-      <c r="D157" t="s">
+      <c r="D160" t="s">
         <v>3</v>
       </c>
-      <c r="E157" t="s">
+      <c r="E160" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" t="s">
+    <row r="161">
+      <c r="A161" t="s">
         <v>483</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B161" t="s">
         <v>583</v>
       </c>
-      <c r="C158" t="s">
+      <c r="C161" t="s">
         <v>584</v>
       </c>
-      <c r="D158" t="s">
-        <v>18</v>
-      </c>
-      <c r="E158" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159"/>
-      <c r="B159" t="s">
+      <c r="D161" t="s">
+        <v>18</v>
+      </c>
+      <c r="E161" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162"/>
+      <c r="B162" t="s">
         <v>585</v>
       </c>
-      <c r="C159" t="s">
+      <c r="C162" t="s">
         <v>586</v>
       </c>
-      <c r="D159" t="s">
-        <v>18</v>
-      </c>
-      <c r="E159" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160"/>
-      <c r="B160" t="s">
+      <c r="D162" t="s">
+        <v>18</v>
+      </c>
+      <c r="E162" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163"/>
+      <c r="B163" t="s">
         <v>274</v>
       </c>
-      <c r="C160" t="s">
+      <c r="C163" t="s">
         <v>587</v>
       </c>
-      <c r="D160" t="s">
-        <v>18</v>
-      </c>
-      <c r="E160" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161"/>
-      <c r="B161" t="s">
+      <c r="D163" t="s">
+        <v>18</v>
+      </c>
+      <c r="E163" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164"/>
+      <c r="B164" t="s">
         <v>341</v>
       </c>
-      <c r="C161" t="s">
+      <c r="C164" t="s">
         <v>342</v>
       </c>
-      <c r="D161" t="s">
-        <v>18</v>
-      </c>
-      <c r="E161" t="s">
+      <c r="D164" t="s">
+        <v>18</v>
+      </c>
+      <c r="E164" t="s">
         <v>18</v>
       </c>
     </row>
@@ -13397,7 +13460,7 @@
         <v>357</v>
       </c>
       <c r="C2" t="s">
-        <v>1471</v>
+        <v>1477</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>18</v>
@@ -13440,7 +13503,7 @@
         <v>1332</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>1472</v>
+        <v>1478</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -13452,13 +13515,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1473</v>
+        <v>1479</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>364</v>
       </c>
       <c r="C5" t="s">
-        <v>1474</v>
+        <v>1480</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>18</v>
@@ -13473,16 +13536,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1475</v>
+        <v>1481</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>1476</v>
+        <v>1482</v>
       </c>
       <c r="C6" t="s">
-        <v>1477</v>
+        <v>1483</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>1478</v>
+        <v>1484</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -13500,10 +13563,10 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>1480</v>
+        <v>1486</v>
       </c>
       <c r="E7"/>
       <c r="G7" s="12" t="s">
@@ -13538,7 +13601,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>1481</v>
+        <v>1487</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>18</v>
@@ -13557,7 +13620,7 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>1482</v>
+        <v>1488</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>18</v>
@@ -14465,13 +14528,13 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>1476</v>
+        <v>1482</v>
       </c>
       <c r="B72" t="s">
-        <v>1483</v>
+        <v>1489</v>
       </c>
       <c r="C72" t="s">
-        <v>1484</v>
+        <v>1490</v>
       </c>
       <c r="D72" t="s">
         <v>18</v>
@@ -14483,31 +14546,31 @@
     <row r="73">
       <c r="A73"/>
       <c r="B73" t="s">
-        <v>1485</v>
+        <v>1491</v>
       </c>
       <c r="C73" t="s">
-        <v>1486</v>
+        <v>1492</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
       </c>
       <c r="E73" t="s">
-        <v>1487</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="74">
       <c r="A74"/>
       <c r="B74" t="s">
-        <v>1488</v>
+        <v>1494</v>
       </c>
       <c r="C74" t="s">
-        <v>1489</v>
+        <v>1495</v>
       </c>
       <c r="D74" t="s">
         <v>18</v>
       </c>
       <c r="E74" t="s">
-        <v>1490</v>
+        <v>1496</v>
       </c>
     </row>
   </sheetData>
@@ -14563,13 +14626,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1491</v>
+        <v>1497</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>1338</v>
       </c>
       <c r="C2" t="s">
-        <v>1492</v>
+        <v>1498</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>18</v>
@@ -14582,10 +14645,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1493</v>
+        <v>1499</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>1494</v>
+        <v>1500</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -14601,13 +14664,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1495</v>
+        <v>1501</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>1496</v>
+        <v>1502</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>18</v>
@@ -14620,13 +14683,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1497</v>
+        <v>1503</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>1498</v>
+        <v>1504</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>18</v>
@@ -14639,16 +14702,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1499</v>
+        <v>1505</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>1500</v>
+        <v>1506</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>1501</v>
+        <v>1507</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -14759,13 +14822,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="C12" t="s">
-        <v>1504</v>
+        <v>1510</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>18</v>
@@ -14780,13 +14843,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1505</v>
+        <v>1511</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>1506</v>
+        <v>1512</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>18</v>
@@ -14799,13 +14862,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1507</v>
+        <v>1513</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>1508</v>
+        <v>1514</v>
       </c>
       <c r="C14" t="s">
-        <v>1509</v>
+        <v>1515</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>18</v>
@@ -14820,7 +14883,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1510</v>
+        <v>1516</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>52</v>
@@ -14841,13 +14904,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1511</v>
+        <v>1517</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>1512</v>
+        <v>1518</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>18</v>
@@ -14860,13 +14923,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>1513</v>
+        <v>1519</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>1514</v>
+        <v>1520</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>18</v>
@@ -14879,13 +14942,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>1515</v>
+        <v>1521</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>1516</v>
+        <v>1522</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>18</v>
@@ -14898,13 +14961,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>1517</v>
+        <v>1523</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>1518</v>
+        <v>1524</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>18</v>
@@ -14917,13 +14980,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>1519</v>
+        <v>1525</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>1520</v>
+        <v>1526</v>
       </c>
       <c r="C20" t="s">
-        <v>1521</v>
+        <v>1527</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>18</v>
@@ -14936,13 +14999,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>1522</v>
+        <v>1528</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>1523</v>
+        <v>1529</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>18</v>
@@ -14955,7 +15018,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>1524</v>
+        <v>1530</v>
       </c>
       <c r="B22" s="13" t="s">
         <v>9</v>
@@ -14974,13 +15037,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>1526</v>
+        <v>1532</v>
       </c>
       <c r="C23" t="s">
-        <v>1527</v>
+        <v>1533</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>18</v>
@@ -14993,10 +15056,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>1528</v>
+        <v>1534</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>1529</v>
+        <v>1535</v>
       </c>
       <c r="C24" t="s">
         <v>18</v>
@@ -15012,13 +15075,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>1530</v>
+        <v>1536</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>480</v>
       </c>
       <c r="C25" t="s">
-        <v>1531</v>
+        <v>1537</v>
       </c>
       <c r="D25" s="13" t="s">
         <v>18</v>
@@ -15031,13 +15094,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>1532</v>
+        <v>1538</v>
       </c>
       <c r="B26" s="13" t="s">
         <v>480</v>
       </c>
       <c r="C26" t="s">
-        <v>1533</v>
+        <v>1539</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>18</v>
@@ -15050,13 +15113,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>1534</v>
+        <v>1540</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>1535</v>
+        <v>1541</v>
       </c>
       <c r="C27" t="s">
-        <v>1536</v>
+        <v>1542</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>18</v>
@@ -15069,13 +15132,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>1537</v>
+        <v>1543</v>
       </c>
       <c r="B28" s="13" t="s">
         <v>480</v>
       </c>
       <c r="C28" t="s">
-        <v>1538</v>
+        <v>1544</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>18</v>
@@ -15088,13 +15151,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>1539</v>
+        <v>1545</v>
       </c>
       <c r="B29" s="13" t="s">
         <v>480</v>
       </c>
       <c r="C29" t="s">
-        <v>1540</v>
+        <v>1546</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>18</v>
@@ -15107,11 +15170,11 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>1541</v>
+        <v>1547</v>
       </c>
       <c r="B30" s="13"/>
       <c r="C30" t="s">
-        <v>1542</v>
+        <v>1548</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>18</v>
@@ -15124,11 +15187,11 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>1543</v>
+        <v>1549</v>
       </c>
       <c r="B31" s="13"/>
       <c r="C31" t="s">
-        <v>1544</v>
+        <v>1550</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>18</v>
@@ -15141,13 +15204,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>1545</v>
+        <v>1551</v>
       </c>
       <c r="B32" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>1546</v>
+        <v>1552</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>18</v>
@@ -15160,13 +15223,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>1547</v>
+        <v>1553</v>
       </c>
       <c r="B33" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>1548</v>
+        <v>1554</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>18</v>
@@ -15196,13 +15259,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="B36" t="s">
-        <v>1549</v>
+        <v>1555</v>
       </c>
       <c r="C36" t="s">
-        <v>1550</v>
+        <v>1556</v>
       </c>
       <c r="D36" t="s">
         <v>18</v>
@@ -15214,10 +15277,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>1551</v>
+        <v>1557</v>
       </c>
       <c r="C37" t="s">
-        <v>1552</v>
+        <v>1558</v>
       </c>
       <c r="D37" t="s">
         <v>18</v>
@@ -15229,10 +15292,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>1553</v>
+        <v>1559</v>
       </c>
       <c r="C38" t="s">
-        <v>1554</v>
+        <v>1560</v>
       </c>
       <c r="D38" t="s">
         <v>18</v>
@@ -15244,10 +15307,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>1555</v>
+        <v>1561</v>
       </c>
       <c r="C39" t="s">
-        <v>1556</v>
+        <v>1562</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
@@ -15259,10 +15322,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="C40" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="D40" t="s">
         <v>18</v>
@@ -15274,10 +15337,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>1559</v>
+        <v>1565</v>
       </c>
       <c r="C41" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="D41" t="s">
         <v>18</v>
@@ -15289,10 +15352,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>1561</v>
+        <v>1567</v>
       </c>
       <c r="C42" t="s">
-        <v>1562</v>
+        <v>1568</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
@@ -15304,10 +15367,10 @@
     <row r="43">
       <c r="A43"/>
       <c r="B43" t="s">
-        <v>1563</v>
+        <v>1569</v>
       </c>
       <c r="C43" t="s">
-        <v>1564</v>
+        <v>1570</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
@@ -15319,10 +15382,10 @@
     <row r="44">
       <c r="A44"/>
       <c r="B44" t="s">
-        <v>1565</v>
+        <v>1571</v>
       </c>
       <c r="C44" t="s">
-        <v>1566</v>
+        <v>1572</v>
       </c>
       <c r="D44" t="s">
         <v>18</v>
@@ -15334,10 +15397,10 @@
     <row r="45">
       <c r="A45"/>
       <c r="B45" t="s">
-        <v>1567</v>
+        <v>1573</v>
       </c>
       <c r="C45" t="s">
-        <v>1568</v>
+        <v>1574</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -15349,10 +15412,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>1569</v>
+        <v>1575</v>
       </c>
       <c r="C46" t="s">
-        <v>1570</v>
+        <v>1576</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -15364,10 +15427,10 @@
     <row r="47">
       <c r="A47"/>
       <c r="B47" t="s">
-        <v>1571</v>
+        <v>1577</v>
       </c>
       <c r="C47" t="s">
-        <v>1572</v>
+        <v>1578</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -15379,10 +15442,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>1573</v>
+        <v>1579</v>
       </c>
       <c r="C48" t="s">
-        <v>1574</v>
+        <v>1580</v>
       </c>
       <c r="D48" t="s">
         <v>18</v>
@@ -15394,10 +15457,10 @@
     <row r="49">
       <c r="A49"/>
       <c r="B49" t="s">
-        <v>1575</v>
+        <v>1581</v>
       </c>
       <c r="C49" t="s">
-        <v>1576</v>
+        <v>1582</v>
       </c>
       <c r="D49" t="s">
         <v>18</v>
@@ -15409,10 +15472,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>1577</v>
+        <v>1583</v>
       </c>
       <c r="C50" t="s">
-        <v>1578</v>
+        <v>1584</v>
       </c>
       <c r="D50" t="s">
         <v>18</v>
@@ -15424,10 +15487,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>1579</v>
+        <v>1585</v>
       </c>
       <c r="C51" t="s">
-        <v>1580</v>
+        <v>1586</v>
       </c>
       <c r="D51" t="s">
         <v>18</v>
@@ -15439,10 +15502,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>1581</v>
+        <v>1587</v>
       </c>
       <c r="C52" t="s">
-        <v>1582</v>
+        <v>1588</v>
       </c>
       <c r="D52" t="s">
         <v>18</v>
@@ -15454,10 +15517,10 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>1583</v>
+        <v>1589</v>
       </c>
       <c r="C53" t="s">
-        <v>1584</v>
+        <v>1590</v>
       </c>
       <c r="D53" t="s">
         <v>18</v>
@@ -15469,10 +15532,10 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>1585</v>
+        <v>1591</v>
       </c>
       <c r="C54" t="s">
-        <v>1586</v>
+        <v>1592</v>
       </c>
       <c r="D54" t="s">
         <v>18</v>
@@ -15515,13 +15578,13 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>1508</v>
+        <v>1514</v>
       </c>
       <c r="B58" t="s">
-        <v>1587</v>
+        <v>1593</v>
       </c>
       <c r="C58" t="s">
-        <v>1588</v>
+        <v>1594</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -15533,10 +15596,10 @@
     <row r="59">
       <c r="A59"/>
       <c r="B59" t="s">
-        <v>1589</v>
+        <v>1595</v>
       </c>
       <c r="C59" t="s">
-        <v>1590</v>
+        <v>1596</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -15564,13 +15627,13 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>1520</v>
+        <v>1526</v>
       </c>
       <c r="B62" t="s">
-        <v>1591</v>
+        <v>1597</v>
       </c>
       <c r="C62" t="s">
-        <v>1592</v>
+        <v>1598</v>
       </c>
       <c r="D62" t="s">
         <v>18</v>
@@ -15582,10 +15645,10 @@
     <row r="63">
       <c r="A63"/>
       <c r="B63" t="s">
-        <v>1593</v>
+        <v>1599</v>
       </c>
       <c r="C63" t="s">
-        <v>1594</v>
+        <v>1600</v>
       </c>
       <c r="D63" t="s">
         <v>18</v>
@@ -15613,13 +15676,13 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>1526</v>
+        <v>1532</v>
       </c>
       <c r="B66" t="s">
-        <v>1595</v>
+        <v>1601</v>
       </c>
       <c r="C66" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="D66" t="s">
         <v>18</v>
@@ -15631,10 +15694,10 @@
     <row r="67">
       <c r="A67"/>
       <c r="B67" t="s">
-        <v>1597</v>
+        <v>1603</v>
       </c>
       <c r="C67" t="s">
-        <v>1598</v>
+        <v>1604</v>
       </c>
       <c r="D67" t="s">
         <v>18</v>
@@ -15646,10 +15709,10 @@
     <row r="68">
       <c r="A68"/>
       <c r="B68" t="s">
-        <v>1599</v>
+        <v>1605</v>
       </c>
       <c r="C68" t="s">
-        <v>1600</v>
+        <v>1606</v>
       </c>
       <c r="D68" t="s">
         <v>18</v>
@@ -15677,13 +15740,13 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>1535</v>
+        <v>1541</v>
       </c>
       <c r="B71" t="s">
-        <v>1601</v>
+        <v>1607</v>
       </c>
       <c r="C71" t="s">
-        <v>1602</v>
+        <v>1608</v>
       </c>
       <c r="D71" t="s">
         <v>18</v>
@@ -15710,10 +15773,10 @@
     <row r="73">
       <c r="A73"/>
       <c r="B73" t="s">
-        <v>1603</v>
+        <v>1609</v>
       </c>
       <c r="C73" t="s">
-        <v>1604</v>
+        <v>1610</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
@@ -15725,10 +15788,10 @@
     <row r="74">
       <c r="A74"/>
       <c r="B74" t="s">
-        <v>1605</v>
+        <v>1611</v>
       </c>
       <c r="C74" t="s">
-        <v>1606</v>
+        <v>1612</v>
       </c>
       <c r="D74" t="s">
         <v>18</v>
@@ -15793,10 +15856,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1529</v>
+        <v>1535</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -15814,16 +15877,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1608</v>
+        <v>1614</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>1609</v>
+        <v>1615</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>1610</v>
+        <v>1616</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -15835,16 +15898,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1611</v>
+        <v>1617</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>1612</v>
+        <v>1618</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>1613</v>
+        <v>1619</v>
       </c>
       <c r="E4"/>
       <c r="G4" s="14" t="s">
@@ -15854,16 +15917,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1614</v>
+        <v>1620</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1615</v>
+        <v>1621</v>
       </c>
       <c r="C5" t="s">
-        <v>1616</v>
+        <v>1622</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1617</v>
+        <v>1623</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -15875,16 +15938,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1618</v>
+        <v>1624</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>1619</v>
+        <v>1625</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1620</v>
+        <v>1626</v>
       </c>
       <c r="E6"/>
       <c r="G6" s="14" t="s">
@@ -15894,16 +15957,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1621</v>
+        <v>1627</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>1622</v>
+        <v>1628</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>1623</v>
+        <v>1629</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -15915,7 +15978,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1510</v>
+        <v>1516</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>52</v>
@@ -15924,7 +15987,7 @@
         <v>597</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1624</v>
+        <v>1630</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -15936,16 +15999,16 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1511</v>
+        <v>1517</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>1512</v>
+        <v>1518</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1625</v>
+        <v>1631</v>
       </c>
       <c r="E9"/>
       <c r="G9" s="14" t="s">
@@ -15955,7 +16018,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1626</v>
+        <v>1632</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>364</v>
@@ -15976,16 +16039,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1627</v>
+        <v>1633</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1535</v>
+        <v>1541</v>
       </c>
       <c r="C11" t="s">
-        <v>1628</v>
+        <v>1634</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>1629</v>
+        <v>1635</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -15997,16 +16060,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1630</v>
+        <v>1636</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>1631</v>
+        <v>1637</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>1632</v>
+        <v>1638</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -16018,16 +16081,16 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1633</v>
+        <v>1639</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>480</v>
       </c>
       <c r="C13" t="s">
-        <v>1634</v>
+        <v>1640</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>1635</v>
+        <v>1641</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -16039,16 +16102,16 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1636</v>
+        <v>1642</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>480</v>
       </c>
       <c r="C14" t="s">
-        <v>1637</v>
+        <v>1643</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>1638</v>
+        <v>1644</v>
       </c>
       <c r="E14"/>
       <c r="G14" s="14" t="s">
@@ -16058,16 +16121,16 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1639</v>
+        <v>1645</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>1640</v>
+        <v>1646</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>1641</v>
+        <v>1647</v>
       </c>
       <c r="E15"/>
       <c r="G15" s="14" t="s">
@@ -16077,13 +16140,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1642</v>
+        <v>1648</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>1643</v>
+        <v>1649</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>18</v>
@@ -16972,13 +17035,13 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>1615</v>
+        <v>1621</v>
       </c>
       <c r="B77" t="s">
-        <v>1644</v>
+        <v>1650</v>
       </c>
       <c r="C77" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="D77" t="s">
         <v>18</v>
@@ -16990,10 +17053,10 @@
     <row r="78">
       <c r="A78"/>
       <c r="B78" t="s">
-        <v>1646</v>
+        <v>1652</v>
       </c>
       <c r="C78" t="s">
-        <v>1647</v>
+        <v>1653</v>
       </c>
       <c r="D78" t="s">
         <v>18</v>
@@ -17005,10 +17068,10 @@
     <row r="79">
       <c r="A79"/>
       <c r="B79" t="s">
-        <v>1648</v>
+        <v>1654</v>
       </c>
       <c r="C79" t="s">
-        <v>1649</v>
+        <v>1655</v>
       </c>
       <c r="D79" t="s">
         <v>18</v>
@@ -17020,10 +17083,10 @@
     <row r="80">
       <c r="A80"/>
       <c r="B80" t="s">
-        <v>1650</v>
+        <v>1656</v>
       </c>
       <c r="C80" t="s">
-        <v>1651</v>
+        <v>1657</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -17035,10 +17098,10 @@
     <row r="81">
       <c r="A81"/>
       <c r="B81" t="s">
-        <v>1652</v>
+        <v>1658</v>
       </c>
       <c r="C81" t="s">
-        <v>1653</v>
+        <v>1659</v>
       </c>
       <c r="D81" t="s">
         <v>18</v>
@@ -17050,7 +17113,7 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>1654</v>
+        <v>1660</v>
       </c>
       <c r="C82" t="s">
         <v>618</v>
@@ -17065,10 +17128,10 @@
     <row r="83">
       <c r="A83"/>
       <c r="B83" t="s">
-        <v>1655</v>
+        <v>1661</v>
       </c>
       <c r="C83" t="s">
-        <v>1656</v>
+        <v>1662</v>
       </c>
       <c r="D83" t="s">
         <v>18</v>
@@ -17080,10 +17143,10 @@
     <row r="84">
       <c r="A84"/>
       <c r="B84" t="s">
-        <v>1657</v>
+        <v>1663</v>
       </c>
       <c r="C84" t="s">
-        <v>1658</v>
+        <v>1664</v>
       </c>
       <c r="D84" t="s">
         <v>18</v>
@@ -17095,10 +17158,10 @@
     <row r="85">
       <c r="A85"/>
       <c r="B85" t="s">
-        <v>1659</v>
+        <v>1665</v>
       </c>
       <c r="C85" t="s">
-        <v>1660</v>
+        <v>1666</v>
       </c>
       <c r="D85" t="s">
         <v>18</v>
@@ -17110,10 +17173,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>1661</v>
+        <v>1667</v>
       </c>
       <c r="C86" t="s">
-        <v>1662</v>
+        <v>1668</v>
       </c>
       <c r="D86" t="s">
         <v>18</v>
@@ -17125,10 +17188,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>1663</v>
+        <v>1669</v>
       </c>
       <c r="C87" t="s">
-        <v>1664</v>
+        <v>1670</v>
       </c>
       <c r="D87" t="s">
         <v>18</v>
@@ -17140,10 +17203,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>1665</v>
+        <v>1671</v>
       </c>
       <c r="C88" t="s">
-        <v>1666</v>
+        <v>1672</v>
       </c>
       <c r="D88" t="s">
         <v>18</v>
@@ -17155,10 +17218,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>1667</v>
+        <v>1673</v>
       </c>
       <c r="C89" t="s">
-        <v>1668</v>
+        <v>1674</v>
       </c>
       <c r="D89" t="s">
         <v>18</v>
@@ -17170,10 +17233,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C90" t="s">
-        <v>1670</v>
+        <v>1676</v>
       </c>
       <c r="D90" t="s">
         <v>18</v>
@@ -17185,10 +17248,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>1671</v>
+        <v>1677</v>
       </c>
       <c r="C91" t="s">
-        <v>1672</v>
+        <v>1678</v>
       </c>
       <c r="D91" t="s">
         <v>18</v>
@@ -17200,10 +17263,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>1673</v>
+        <v>1679</v>
       </c>
       <c r="C92" t="s">
-        <v>1674</v>
+        <v>1680</v>
       </c>
       <c r="D92" t="s">
         <v>18</v>
@@ -17215,10 +17278,10 @@
     <row r="93">
       <c r="A93"/>
       <c r="B93" t="s">
-        <v>1675</v>
+        <v>1681</v>
       </c>
       <c r="C93" t="s">
-        <v>1676</v>
+        <v>1682</v>
       </c>
       <c r="D93" t="s">
         <v>18</v>
@@ -17230,10 +17293,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>1677</v>
+        <v>1683</v>
       </c>
       <c r="C94" t="s">
-        <v>1678</v>
+        <v>1684</v>
       </c>
       <c r="D94" t="s">
         <v>18</v>
@@ -17276,13 +17339,13 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>1535</v>
+        <v>1541</v>
       </c>
       <c r="B98" t="s">
-        <v>1601</v>
+        <v>1607</v>
       </c>
       <c r="C98" t="s">
-        <v>1602</v>
+        <v>1608</v>
       </c>
       <c r="D98" t="s">
         <v>18</v>
@@ -17309,10 +17372,10 @@
     <row r="100">
       <c r="A100"/>
       <c r="B100" t="s">
-        <v>1603</v>
+        <v>1609</v>
       </c>
       <c r="C100" t="s">
-        <v>1604</v>
+        <v>1610</v>
       </c>
       <c r="D100" t="s">
         <v>18</v>
@@ -17324,10 +17387,10 @@
     <row r="101">
       <c r="A101"/>
       <c r="B101" t="s">
-        <v>1605</v>
+        <v>1611</v>
       </c>
       <c r="C101" t="s">
-        <v>1606</v>
+        <v>1612</v>
       </c>
       <c r="D101" t="s">
         <v>18</v>
@@ -17390,10 +17453,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>1529</v>
+        <v>1535</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -17409,13 +17472,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1621</v>
+        <v>1627</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>1622</v>
+        <v>1628</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>18</v>
@@ -17428,13 +17491,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1679</v>
+        <v>1685</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="C4" t="s">
-        <v>1681</v>
+        <v>1687</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>18</v>
@@ -17447,13 +17510,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1682</v>
+        <v>1688</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="C5" t="s">
-        <v>1683</v>
+        <v>1689</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>18</v>
@@ -17466,13 +17529,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1684</v>
+        <v>1690</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="C6" t="s">
-        <v>1685</v>
+        <v>1691</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>18</v>
@@ -17485,13 +17548,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1686</v>
+        <v>1692</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>18</v>
@@ -17504,13 +17567,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1688</v>
+        <v>1694</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>1689</v>
+        <v>1695</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>18</v>
@@ -17523,13 +17586,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1690</v>
+        <v>1696</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>1691</v>
+        <v>1697</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>18</v>
@@ -17542,13 +17605,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1692</v>
+        <v>1698</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>1693</v>
+        <v>1699</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>18</v>
@@ -17561,13 +17624,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1694</v>
+        <v>1700</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>1695</v>
+        <v>1701</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>18</v>
@@ -17580,13 +17643,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1696</v>
+        <v>1702</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>1697</v>
+        <v>1703</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>18</v>
@@ -17599,13 +17662,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1698</v>
+        <v>1704</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>1699</v>
+        <v>1705</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>18</v>
@@ -17618,13 +17681,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>1701</v>
+        <v>1707</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>18</v>
@@ -17637,13 +17700,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1702</v>
+        <v>1708</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>1703</v>
+        <v>1709</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>18</v>
@@ -17656,13 +17719,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1704</v>
+        <v>1710</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>1705</v>
+        <v>1711</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>18</v>
@@ -17675,13 +17738,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>1706</v>
+        <v>1712</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>1707</v>
+        <v>1713</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>18</v>
@@ -17694,13 +17757,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>1708</v>
+        <v>1714</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>1709</v>
+        <v>1715</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>18</v>
@@ -17713,13 +17776,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>1710</v>
+        <v>1716</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>1711</v>
+        <v>1717</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>18</v>
@@ -17732,13 +17795,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>1712</v>
+        <v>1718</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>1713</v>
+        <v>1719</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>18</v>
@@ -17751,13 +17814,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>1714</v>
+        <v>1720</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>1715</v>
+        <v>1721</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>18</v>
@@ -17770,13 +17833,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>1716</v>
+        <v>1722</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C22" t="s">
-        <v>1717</v>
+        <v>1723</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>18</v>
@@ -17789,13 +17852,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>1718</v>
+        <v>1724</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>1719</v>
+        <v>1725</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>18</v>
@@ -17825,13 +17888,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="B26" t="s">
-        <v>1605</v>
+        <v>1611</v>
       </c>
       <c r="C26" t="s">
-        <v>1606</v>
+        <v>1612</v>
       </c>
       <c r="D26" t="s">
         <v>18</v>
@@ -17843,10 +17906,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>1603</v>
+        <v>1609</v>
       </c>
       <c r="C27" t="s">
-        <v>1604</v>
+        <v>1610</v>
       </c>
       <c r="D27" t="s">
         <v>18</v>
@@ -17858,10 +17921,10 @@
     <row r="28">
       <c r="A28"/>
       <c r="B28" t="s">
-        <v>1601</v>
+        <v>1607</v>
       </c>
       <c r="C28" t="s">
-        <v>1602</v>
+        <v>1608</v>
       </c>
       <c r="D28" t="s">
         <v>18</v>
@@ -17922,13 +17985,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1720</v>
+        <v>1726</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>1721</v>
+        <v>1727</v>
       </c>
       <c r="C2" t="s">
-        <v>1722</v>
+        <v>1728</v>
       </c>
       <c r="D2" s="16" t="s">
         <v>18</v>
@@ -17949,7 +18012,7 @@
         <v>1338</v>
       </c>
       <c r="C3" t="s">
-        <v>1492</v>
+        <v>1498</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>18</v>
@@ -17962,13 +18025,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1723</v>
+        <v>1729</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>1724</v>
+        <v>1730</v>
       </c>
       <c r="C4" t="s">
-        <v>1725</v>
+        <v>1731</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>18</v>
@@ -17981,13 +18044,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1726</v>
+        <v>1732</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>1494</v>
+        <v>1500</v>
       </c>
       <c r="C5" t="s">
-        <v>1727</v>
+        <v>1733</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>18</v>
@@ -18000,16 +18063,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1728</v>
+        <v>1734</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>1729</v>
+        <v>1735</v>
       </c>
       <c r="C6" t="s">
-        <v>1730</v>
+        <v>1736</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>1731</v>
+        <v>1737</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -18021,13 +18084,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1732</v>
+        <v>1738</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>1733</v>
+        <v>1739</v>
       </c>
       <c r="C7" t="s">
-        <v>1734</v>
+        <v>1740</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>18</v>
@@ -18040,13 +18103,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1735</v>
+        <v>1741</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>1736</v>
+        <v>1742</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>18</v>
@@ -18061,13 +18124,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1737</v>
+        <v>1743</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>1738</v>
+        <v>1744</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>18</v>
@@ -18080,13 +18143,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1739</v>
+        <v>1745</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>1740</v>
+        <v>1746</v>
       </c>
       <c r="C10" t="s">
-        <v>1741</v>
+        <v>1747</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>18</v>
@@ -18099,13 +18162,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1742</v>
+        <v>1748</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>1743</v>
+        <v>1749</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>18</v>
@@ -18118,13 +18181,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1744</v>
+        <v>1750</v>
       </c>
       <c r="B12" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>1745</v>
+        <v>1751</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>18</v>
@@ -18137,13 +18200,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>1746</v>
+        <v>1752</v>
       </c>
       <c r="B13" s="16" t="s">
         <v>364</v>
       </c>
       <c r="C13" t="s">
-        <v>1747</v>
+        <v>1753</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>18</v>
@@ -18156,13 +18219,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1748</v>
+        <v>1754</v>
       </c>
       <c r="B14" s="16" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>1749</v>
+        <v>1755</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>18</v>
@@ -18175,13 +18238,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1750</v>
+        <v>1756</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>364</v>
       </c>
       <c r="C15" t="s">
-        <v>1751</v>
+        <v>1757</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>18</v>
@@ -18196,13 +18259,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1752</v>
+        <v>1758</v>
       </c>
       <c r="B16" s="16" t="s">
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>1753</v>
+        <v>1759</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>18</v>
@@ -18215,7 +18278,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>1754</v>
+        <v>1760</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>29</v>
@@ -18234,7 +18297,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>1755</v>
+        <v>1761</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>29</v>
@@ -18253,7 +18316,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>1756</v>
+        <v>1762</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>29</v>
@@ -18289,13 +18352,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>1721</v>
+        <v>1727</v>
       </c>
       <c r="B22" t="s">
-        <v>1757</v>
+        <v>1763</v>
       </c>
       <c r="C22" t="s">
-        <v>1758</v>
+        <v>1764</v>
       </c>
       <c r="D22" t="s">
         <v>18</v>
@@ -18307,10 +18370,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>1759</v>
+        <v>1765</v>
       </c>
       <c r="C23" t="s">
-        <v>1760</v>
+        <v>1766</v>
       </c>
       <c r="D23" t="s">
         <v>18</v>
@@ -18322,10 +18385,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>1761</v>
+        <v>1767</v>
       </c>
       <c r="C24" t="s">
-        <v>1762</v>
+        <v>1768</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
@@ -18337,10 +18400,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>1763</v>
+        <v>1769</v>
       </c>
       <c r="C25" t="s">
-        <v>1764</v>
+        <v>1770</v>
       </c>
       <c r="D25" t="s">
         <v>18</v>
@@ -18368,13 +18431,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>1729</v>
+        <v>1735</v>
       </c>
       <c r="B28" t="s">
-        <v>1765</v>
+        <v>1771</v>
       </c>
       <c r="C28" t="s">
-        <v>1766</v>
+        <v>1772</v>
       </c>
       <c r="D28" t="s">
         <v>18</v>
@@ -18386,10 +18449,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>1767</v>
+        <v>1773</v>
       </c>
       <c r="C29" t="s">
-        <v>1768</v>
+        <v>1774</v>
       </c>
       <c r="D29" t="s">
         <v>18</v>
@@ -18401,10 +18464,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>1769</v>
+        <v>1775</v>
       </c>
       <c r="C30" t="s">
-        <v>1770</v>
+        <v>1776</v>
       </c>
       <c r="D30" t="s">
         <v>18</v>
@@ -18416,10 +18479,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>1771</v>
+        <v>1777</v>
       </c>
       <c r="C31" t="s">
-        <v>1772</v>
+        <v>1778</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
@@ -18431,10 +18494,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>1773</v>
+        <v>1779</v>
       </c>
       <c r="C32" t="s">
-        <v>1774</v>
+        <v>1780</v>
       </c>
       <c r="D32" t="s">
         <v>18</v>
@@ -18446,10 +18509,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>1775</v>
+        <v>1781</v>
       </c>
       <c r="C33" t="s">
-        <v>1776</v>
+        <v>1782</v>
       </c>
       <c r="D33" t="s">
         <v>18</v>
@@ -18461,10 +18524,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>1777</v>
+        <v>1783</v>
       </c>
       <c r="C34" t="s">
-        <v>1778</v>
+        <v>1784</v>
       </c>
       <c r="D34" t="s">
         <v>18</v>
@@ -18476,10 +18539,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
       <c r="C35" t="s">
-        <v>1780</v>
+        <v>1786</v>
       </c>
       <c r="D35" t="s">
         <v>18</v>
@@ -18491,10 +18554,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>1781</v>
+        <v>1787</v>
       </c>
       <c r="C36" t="s">
-        <v>1782</v>
+        <v>1788</v>
       </c>
       <c r="D36" t="s">
         <v>18</v>
@@ -18506,10 +18569,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>1783</v>
+        <v>1789</v>
       </c>
       <c r="C37" t="s">
-        <v>1784</v>
+        <v>1790</v>
       </c>
       <c r="D37" t="s">
         <v>18</v>
@@ -18521,10 +18584,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>1785</v>
+        <v>1791</v>
       </c>
       <c r="C38" t="s">
-        <v>1786</v>
+        <v>1792</v>
       </c>
       <c r="D38" t="s">
         <v>18</v>
@@ -18536,10 +18599,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>1787</v>
+        <v>1793</v>
       </c>
       <c r="C39" t="s">
-        <v>1788</v>
+        <v>1794</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
@@ -18551,10 +18614,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>1789</v>
+        <v>1795</v>
       </c>
       <c r="C40" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
       <c r="D40" t="s">
         <v>18</v>
@@ -18566,10 +18629,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>1791</v>
+        <v>1797</v>
       </c>
       <c r="C41" t="s">
-        <v>1792</v>
+        <v>1798</v>
       </c>
       <c r="D41" t="s">
         <v>18</v>
@@ -18581,10 +18644,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>1793</v>
+        <v>1799</v>
       </c>
       <c r="C42" t="s">
-        <v>1794</v>
+        <v>1800</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
@@ -18596,10 +18659,10 @@
     <row r="43">
       <c r="A43"/>
       <c r="B43" t="s">
-        <v>1795</v>
+        <v>1801</v>
       </c>
       <c r="C43" t="s">
-        <v>1796</v>
+        <v>1802</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
@@ -18611,10 +18674,10 @@
     <row r="44">
       <c r="A44"/>
       <c r="B44" t="s">
-        <v>1797</v>
+        <v>1803</v>
       </c>
       <c r="C44" t="s">
-        <v>1798</v>
+        <v>1804</v>
       </c>
       <c r="D44" t="s">
         <v>18</v>
@@ -18629,7 +18692,7 @@
         <v>260</v>
       </c>
       <c r="C45" t="s">
-        <v>1799</v>
+        <v>1805</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -18641,10 +18704,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>1800</v>
+        <v>1806</v>
       </c>
       <c r="C46" t="s">
-        <v>1801</v>
+        <v>1807</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -18656,10 +18719,10 @@
     <row r="47">
       <c r="A47"/>
       <c r="B47" t="s">
-        <v>1802</v>
+        <v>1808</v>
       </c>
       <c r="C47" t="s">
-        <v>1803</v>
+        <v>1809</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -18671,10 +18734,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>1804</v>
+        <v>1810</v>
       </c>
       <c r="C48" t="s">
-        <v>1805</v>
+        <v>1811</v>
       </c>
       <c r="D48" t="s">
         <v>18</v>
@@ -18702,13 +18765,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>1733</v>
+        <v>1739</v>
       </c>
       <c r="B51" t="s">
-        <v>1806</v>
+        <v>1812</v>
       </c>
       <c r="C51" t="s">
-        <v>1807</v>
+        <v>1813</v>
       </c>
       <c r="D51" t="s">
         <v>18</v>
@@ -18720,10 +18783,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>1808</v>
+        <v>1814</v>
       </c>
       <c r="C52" t="s">
-        <v>1809</v>
+        <v>1815</v>
       </c>
       <c r="D52" t="s">
         <v>18</v>
@@ -18735,10 +18798,10 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>1810</v>
+        <v>1816</v>
       </c>
       <c r="C53" t="s">
-        <v>1811</v>
+        <v>1817</v>
       </c>
       <c r="D53" t="s">
         <v>18</v>
@@ -18766,13 +18829,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>1740</v>
+        <v>1746</v>
       </c>
       <c r="B56" t="s">
         <v>542</v>
       </c>
       <c r="C56" t="s">
-        <v>1812</v>
+        <v>1818</v>
       </c>
       <c r="D56" t="s">
         <v>18</v>
@@ -18787,7 +18850,7 @@
         <v>545</v>
       </c>
       <c r="C57" t="s">
-        <v>1813</v>
+        <v>1819</v>
       </c>
       <c r="D57" t="s">
         <v>18</v>
@@ -18799,10 +18862,10 @@
     <row r="58">
       <c r="A58"/>
       <c r="B58" t="s">
-        <v>1814</v>
+        <v>1820</v>
       </c>
       <c r="C58" t="s">
-        <v>1815</v>
+        <v>1821</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -18814,10 +18877,10 @@
     <row r="59">
       <c r="A59"/>
       <c r="B59" t="s">
-        <v>1816</v>
+        <v>1822</v>
       </c>
       <c r="C59" t="s">
-        <v>1817</v>
+        <v>1823</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -18881,16 +18944,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1818</v>
+        <v>1824</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1819</v>
+        <v>1825</v>
       </c>
       <c r="C2" t="s">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>1821</v>
+        <v>1827</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -18902,16 +18965,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1822</v>
+        <v>1828</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>1823</v>
+        <v>1829</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>1824</v>
+        <v>1830</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -18923,16 +18986,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1825</v>
+        <v>1831</v>
       </c>
       <c r="B4" s="17" t="s">
         <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>1826</v>
+        <v>1832</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>1827</v>
+        <v>1833</v>
       </c>
       <c r="E4"/>
       <c r="G4" s="17" t="s">
@@ -18984,13 +19047,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1828</v>
+        <v>1834</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>1829</v>
+        <v>1835</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>18</v>
@@ -19003,16 +19066,16 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1830</v>
+        <v>1836</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1831</v>
+        <v>1837</v>
       </c>
       <c r="C8" t="s">
-        <v>1832</v>
+        <v>1838</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>1833</v>
+        <v>1839</v>
       </c>
       <c r="E8"/>
       <c r="G8" s="17" t="s">
@@ -19022,16 +19085,16 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1834</v>
+        <v>1840</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>1835</v>
+        <v>1841</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>1836</v>
+        <v>1842</v>
       </c>
       <c r="E9"/>
       <c r="G9" s="17" t="s">
@@ -19041,16 +19104,16 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1837</v>
+        <v>1843</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>1838</v>
+        <v>1844</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>1839</v>
+        <v>1845</v>
       </c>
       <c r="E10"/>
       <c r="G10" s="17" t="s">
@@ -19060,16 +19123,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1840</v>
+        <v>1846</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>1841</v>
+        <v>1847</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="E11"/>
       <c r="G11" s="17" t="s">
@@ -19079,16 +19142,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>1843</v>
+        <v>1849</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>1844</v>
+        <v>1850</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="E12"/>
       <c r="G12" s="17" t="s">
@@ -19155,13 +19218,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1846</v>
+        <v>1852</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>1847</v>
+        <v>1853</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>18</v>
@@ -19248,13 +19311,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>1819</v>
+        <v>1825</v>
       </c>
       <c r="B22" t="s">
-        <v>1848</v>
+        <v>1854</v>
       </c>
       <c r="C22" t="s">
-        <v>1849</v>
+        <v>1855</v>
       </c>
       <c r="D22" t="s">
         <v>18</v>
@@ -19269,7 +19332,7 @@
         <v>536</v>
       </c>
       <c r="C23" t="s">
-        <v>1762</v>
+        <v>1768</v>
       </c>
       <c r="D23" t="s">
         <v>18</v>
@@ -19281,16 +19344,16 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>1850</v>
+        <v>1856</v>
       </c>
       <c r="C24" t="s">
-        <v>1851</v>
+        <v>1857</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>1852</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="26">
@@ -19312,13 +19375,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>1831</v>
+        <v>1837</v>
       </c>
       <c r="B27" t="s">
-        <v>1853</v>
+        <v>1859</v>
       </c>
       <c r="C27" t="s">
-        <v>1854</v>
+        <v>1860</v>
       </c>
       <c r="D27" t="s">
         <v>18</v>
@@ -19360,10 +19423,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>1855</v>
+        <v>1861</v>
       </c>
       <c r="C30" t="s">
-        <v>1856</v>
+        <v>1862</v>
       </c>
       <c r="D30" t="s">
         <v>18</v>
@@ -19375,10 +19438,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>1857</v>
+        <v>1863</v>
       </c>
       <c r="C31" t="s">
-        <v>1858</v>
+        <v>1864</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
@@ -20330,13 +20393,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1723</v>
+        <v>1729</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>1724</v>
+        <v>1730</v>
       </c>
       <c r="C2" t="s">
-        <v>1762</v>
+        <v>1768</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>18</v>
@@ -20354,10 +20417,10 @@
         <v>356</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>1859</v>
+        <v>1865</v>
       </c>
       <c r="C3" t="s">
-        <v>1859</v>
+        <v>1865</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>18</v>
@@ -20372,13 +20435,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1860</v>
+        <v>1866</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>1861</v>
+        <v>1867</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>18</v>
@@ -20459,13 +20522,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
       <c r="D2" s="19" t="s">
         <v>18</v>
@@ -20560,7 +20623,7 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>1864</v>
+        <v>1870</v>
       </c>
       <c r="D7" s="19" t="s">
         <v>18</v>
@@ -20579,7 +20642,7 @@
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>1865</v>
+        <v>1871</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>18</v>
@@ -20592,10 +20655,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1866</v>
+        <v>1872</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>1867</v>
+        <v>1873</v>
       </c>
       <c r="C9" t="s">
         <v>18</v>
@@ -20611,7 +20674,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1868</v>
+        <v>1874</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>480</v>
@@ -20630,7 +20693,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1869</v>
+        <v>1875</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>480</v>
@@ -20685,7 +20748,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>1867</v>
+        <v>1873</v>
       </c>
       <c r="B15" t="s">
         <v>278</v>
@@ -21120,13 +21183,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="B2" s="20" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
       <c r="D2" s="20" t="s">
         <v>18</v>
@@ -21139,13 +21202,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1870</v>
+        <v>1876</v>
       </c>
       <c r="B3" s="20" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>1871</v>
+        <v>1877</v>
       </c>
       <c r="D3" s="20" t="s">
         <v>18</v>
@@ -21158,13 +21221,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1872</v>
+        <v>1878</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>1873</v>
+        <v>1879</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>18</v>
@@ -21177,7 +21240,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1869</v>
+        <v>1875</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>480</v>
@@ -21264,13 +21327,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="B2" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>18</v>
@@ -21283,13 +21346,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1870</v>
+        <v>1876</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>1871</v>
+        <v>1877</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>18</v>
@@ -21302,13 +21365,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1872</v>
+        <v>1878</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>1873</v>
+        <v>1879</v>
       </c>
       <c r="D4" s="21" t="s">
         <v>18</v>
@@ -21340,7 +21403,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1869</v>
+        <v>1875</v>
       </c>
       <c r="B6" s="21" t="s">
         <v>480</v>
@@ -21427,13 +21490,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
       <c r="D2" s="22" t="s">
         <v>18</v>
@@ -21484,7 +21547,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1869</v>
+        <v>1875</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>480</v>
@@ -21571,13 +21634,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1874</v>
+        <v>1880</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>480</v>
       </c>
       <c r="C2" t="s">
-        <v>1875</v>
+        <v>1881</v>
       </c>
       <c r="D2" s="23" t="s">
         <v>18</v>
@@ -21590,13 +21653,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1876</v>
+        <v>1882</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>1877</v>
+        <v>1883</v>
       </c>
       <c r="D3" s="23" t="s">
         <v>18</v>
@@ -21647,13 +21710,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1878</v>
+        <v>1884</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>1844</v>
+        <v>1850</v>
       </c>
       <c r="D6" s="23" t="s">
         <v>18</v>
@@ -21704,11 +21767,11 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1879</v>
+        <v>1885</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" t="s">
-        <v>1880</v>
+        <v>1886</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>18</v>
@@ -21797,7 +21860,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>1881</v>
+        <v>1887</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>52</v>
@@ -21822,7 +21885,7 @@
         <v>471</v>
       </c>
       <c r="C15" t="s">
-        <v>1882</v>
+        <v>1888</v>
       </c>
       <c r="D15" s="23" t="s">
         <v>18</v>
@@ -21835,13 +21898,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1883</v>
+        <v>1889</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>364</v>
       </c>
       <c r="C16" t="s">
-        <v>1884</v>
+        <v>1890</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>18</v>
@@ -21854,16 +21917,16 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>1885</v>
+        <v>1891</v>
       </c>
       <c r="B17" s="23" t="s">
         <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>1886</v>
+        <v>1892</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>1887</v>
+        <v>1893</v>
       </c>
       <c r="E17"/>
       <c r="G17" s="23" t="s">
@@ -21873,10 +21936,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>1888</v>
+        <v>1894</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>1889</v>
+        <v>1895</v>
       </c>
       <c r="C18" t="s">
         <v>18</v>
@@ -22768,13 +22831,13 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>1889</v>
+        <v>1895</v>
       </c>
       <c r="B79" t="s">
-        <v>1890</v>
+        <v>1896</v>
       </c>
       <c r="C79" t="s">
-        <v>1891</v>
+        <v>1897</v>
       </c>
       <c r="D79" t="s">
         <v>18</v>
@@ -22786,10 +22849,10 @@
     <row r="80">
       <c r="A80"/>
       <c r="B80" t="s">
-        <v>1892</v>
+        <v>1898</v>
       </c>
       <c r="C80" t="s">
-        <v>1893</v>
+        <v>1899</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -22801,10 +22864,10 @@
     <row r="81">
       <c r="A81"/>
       <c r="B81" t="s">
-        <v>1894</v>
+        <v>1900</v>
       </c>
       <c r="C81" t="s">
-        <v>1895</v>
+        <v>1901</v>
       </c>
       <c r="D81" t="s">
         <v>18</v>
@@ -22816,10 +22879,10 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>1896</v>
+        <v>1902</v>
       </c>
       <c r="C82" t="s">
-        <v>1897</v>
+        <v>1903</v>
       </c>
       <c r="D82" t="s">
         <v>18</v>
@@ -22831,10 +22894,10 @@
     <row r="83">
       <c r="A83"/>
       <c r="B83" t="s">
-        <v>1898</v>
+        <v>1904</v>
       </c>
       <c r="C83" t="s">
-        <v>1899</v>
+        <v>1905</v>
       </c>
       <c r="D83" t="s">
         <v>18</v>
@@ -22846,10 +22909,10 @@
     <row r="84">
       <c r="A84"/>
       <c r="B84" t="s">
-        <v>1900</v>
+        <v>1906</v>
       </c>
       <c r="C84" t="s">
-        <v>1901</v>
+        <v>1907</v>
       </c>
       <c r="D84" t="s">
         <v>18</v>
@@ -22861,10 +22924,10 @@
     <row r="85">
       <c r="A85"/>
       <c r="B85" t="s">
-        <v>1902</v>
+        <v>1908</v>
       </c>
       <c r="C85" t="s">
-        <v>1903</v>
+        <v>1909</v>
       </c>
       <c r="D85" t="s">
         <v>18</v>
@@ -22890,12 +22953,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>1904</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1905</v>
+        <v>1911</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#1637: Consider the facility type during import
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -1228,6 +1228,12 @@
     <t>Describe sequelae</t>
   </si>
   <si>
+    <t>facilityType</t>
+  </si>
+  <si>
+    <t>FacilityType</t>
+  </si>
+  <si>
     <t>healthFacility</t>
   </si>
   <si>
@@ -1582,12 +1588,6 @@
     <t>Trimester</t>
   </si>
   <si>
-    <t>facilityType</t>
-  </si>
-  <si>
-    <t>FacilityType</t>
-  </si>
-  <si>
     <t>BUBONIC</t>
   </si>
   <si>
@@ -1735,6 +1735,246 @@
     <t>No</t>
   </si>
   <si>
+    <t>ASSOCIATION</t>
+  </si>
+  <si>
+    <t>Association, club</t>
+  </si>
+  <si>
+    <t>BUSINESS</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>CAMPSITE</t>
+  </si>
+  <si>
+    <t>Campsite</t>
+  </si>
+  <si>
+    <t>CANTINE</t>
+  </si>
+  <si>
+    <t>Cantine</t>
+  </si>
+  <si>
+    <t>CHILDRENS_DAY_CARE</t>
+  </si>
+  <si>
+    <t>Children's day care</t>
+  </si>
+  <si>
+    <t>CHILDRENS_HOME</t>
+  </si>
+  <si>
+    <t>Children's home</t>
+  </si>
+  <si>
+    <t>CORRECTIONAL_FACILITY</t>
+  </si>
+  <si>
+    <t>Correctional facility</t>
+  </si>
+  <si>
+    <t>CRUISE_SHIP</t>
+  </si>
+  <si>
+    <t>Cruise ship</t>
+  </si>
+  <si>
+    <t>ELDERLY_CARE</t>
+  </si>
+  <si>
+    <t>Elderly care</t>
+  </si>
+  <si>
+    <t>EVENT_VENUE</t>
+  </si>
+  <si>
+    <t>Event venue</t>
+  </si>
+  <si>
+    <t>FOOD_STALL</t>
+  </si>
+  <si>
+    <t>Food stall</t>
+  </si>
+  <si>
+    <t>HOLIDAY_CAMP</t>
+  </si>
+  <si>
+    <t>Holiday camp</t>
+  </si>
+  <si>
+    <t>HOMELESS_SHELTER</t>
+  </si>
+  <si>
+    <t>Homeless shelter</t>
+  </si>
+  <si>
+    <t>HOSTEL</t>
+  </si>
+  <si>
+    <t>Hostel, dormitory</t>
+  </si>
+  <si>
+    <t>HOTEL</t>
+  </si>
+  <si>
+    <t>Hotel, B&amp;B, inn, lodge</t>
+  </si>
+  <si>
+    <t>KINDERGARTEN</t>
+  </si>
+  <si>
+    <t>Kindergarten/After school care</t>
+  </si>
+  <si>
+    <t>LABORATORY</t>
+  </si>
+  <si>
+    <t>Laboratory</t>
+  </si>
+  <si>
+    <t>MASS_ACCOMMODATION</t>
+  </si>
+  <si>
+    <t>Mass accomodation (e.g. guest and harvest workers)</t>
+  </si>
+  <si>
+    <t>MILITARY_BARRACKS</t>
+  </si>
+  <si>
+    <t>Military barracks</t>
+  </si>
+  <si>
+    <t>MOBILE_NURSING_SERVICE</t>
+  </si>
+  <si>
+    <t>Mobile nursing service</t>
+  </si>
+  <si>
+    <t>OTHER_ACCOMMODATION</t>
+  </si>
+  <si>
+    <t>Other Accomodation</t>
+  </si>
+  <si>
+    <t>OTHER_CARE_FACILITY</t>
+  </si>
+  <si>
+    <t>Other Care facility</t>
+  </si>
+  <si>
+    <t>OTHER_CATERING_OUTLET</t>
+  </si>
+  <si>
+    <t>Other Catering outlet</t>
+  </si>
+  <si>
+    <t>OTHER_EDUCATIONAL_FACILITY</t>
+  </si>
+  <si>
+    <t>Other Educational facility</t>
+  </si>
+  <si>
+    <t>OTHER_LEISURE_FACILITY</t>
+  </si>
+  <si>
+    <t>Other Leisure facility</t>
+  </si>
+  <si>
+    <t>OTHER_MEDICAL_FACILITY</t>
+  </si>
+  <si>
+    <t>Other Medical facility</t>
+  </si>
+  <si>
+    <t>OTHER_RESIDENCE</t>
+  </si>
+  <si>
+    <t>Other Residence</t>
+  </si>
+  <si>
+    <t>OTHER_WORKING_PLACE</t>
+  </si>
+  <si>
+    <t>Other Working place/company</t>
+  </si>
+  <si>
+    <t>OUTPATIENT_TREATMENT_FACILITY</t>
+  </si>
+  <si>
+    <t>Outpatient treatment facility</t>
+  </si>
+  <si>
+    <t>PLACE_OF_WORSHIP</t>
+  </si>
+  <si>
+    <t>Place of worship</t>
+  </si>
+  <si>
+    <t>PUBLIC_PLACE</t>
+  </si>
+  <si>
+    <t>Public place/playground</t>
+  </si>
+  <si>
+    <t>REFUGEE_ACCOMMODATION</t>
+  </si>
+  <si>
+    <t>Refrugee accomodation/initial reception facility</t>
+  </si>
+  <si>
+    <t>REHAB_FACILITY</t>
+  </si>
+  <si>
+    <t>Rehab facility</t>
+  </si>
+  <si>
+    <t>RESTAURANT</t>
+  </si>
+  <si>
+    <t>Restaurant/tavern</t>
+  </si>
+  <si>
+    <t>RETIREMENT_HOME</t>
+  </si>
+  <si>
+    <t>Retirement home</t>
+  </si>
+  <si>
+    <t>SCHOOL</t>
+  </si>
+  <si>
+    <t>School</t>
+  </si>
+  <si>
+    <t>SWIMMING_POOL</t>
+  </si>
+  <si>
+    <t>Swimming pool</t>
+  </si>
+  <si>
+    <t>THEATER</t>
+  </si>
+  <si>
+    <t>Theater/cinema</t>
+  </si>
+  <si>
+    <t>UNIVERSITY</t>
+  </si>
+  <si>
+    <t>University</t>
+  </si>
+  <si>
+    <t>ZOO</t>
+  </si>
+  <si>
+    <t>Zoological garden, animal park</t>
+  </si>
+  <si>
     <t>VACCINATED</t>
   </si>
   <si>
@@ -1840,12 +2080,6 @@
     <t>Community facility</t>
   </si>
   <si>
-    <t>LABORATORY</t>
-  </si>
-  <si>
-    <t>Laboratory</t>
-  </si>
-  <si>
     <t>OWN_DETERMINATION</t>
   </si>
   <si>
@@ -1880,240 +2114,6 @@
   </si>
   <si>
     <t>Third</t>
-  </si>
-  <si>
-    <t>ASSOCIATION</t>
-  </si>
-  <si>
-    <t>Association, club</t>
-  </si>
-  <si>
-    <t>BUSINESS</t>
-  </si>
-  <si>
-    <t>Business</t>
-  </si>
-  <si>
-    <t>CAMPSITE</t>
-  </si>
-  <si>
-    <t>Campsite</t>
-  </si>
-  <si>
-    <t>CANTINE</t>
-  </si>
-  <si>
-    <t>Cantine</t>
-  </si>
-  <si>
-    <t>CHILDRENS_DAY_CARE</t>
-  </si>
-  <si>
-    <t>Children's day care</t>
-  </si>
-  <si>
-    <t>CHILDRENS_HOME</t>
-  </si>
-  <si>
-    <t>Children's home</t>
-  </si>
-  <si>
-    <t>CORRECTIONAL_FACILITY</t>
-  </si>
-  <si>
-    <t>Correctional facility</t>
-  </si>
-  <si>
-    <t>CRUISE_SHIP</t>
-  </si>
-  <si>
-    <t>Cruise ship</t>
-  </si>
-  <si>
-    <t>ELDERLY_CARE</t>
-  </si>
-  <si>
-    <t>Elderly care</t>
-  </si>
-  <si>
-    <t>EVENT_VENUE</t>
-  </si>
-  <si>
-    <t>Event venue</t>
-  </si>
-  <si>
-    <t>FOOD_STALL</t>
-  </si>
-  <si>
-    <t>Food stall</t>
-  </si>
-  <si>
-    <t>HOLIDAY_CAMP</t>
-  </si>
-  <si>
-    <t>Holiday camp</t>
-  </si>
-  <si>
-    <t>HOMELESS_SHELTER</t>
-  </si>
-  <si>
-    <t>Homeless shelter</t>
-  </si>
-  <si>
-    <t>HOSTEL</t>
-  </si>
-  <si>
-    <t>Hostel, dormitory</t>
-  </si>
-  <si>
-    <t>HOTEL</t>
-  </si>
-  <si>
-    <t>Hotel, B&amp;B, inn, lodge</t>
-  </si>
-  <si>
-    <t>KINDERGARTEN</t>
-  </si>
-  <si>
-    <t>Kindergarten/After school care</t>
-  </si>
-  <si>
-    <t>MASS_ACCOMMODATION</t>
-  </si>
-  <si>
-    <t>Mass accomodation (e.g. guest and harvest workers)</t>
-  </si>
-  <si>
-    <t>MILITARY_BARRACKS</t>
-  </si>
-  <si>
-    <t>Military barracks</t>
-  </si>
-  <si>
-    <t>MOBILE_NURSING_SERVICE</t>
-  </si>
-  <si>
-    <t>Mobile nursing service</t>
-  </si>
-  <si>
-    <t>OTHER_ACCOMMODATION</t>
-  </si>
-  <si>
-    <t>Other Accomodation</t>
-  </si>
-  <si>
-    <t>OTHER_CARE_FACILITY</t>
-  </si>
-  <si>
-    <t>Other Care facility</t>
-  </si>
-  <si>
-    <t>OTHER_CATERING_OUTLET</t>
-  </si>
-  <si>
-    <t>Other Catering outlet</t>
-  </si>
-  <si>
-    <t>OTHER_EDUCATIONAL_FACILITY</t>
-  </si>
-  <si>
-    <t>Other Educational facility</t>
-  </si>
-  <si>
-    <t>OTHER_LEISURE_FACILITY</t>
-  </si>
-  <si>
-    <t>Other Leisure facility</t>
-  </si>
-  <si>
-    <t>OTHER_MEDICAL_FACILITY</t>
-  </si>
-  <si>
-    <t>Other Medical facility</t>
-  </si>
-  <si>
-    <t>OTHER_RESIDENCE</t>
-  </si>
-  <si>
-    <t>Other Residence</t>
-  </si>
-  <si>
-    <t>OTHER_WORKING_PLACE</t>
-  </si>
-  <si>
-    <t>Other Working place/company</t>
-  </si>
-  <si>
-    <t>OUTPATIENT_TREATMENT_FACILITY</t>
-  </si>
-  <si>
-    <t>Outpatient treatment facility</t>
-  </si>
-  <si>
-    <t>PLACE_OF_WORSHIP</t>
-  </si>
-  <si>
-    <t>Place of worship</t>
-  </si>
-  <si>
-    <t>PUBLIC_PLACE</t>
-  </si>
-  <si>
-    <t>Public place/playground</t>
-  </si>
-  <si>
-    <t>REFUGEE_ACCOMMODATION</t>
-  </si>
-  <si>
-    <t>Refrugee accomodation/initial reception facility</t>
-  </si>
-  <si>
-    <t>REHAB_FACILITY</t>
-  </si>
-  <si>
-    <t>Rehab facility</t>
-  </si>
-  <si>
-    <t>RESTAURANT</t>
-  </si>
-  <si>
-    <t>Restaurant/tavern</t>
-  </si>
-  <si>
-    <t>RETIREMENT_HOME</t>
-  </si>
-  <si>
-    <t>Retirement home</t>
-  </si>
-  <si>
-    <t>SCHOOL</t>
-  </si>
-  <si>
-    <t>School</t>
-  </si>
-  <si>
-    <t>SWIMMING_POOL</t>
-  </si>
-  <si>
-    <t>Swimming pool</t>
-  </si>
-  <si>
-    <t>THEATER</t>
-  </si>
-  <si>
-    <t>Theater/cinema</t>
-  </si>
-  <si>
-    <t>UNIVERSITY</t>
-  </si>
-  <si>
-    <t>University</t>
-  </si>
-  <si>
-    <t>ZOO</t>
-  </si>
-  <si>
-    <t>Zoological garden, animal park</t>
   </si>
   <si>
     <t>admittedToHealthFacility</t>
@@ -6457,7 +6457,7 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="CaseVaccination" displayName="CaseVaccination" ref="A174:E177">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="CaseFacilityType" displayName="CaseFacilityType" ref="A174:E215">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6471,7 +6471,7 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="CaseVaccinationInfoSource" displayName="CaseVaccinationInfoSource" ref="A179:E181">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="CaseVaccination" displayName="CaseVaccination" ref="A217:E220">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6485,7 +6485,7 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="CaseHospitalWardType" displayName="CaseHospitalWardType" ref="A183:E192">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="CaseVaccinationInfoSource" displayName="CaseVaccinationInfoSource" ref="A222:E224">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6499,7 +6499,7 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="CaseCaseOrigin" displayName="CaseCaseOrigin" ref="A194:E196">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="CaseHospitalWardType" displayName="CaseHospitalWardType" ref="A226:E235">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6513,7 +6513,7 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="CaseQuarantineType" displayName="CaseQuarantineType" ref="A198:E203">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="CaseCaseOrigin" displayName="CaseCaseOrigin" ref="A237:E239">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6527,7 +6527,7 @@
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="CaseReportingType" displayName="CaseReportingType" ref="A205:E214">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="CaseQuarantineType" displayName="CaseQuarantineType" ref="A241:E246">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6541,7 +6541,7 @@
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="CaseTrimester" displayName="CaseTrimester" ref="A216:E220">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="CaseReportingType" displayName="CaseReportingType" ref="A248:E257">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -6555,7 +6555,7 @@
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="CaseFacilityType" displayName="CaseFacilityType" ref="A222:E263">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="CaseTrimester" displayName="CaseTrimester" ref="A259:E263">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -10242,7 +10242,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>1413</v>
@@ -10261,10 +10261,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -11402,7 +11402,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>29</v>
@@ -11421,7 +11421,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>29</v>
@@ -11440,7 +11440,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>29</v>
@@ -11673,7 +11673,7 @@
         <v>1458</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C23" t="s">
         <v>1459</v>
@@ -11746,13 +11746,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>18</v>
@@ -11768,7 +11768,7 @@
         <v>1468</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C28" t="s">
         <v>1469</v>
@@ -11841,13 +11841,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="C32" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>18</v>
@@ -11860,13 +11860,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>18</v>
@@ -11879,13 +11879,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>18</v>
@@ -11898,13 +11898,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>18</v>
@@ -11995,13 +11995,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C40" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>18</v>
@@ -12014,13 +12014,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C41" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>18</v>
@@ -12033,13 +12033,13 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C42" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>18</v>
@@ -12052,13 +12052,13 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D43" s="11" t="s">
         <v>18</v>
@@ -12071,13 +12071,13 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C44" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D44" s="11" t="s">
         <v>18</v>
@@ -12090,13 +12090,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>393</v>
       </c>
       <c r="C45" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D45" s="11" t="s">
         <v>18</v>
@@ -12109,13 +12109,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C46" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D46" s="11" t="s">
         <v>18</v>
@@ -12128,13 +12128,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>393</v>
       </c>
       <c r="C47" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D47" s="11" t="s">
         <v>18</v>
@@ -12147,13 +12147,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C48" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D48" s="11" t="s">
         <v>18</v>
@@ -12166,13 +12166,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C49" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="D49" s="11" t="s">
         <v>18</v>
@@ -12185,13 +12185,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C50" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D50" s="11" t="s">
         <v>18</v>
@@ -13783,13 +13783,13 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B163" t="s">
-        <v>588</v>
+        <v>668</v>
       </c>
       <c r="C163" t="s">
-        <v>589</v>
+        <v>669</v>
       </c>
       <c r="D163" t="s">
         <v>18</v>
@@ -13801,10 +13801,10 @@
     <row r="164">
       <c r="A164"/>
       <c r="B164" t="s">
-        <v>590</v>
+        <v>670</v>
       </c>
       <c r="C164" t="s">
-        <v>591</v>
+        <v>671</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>
@@ -13819,7 +13819,7 @@
         <v>274</v>
       </c>
       <c r="C165" t="s">
-        <v>592</v>
+        <v>672</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>
@@ -14040,13 +14040,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C8" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>18</v>
@@ -14059,7 +14059,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>29</v>
@@ -14078,7 +14078,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>29</v>
@@ -14097,7 +14097,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>29</v>
@@ -15248,7 +15248,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>29</v>
@@ -15267,7 +15267,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>29</v>
@@ -15286,7 +15286,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>29</v>
@@ -15372,7 +15372,7 @@
         <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>18</v>
@@ -15507,7 +15507,7 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>18</v>
@@ -15561,7 +15561,7 @@
         <v>1621</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C26" t="s">
         <v>1622</v>
@@ -15580,7 +15580,7 @@
         <v>1623</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C27" t="s">
         <v>1624</v>
@@ -15618,7 +15618,7 @@
         <v>1628</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C29" t="s">
         <v>1629</v>
@@ -15637,7 +15637,7 @@
         <v>1630</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C30" t="s">
         <v>1631</v>
@@ -16467,7 +16467,7 @@
         <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>1715</v>
@@ -16567,7 +16567,7 @@
         <v>1724</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C13" t="s">
         <v>1725</v>
@@ -16588,7 +16588,7 @@
         <v>1727</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C14" t="s">
         <v>1728</v>
@@ -19454,7 +19454,7 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D3" s="17" t="s">
         <v>18</v>
@@ -19815,13 +19815,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>364</v>
       </c>
       <c r="C22" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>18</v>
@@ -19853,7 +19853,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>29</v>
@@ -19872,7 +19872,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>29</v>
@@ -19891,7 +19891,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B26" s="17" t="s">
         <v>29</v>
@@ -20103,10 +20103,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>590</v>
+        <v>670</v>
       </c>
       <c r="C42" t="s">
-        <v>591</v>
+        <v>671</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
@@ -20148,7 +20148,7 @@
     <row r="45">
       <c r="A45"/>
       <c r="B45" t="s">
-        <v>673</v>
+        <v>626</v>
       </c>
       <c r="C45" t="s">
         <v>1966</v>
@@ -21449,7 +21449,7 @@
         <v>1982</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>516</v>
+        <v>398</v>
       </c>
       <c r="C9" t="s">
         <v>1983</v>
@@ -21468,7 +21468,7 @@
         <v>1984</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
@@ -21487,7 +21487,7 @@
         <v>1985</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C11" t="s">
         <v>18</v>
@@ -21503,13 +21503,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D12" s="19" t="s">
         <v>18</v>
@@ -21539,13 +21539,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>516</v>
+        <v>398</v>
       </c>
       <c r="B15" t="s">
-        <v>615</v>
+        <v>566</v>
       </c>
       <c r="C15" t="s">
-        <v>616</v>
+        <v>567</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
@@ -21557,10 +21557,10 @@
     <row r="16">
       <c r="A16"/>
       <c r="B16" t="s">
-        <v>617</v>
+        <v>568</v>
       </c>
       <c r="C16" t="s">
-        <v>618</v>
+        <v>569</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -21572,10 +21572,10 @@
     <row r="17">
       <c r="A17"/>
       <c r="B17" t="s">
-        <v>619</v>
+        <v>570</v>
       </c>
       <c r="C17" t="s">
-        <v>620</v>
+        <v>571</v>
       </c>
       <c r="D17" t="s">
         <v>18</v>
@@ -21587,10 +21587,10 @@
     <row r="18">
       <c r="A18"/>
       <c r="B18" t="s">
-        <v>621</v>
+        <v>572</v>
       </c>
       <c r="C18" t="s">
-        <v>622</v>
+        <v>573</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
@@ -21602,10 +21602,10 @@
     <row r="19">
       <c r="A19"/>
       <c r="B19" t="s">
-        <v>623</v>
+        <v>574</v>
       </c>
       <c r="C19" t="s">
-        <v>624</v>
+        <v>575</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -21617,10 +21617,10 @@
     <row r="20">
       <c r="A20"/>
       <c r="B20" t="s">
-        <v>625</v>
+        <v>576</v>
       </c>
       <c r="C20" t="s">
-        <v>626</v>
+        <v>577</v>
       </c>
       <c r="D20" t="s">
         <v>18</v>
@@ -21632,10 +21632,10 @@
     <row r="21">
       <c r="A21"/>
       <c r="B21" t="s">
-        <v>627</v>
+        <v>578</v>
       </c>
       <c r="C21" t="s">
-        <v>628</v>
+        <v>579</v>
       </c>
       <c r="D21" t="s">
         <v>18</v>
@@ -21647,10 +21647,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>629</v>
+        <v>580</v>
       </c>
       <c r="C22" t="s">
-        <v>630</v>
+        <v>581</v>
       </c>
       <c r="D22" t="s">
         <v>18</v>
@@ -21662,10 +21662,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>631</v>
+        <v>582</v>
       </c>
       <c r="C23" t="s">
-        <v>632</v>
+        <v>583</v>
       </c>
       <c r="D23" t="s">
         <v>18</v>
@@ -21677,10 +21677,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>633</v>
+        <v>584</v>
       </c>
       <c r="C24" t="s">
-        <v>634</v>
+        <v>585</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
@@ -21692,10 +21692,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>635</v>
+        <v>586</v>
       </c>
       <c r="C25" t="s">
-        <v>636</v>
+        <v>587</v>
       </c>
       <c r="D25" t="s">
         <v>18</v>
@@ -21707,10 +21707,10 @@
     <row r="26">
       <c r="A26"/>
       <c r="B26" t="s">
-        <v>637</v>
+        <v>588</v>
       </c>
       <c r="C26" t="s">
-        <v>638</v>
+        <v>589</v>
       </c>
       <c r="D26" t="s">
         <v>18</v>
@@ -21722,10 +21722,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>639</v>
+        <v>590</v>
       </c>
       <c r="C27" t="s">
-        <v>640</v>
+        <v>591</v>
       </c>
       <c r="D27" t="s">
         <v>18</v>
@@ -21752,10 +21752,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>641</v>
+        <v>592</v>
       </c>
       <c r="C29" t="s">
-        <v>642</v>
+        <v>593</v>
       </c>
       <c r="D29" t="s">
         <v>18</v>
@@ -21767,10 +21767,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>643</v>
+        <v>594</v>
       </c>
       <c r="C30" t="s">
-        <v>644</v>
+        <v>595</v>
       </c>
       <c r="D30" t="s">
         <v>18</v>
@@ -21782,10 +21782,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>645</v>
+        <v>596</v>
       </c>
       <c r="C31" t="s">
-        <v>646</v>
+        <v>597</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
@@ -21797,10 +21797,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="C32" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D32" t="s">
         <v>18</v>
@@ -21812,10 +21812,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>647</v>
+        <v>600</v>
       </c>
       <c r="C33" t="s">
-        <v>648</v>
+        <v>601</v>
       </c>
       <c r="D33" t="s">
         <v>18</v>
@@ -21827,10 +21827,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>649</v>
+        <v>602</v>
       </c>
       <c r="C34" t="s">
-        <v>650</v>
+        <v>603</v>
       </c>
       <c r="D34" t="s">
         <v>18</v>
@@ -21842,10 +21842,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>651</v>
+        <v>604</v>
       </c>
       <c r="C35" t="s">
-        <v>652</v>
+        <v>605</v>
       </c>
       <c r="D35" t="s">
         <v>18</v>
@@ -21857,10 +21857,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>653</v>
+        <v>606</v>
       </c>
       <c r="C36" t="s">
-        <v>654</v>
+        <v>607</v>
       </c>
       <c r="D36" t="s">
         <v>18</v>
@@ -21872,10 +21872,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>655</v>
+        <v>608</v>
       </c>
       <c r="C37" t="s">
-        <v>656</v>
+        <v>609</v>
       </c>
       <c r="D37" t="s">
         <v>18</v>
@@ -21887,10 +21887,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>657</v>
+        <v>610</v>
       </c>
       <c r="C38" t="s">
-        <v>658</v>
+        <v>611</v>
       </c>
       <c r="D38" t="s">
         <v>18</v>
@@ -21902,10 +21902,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>659</v>
+        <v>612</v>
       </c>
       <c r="C39" t="s">
-        <v>660</v>
+        <v>613</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
@@ -21917,10 +21917,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>661</v>
+        <v>614</v>
       </c>
       <c r="C40" t="s">
-        <v>662</v>
+        <v>615</v>
       </c>
       <c r="D40" t="s">
         <v>18</v>
@@ -21932,10 +21932,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>663</v>
+        <v>616</v>
       </c>
       <c r="C41" t="s">
-        <v>664</v>
+        <v>617</v>
       </c>
       <c r="D41" t="s">
         <v>18</v>
@@ -21947,10 +21947,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>665</v>
+        <v>618</v>
       </c>
       <c r="C42" t="s">
-        <v>666</v>
+        <v>619</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
@@ -21962,10 +21962,10 @@
     <row r="43">
       <c r="A43"/>
       <c r="B43" t="s">
-        <v>667</v>
+        <v>620</v>
       </c>
       <c r="C43" t="s">
-        <v>668</v>
+        <v>621</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
@@ -21977,10 +21977,10 @@
     <row r="44">
       <c r="A44"/>
       <c r="B44" t="s">
-        <v>669</v>
+        <v>622</v>
       </c>
       <c r="C44" t="s">
-        <v>670</v>
+        <v>623</v>
       </c>
       <c r="D44" t="s">
         <v>18</v>
@@ -21992,10 +21992,10 @@
     <row r="45">
       <c r="A45"/>
       <c r="B45" t="s">
-        <v>671</v>
+        <v>624</v>
       </c>
       <c r="C45" t="s">
-        <v>672</v>
+        <v>625</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -22007,10 +22007,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>673</v>
+        <v>626</v>
       </c>
       <c r="C46" t="s">
-        <v>674</v>
+        <v>627</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -22022,10 +22022,10 @@
     <row r="47">
       <c r="A47"/>
       <c r="B47" t="s">
-        <v>675</v>
+        <v>628</v>
       </c>
       <c r="C47" t="s">
-        <v>676</v>
+        <v>629</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -22037,10 +22037,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>677</v>
+        <v>630</v>
       </c>
       <c r="C48" t="s">
-        <v>678</v>
+        <v>631</v>
       </c>
       <c r="D48" t="s">
         <v>18</v>
@@ -22052,10 +22052,10 @@
     <row r="49">
       <c r="A49"/>
       <c r="B49" t="s">
-        <v>679</v>
+        <v>632</v>
       </c>
       <c r="C49" t="s">
-        <v>680</v>
+        <v>633</v>
       </c>
       <c r="D49" t="s">
         <v>18</v>
@@ -22067,10 +22067,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>681</v>
+        <v>634</v>
       </c>
       <c r="C50" t="s">
-        <v>682</v>
+        <v>635</v>
       </c>
       <c r="D50" t="s">
         <v>18</v>
@@ -22082,10 +22082,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>683</v>
+        <v>636</v>
       </c>
       <c r="C51" t="s">
-        <v>684</v>
+        <v>637</v>
       </c>
       <c r="D51" t="s">
         <v>18</v>
@@ -22097,10 +22097,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>685</v>
+        <v>638</v>
       </c>
       <c r="C52" t="s">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="D52" t="s">
         <v>18</v>
@@ -22112,10 +22112,10 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>687</v>
+        <v>640</v>
       </c>
       <c r="C53" t="s">
-        <v>688</v>
+        <v>641</v>
       </c>
       <c r="D53" t="s">
         <v>18</v>
@@ -22127,10 +22127,10 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>689</v>
+        <v>642</v>
       </c>
       <c r="C54" t="s">
-        <v>690</v>
+        <v>643</v>
       </c>
       <c r="D54" t="s">
         <v>18</v>
@@ -22142,10 +22142,10 @@
     <row r="55">
       <c r="A55"/>
       <c r="B55" t="s">
-        <v>691</v>
+        <v>644</v>
       </c>
       <c r="C55" t="s">
-        <v>692</v>
+        <v>645</v>
       </c>
       <c r="D55" t="s">
         <v>18</v>
@@ -22589,7 +22589,7 @@
         <v>1985</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
@@ -22605,13 +22605,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B6" s="20" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>18</v>
@@ -22771,7 +22771,7 @@
         <v>1985</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
@@ -22787,13 +22787,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>18</v>
@@ -22915,7 +22915,7 @@
         <v>1985</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
@@ -22931,13 +22931,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>18</v>
@@ -23002,7 +23002,7 @@
         <v>1992</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C2" t="s">
         <v>1993</v>
@@ -23206,13 +23206,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B13" s="23" t="s">
         <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D13" s="23" t="s">
         <v>18</v>
@@ -23231,7 +23231,7 @@
         <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D14" s="23" t="s">
         <v>18</v>
@@ -23244,10 +23244,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C15" t="s">
         <v>2001</v>
@@ -24983,38 +24983,36 @@
         <v>397</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>52</v>
+        <v>398</v>
       </c>
       <c r="C27" t="s">
-        <v>398</v>
+        <v>18</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="E27" t="b">
-        <v>1</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="E27"/>
       <c r="G27" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H27" t="b">
-        <v>1</v>
-      </c>
+      <c r="H27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>399</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
         <v>400</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" t="s">
-        <v>55</v>
-      </c>
       <c r="D28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28"/>
+        <v>401</v>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
       <c r="G28" s="3" t="s">
         <v>12</v>
       </c>
@@ -25024,60 +25022,60 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>393</v>
+        <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>402</v>
+        <v>55</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="E29"/>
       <c r="G29" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H29"/>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
+        <v>403</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C30" t="s">
         <v>404</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>405</v>
-      </c>
-      <c r="C30" t="s">
-        <v>406</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="E30"/>
       <c r="G30" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="H30" t="b">
-        <v>1</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="H30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
+        <v>406</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C31" t="s">
         <v>408</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" t="s">
-        <v>409</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E31"/>
       <c r="G31" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="H31" t="b">
         <v>1</v>
@@ -25085,20 +25083,20 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
+        <v>410</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
         <v>411</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" t="s">
-        <v>412</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E32"/>
       <c r="G32" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="H32" t="b">
         <v>1</v>
@@ -25106,29 +25104,31 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
+        <v>413</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
         <v>414</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>415</v>
-      </c>
-      <c r="C33" t="s">
-        <v>416</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E33"/>
       <c r="G33" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="H33"/>
+        <v>415</v>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
+        <v>416</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>417</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C34" t="s">
         <v>418</v>
@@ -25138,30 +25138,30 @@
       </c>
       <c r="E34"/>
       <c r="G34" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="H34" t="b">
-        <v>1</v>
-      </c>
+        <v>409</v>
+      </c>
+      <c r="H34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
+        <v>419</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
         <v>420</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="C35" t="s">
-        <v>421</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E35"/>
       <c r="G35" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="H35"/>
+        <v>421</v>
+      </c>
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
@@ -25187,7 +25187,7 @@
         <v>424</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="C37" t="s">
         <v>425</v>
@@ -25197,18 +25197,16 @@
       </c>
       <c r="E37"/>
       <c r="G37" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H37" t="b">
-        <v>1</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="H37"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
         <v>426</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>9</v>
+        <v>364</v>
       </c>
       <c r="C38" t="s">
         <v>427</v>
@@ -25220,7 +25218,9 @@
       <c r="G38" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H38"/>
+      <c r="H38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
@@ -25265,26 +25265,26 @@
         <v>432</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
         <v>433</v>
-      </c>
-      <c r="C41" t="s">
-        <v>434</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E41"/>
       <c r="G41" s="3" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="H41"/>
     </row>
     <row r="42">
       <c r="A42" t="s">
+        <v>434</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>435</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C42" t="s">
         <v>436</v>
@@ -25303,7 +25303,7 @@
         <v>437</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>364</v>
+        <v>9</v>
       </c>
       <c r="C43" t="s">
         <v>438</v>
@@ -25313,7 +25313,7 @@
       </c>
       <c r="E43"/>
       <c r="G43" s="3" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="H43"/>
     </row>
@@ -25322,13 +25322,13 @@
         <v>439</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>29</v>
+        <v>364</v>
       </c>
       <c r="C44" t="s">
         <v>440</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>441</v>
+        <v>18</v>
       </c>
       <c r="E44"/>
       <c r="G44" s="3" t="s">
@@ -25338,16 +25338,16 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C45" t="s">
+        <v>442</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>443</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>444</v>
       </c>
       <c r="E45"/>
       <c r="G45" s="3" t="s">
@@ -25357,16 +25357,16 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C46" t="s">
+        <v>445</v>
+      </c>
+      <c r="D46" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>447</v>
       </c>
       <c r="E46"/>
       <c r="G46" s="3" t="s">
@@ -25376,16 +25376,16 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
+        <v>447</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47" t="s">
         <v>448</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="D47" s="3" t="s">
         <v>449</v>
-      </c>
-      <c r="C47" t="s">
-        <v>449</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="E47"/>
       <c r="G47" s="3" t="s">
@@ -25420,7 +25420,7 @@
         <v>453</v>
       </c>
       <c r="C49" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>18</v>
@@ -25433,10 +25433,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>454</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>455</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>456</v>
       </c>
       <c r="C50" t="s">
         <v>456</v>
@@ -25458,7 +25458,7 @@
         <v>458</v>
       </c>
       <c r="C51" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>18</v>
@@ -25471,13 +25471,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
+        <v>459</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="C52" t="s">
         <v>461</v>
-      </c>
-      <c r="C52" t="s">
-        <v>462</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>18</v>
@@ -25490,13 +25490,13 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
+        <v>462</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="C53" t="s">
-        <v>18</v>
+        <v>464</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>18</v>
@@ -25509,13 +25509,13 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>465</v>
+        <v>9</v>
       </c>
       <c r="C54" t="s">
-        <v>466</v>
+        <v>18</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>18</v>
@@ -25528,13 +25528,13 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
+        <v>466</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>467</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="C55" t="s">
         <v>468</v>
-      </c>
-      <c r="C55" t="s">
-        <v>469</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>18</v>
@@ -25547,13 +25547,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
+        <v>469</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>470</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="C56" t="s">
         <v>471</v>
-      </c>
-      <c r="C56" t="s">
-        <v>472</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>18</v>
@@ -25566,10 +25566,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
+        <v>472</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C57" t="s">
         <v>474</v>
@@ -25626,10 +25626,10 @@
         <v>479</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" t="s">
         <v>480</v>
-      </c>
-      <c r="C60" t="s">
-        <v>481</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>18</v>
@@ -25642,13 +25642,13 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
+        <v>481</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>482</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="C61" t="s">
         <v>483</v>
-      </c>
-      <c r="C61" t="s">
-        <v>484</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>18</v>
@@ -25661,10 +25661,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
+        <v>484</v>
+      </c>
+      <c r="B62" s="3" t="s">
         <v>485</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C62" t="s">
         <v>486</v>
@@ -25683,7 +25683,7 @@
         <v>487</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C63" t="s">
         <v>488</v>
@@ -25721,7 +25721,7 @@
         <v>491</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C65" t="s">
         <v>492</v>
@@ -25740,7 +25740,7 @@
         <v>493</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>480</v>
+        <v>9</v>
       </c>
       <c r="C66" t="s">
         <v>494</v>
@@ -25759,7 +25759,7 @@
         <v>495</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C67" t="s">
         <v>496</v>
@@ -25778,7 +25778,7 @@
         <v>497</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>39</v>
+        <v>482</v>
       </c>
       <c r="C68" t="s">
         <v>498</v>
@@ -25816,7 +25816,7 @@
         <v>501</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>393</v>
+        <v>39</v>
       </c>
       <c r="C70" t="s">
         <v>502</v>
@@ -25835,7 +25835,7 @@
         <v>503</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>9</v>
+        <v>393</v>
       </c>
       <c r="C71" t="s">
         <v>504</v>
@@ -25854,7 +25854,7 @@
         <v>505</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>393</v>
+        <v>9</v>
       </c>
       <c r="C72" t="s">
         <v>506</v>
@@ -25873,10 +25873,10 @@
         <v>507</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>9</v>
+        <v>393</v>
       </c>
       <c r="C73" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>18</v>
@@ -25889,13 +25889,13 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>509</v>
+        <v>9</v>
       </c>
       <c r="C74" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>18</v>
@@ -25908,10 +25908,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
+        <v>510</v>
+      </c>
+      <c r="B75" s="3" t="s">
         <v>511</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>393</v>
       </c>
       <c r="C75" t="s">
         <v>512</v>
@@ -25930,7 +25930,7 @@
         <v>513</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>514</v>
+        <v>393</v>
       </c>
       <c r="C76" t="s">
         <v>514</v>
@@ -25952,7 +25952,7 @@
         <v>516</v>
       </c>
       <c r="C77" t="s">
-        <v>18</v>
+        <v>516</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>18</v>
@@ -27319,7 +27319,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B175" t="s">
         <v>566</v>
@@ -27352,10 +27352,10 @@
     <row r="177">
       <c r="A177"/>
       <c r="B177" t="s">
-        <v>341</v>
+        <v>570</v>
       </c>
       <c r="C177" t="s">
-        <v>342</v>
+        <v>571</v>
       </c>
       <c r="D177" t="s">
         <v>18</v>
@@ -27364,32 +27364,43 @@
         <v>18</v>
       </c>
     </row>
+    <row r="178">
+      <c r="A178"/>
+      <c r="B178" t="s">
+        <v>572</v>
+      </c>
+      <c r="C178" t="s">
+        <v>573</v>
+      </c>
+      <c r="D178" t="s">
+        <v>18</v>
+      </c>
+      <c r="E178" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="179">
-      <c r="A179" t="s">
-        <v>1</v>
-      </c>
+      <c r="A179"/>
       <c r="B179" t="s">
-        <v>123</v>
+        <v>574</v>
       </c>
       <c r="C179" t="s">
-        <v>2</v>
+        <v>575</v>
       </c>
       <c r="D179" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E179" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="s">
-        <v>415</v>
-      </c>
+      <c r="A180"/>
       <c r="B180" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="C180" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D180" t="s">
         <v>18</v>
@@ -27401,10 +27412,10 @@
     <row r="181">
       <c r="A181"/>
       <c r="B181" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C181" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D181" t="s">
         <v>18</v>
@@ -27413,32 +27424,43 @@
         <v>18</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182"/>
+      <c r="B182" t="s">
+        <v>580</v>
+      </c>
+      <c r="C182" t="s">
+        <v>581</v>
+      </c>
+      <c r="D182" t="s">
+        <v>18</v>
+      </c>
+      <c r="E182" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="183">
-      <c r="A183" t="s">
-        <v>1</v>
-      </c>
+      <c r="A183"/>
       <c r="B183" t="s">
-        <v>123</v>
+        <v>582</v>
       </c>
       <c r="C183" t="s">
-        <v>2</v>
+        <v>583</v>
       </c>
       <c r="D183" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E183" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="s">
-        <v>433</v>
-      </c>
+      <c r="A184"/>
       <c r="B184" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="C184" t="s">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="D184" t="s">
         <v>18</v>
@@ -27450,10 +27472,10 @@
     <row r="185">
       <c r="A185"/>
       <c r="B185" t="s">
-        <v>276</v>
+        <v>586</v>
       </c>
       <c r="C185" t="s">
-        <v>277</v>
+        <v>587</v>
       </c>
       <c r="D185" t="s">
         <v>18</v>
@@ -27465,10 +27487,10 @@
     <row r="186">
       <c r="A186"/>
       <c r="B186" t="s">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="C186" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="D186" t="s">
         <v>18</v>
@@ -27480,10 +27502,10 @@
     <row r="187">
       <c r="A187"/>
       <c r="B187" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="C187" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="D187" t="s">
         <v>18</v>
@@ -27495,10 +27517,10 @@
     <row r="188">
       <c r="A188"/>
       <c r="B188" t="s">
-        <v>578</v>
+        <v>268</v>
       </c>
       <c r="C188" t="s">
-        <v>578</v>
+        <v>269</v>
       </c>
       <c r="D188" t="s">
         <v>18</v>
@@ -27510,10 +27532,10 @@
     <row r="189">
       <c r="A189"/>
       <c r="B189" t="s">
-        <v>579</v>
+        <v>592</v>
       </c>
       <c r="C189" t="s">
-        <v>580</v>
+        <v>593</v>
       </c>
       <c r="D189" t="s">
         <v>18</v>
@@ -27525,10 +27547,10 @@
     <row r="190">
       <c r="A190"/>
       <c r="B190" t="s">
-        <v>581</v>
+        <v>594</v>
       </c>
       <c r="C190" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="D190" t="s">
         <v>18</v>
@@ -27540,10 +27562,10 @@
     <row r="191">
       <c r="A191"/>
       <c r="B191" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="C191" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="D191" t="s">
         <v>18</v>
@@ -27555,10 +27577,10 @@
     <row r="192">
       <c r="A192"/>
       <c r="B192" t="s">
-        <v>260</v>
+        <v>598</v>
       </c>
       <c r="C192" t="s">
-        <v>262</v>
+        <v>599</v>
       </c>
       <c r="D192" t="s">
         <v>18</v>
@@ -27567,32 +27589,43 @@
         <v>18</v>
       </c>
     </row>
+    <row r="193">
+      <c r="A193"/>
+      <c r="B193" t="s">
+        <v>600</v>
+      </c>
+      <c r="C193" t="s">
+        <v>601</v>
+      </c>
+      <c r="D193" t="s">
+        <v>18</v>
+      </c>
+      <c r="E193" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="194">
-      <c r="A194" t="s">
-        <v>1</v>
-      </c>
+      <c r="A194"/>
       <c r="B194" t="s">
-        <v>123</v>
+        <v>602</v>
       </c>
       <c r="C194" t="s">
-        <v>2</v>
+        <v>603</v>
       </c>
       <c r="D194" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E194" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="s">
-        <v>468</v>
-      </c>
+      <c r="A195"/>
       <c r="B195" t="s">
-        <v>584</v>
+        <v>604</v>
       </c>
       <c r="C195" t="s">
-        <v>585</v>
+        <v>605</v>
       </c>
       <c r="D195" t="s">
         <v>18</v>
@@ -27604,10 +27637,10 @@
     <row r="196">
       <c r="A196"/>
       <c r="B196" t="s">
-        <v>586</v>
+        <v>606</v>
       </c>
       <c r="C196" t="s">
-        <v>587</v>
+        <v>607</v>
       </c>
       <c r="D196" t="s">
         <v>18</v>
@@ -27616,32 +27649,43 @@
         <v>18</v>
       </c>
     </row>
+    <row r="197">
+      <c r="A197"/>
+      <c r="B197" t="s">
+        <v>608</v>
+      </c>
+      <c r="C197" t="s">
+        <v>609</v>
+      </c>
+      <c r="D197" t="s">
+        <v>18</v>
+      </c>
+      <c r="E197" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="198">
-      <c r="A198" t="s">
-        <v>1</v>
-      </c>
+      <c r="A198"/>
       <c r="B198" t="s">
-        <v>123</v>
+        <v>610</v>
       </c>
       <c r="C198" t="s">
-        <v>2</v>
+        <v>611</v>
       </c>
       <c r="D198" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E198" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="s">
-        <v>483</v>
-      </c>
+      <c r="A199"/>
       <c r="B199" t="s">
-        <v>588</v>
+        <v>612</v>
       </c>
       <c r="C199" t="s">
-        <v>589</v>
+        <v>613</v>
       </c>
       <c r="D199" t="s">
         <v>18</v>
@@ -27653,10 +27697,10 @@
     <row r="200">
       <c r="A200"/>
       <c r="B200" t="s">
-        <v>590</v>
+        <v>614</v>
       </c>
       <c r="C200" t="s">
-        <v>591</v>
+        <v>615</v>
       </c>
       <c r="D200" t="s">
         <v>18</v>
@@ -27668,10 +27712,10 @@
     <row r="201">
       <c r="A201"/>
       <c r="B201" t="s">
-        <v>274</v>
+        <v>616</v>
       </c>
       <c r="C201" t="s">
-        <v>592</v>
+        <v>617</v>
       </c>
       <c r="D201" t="s">
         <v>18</v>
@@ -27683,10 +27727,10 @@
     <row r="202">
       <c r="A202"/>
       <c r="B202" t="s">
-        <v>341</v>
+        <v>618</v>
       </c>
       <c r="C202" t="s">
-        <v>342</v>
+        <v>619</v>
       </c>
       <c r="D202" t="s">
         <v>18</v>
@@ -27698,10 +27742,10 @@
     <row r="203">
       <c r="A203"/>
       <c r="B203" t="s">
-        <v>260</v>
+        <v>620</v>
       </c>
       <c r="C203" t="s">
-        <v>262</v>
+        <v>621</v>
       </c>
       <c r="D203" t="s">
         <v>18</v>
@@ -27710,32 +27754,43 @@
         <v>18</v>
       </c>
     </row>
+    <row r="204">
+      <c r="A204"/>
+      <c r="B204" t="s">
+        <v>622</v>
+      </c>
+      <c r="C204" t="s">
+        <v>623</v>
+      </c>
+      <c r="D204" t="s">
+        <v>18</v>
+      </c>
+      <c r="E204" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="205">
-      <c r="A205" t="s">
-        <v>1</v>
-      </c>
+      <c r="A205"/>
       <c r="B205" t="s">
-        <v>123</v>
+        <v>624</v>
       </c>
       <c r="C205" t="s">
-        <v>2</v>
+        <v>625</v>
       </c>
       <c r="D205" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E205" t="s">
-        <v>124</v>
+        <v>18</v>
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="s">
-        <v>509</v>
-      </c>
+      <c r="A206"/>
       <c r="B206" t="s">
-        <v>593</v>
+        <v>626</v>
       </c>
       <c r="C206" t="s">
-        <v>594</v>
+        <v>627</v>
       </c>
       <c r="D206" t="s">
         <v>18</v>
@@ -27747,10 +27802,10 @@
     <row r="207">
       <c r="A207"/>
       <c r="B207" t="s">
-        <v>595</v>
+        <v>628</v>
       </c>
       <c r="C207" t="s">
-        <v>596</v>
+        <v>629</v>
       </c>
       <c r="D207" t="s">
         <v>18</v>
@@ -27762,10 +27817,10 @@
     <row r="208">
       <c r="A208"/>
       <c r="B208" t="s">
-        <v>597</v>
+        <v>630</v>
       </c>
       <c r="C208" t="s">
-        <v>598</v>
+        <v>631</v>
       </c>
       <c r="D208" t="s">
         <v>18</v>
@@ -27777,10 +27832,10 @@
     <row r="209">
       <c r="A209"/>
       <c r="B209" t="s">
-        <v>599</v>
+        <v>632</v>
       </c>
       <c r="C209" t="s">
-        <v>600</v>
+        <v>633</v>
       </c>
       <c r="D209" t="s">
         <v>18</v>
@@ -27792,10 +27847,10 @@
     <row r="210">
       <c r="A210"/>
       <c r="B210" t="s">
-        <v>601</v>
+        <v>634</v>
       </c>
       <c r="C210" t="s">
-        <v>602</v>
+        <v>635</v>
       </c>
       <c r="D210" t="s">
         <v>18</v>
@@ -27807,10 +27862,10 @@
     <row r="211">
       <c r="A211"/>
       <c r="B211" t="s">
-        <v>603</v>
+        <v>636</v>
       </c>
       <c r="C211" t="s">
-        <v>604</v>
+        <v>637</v>
       </c>
       <c r="D211" t="s">
         <v>18</v>
@@ -27822,10 +27877,10 @@
     <row r="212">
       <c r="A212"/>
       <c r="B212" t="s">
-        <v>605</v>
+        <v>638</v>
       </c>
       <c r="C212" t="s">
-        <v>606</v>
+        <v>639</v>
       </c>
       <c r="D212" t="s">
         <v>18</v>
@@ -27837,10 +27892,10 @@
     <row r="213">
       <c r="A213"/>
       <c r="B213" t="s">
-        <v>607</v>
+        <v>640</v>
       </c>
       <c r="C213" t="s">
-        <v>608</v>
+        <v>641</v>
       </c>
       <c r="D213" t="s">
         <v>18</v>
@@ -27852,10 +27907,10 @@
     <row r="214">
       <c r="A214"/>
       <c r="B214" t="s">
-        <v>260</v>
+        <v>642</v>
       </c>
       <c r="C214" t="s">
-        <v>262</v>
+        <v>643</v>
       </c>
       <c r="D214" t="s">
         <v>18</v>
@@ -27864,47 +27919,47 @@
         <v>18</v>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" t="s">
-        <v>1</v>
-      </c>
-      <c r="B216" t="s">
-        <v>123</v>
-      </c>
-      <c r="C216" t="s">
-        <v>2</v>
-      </c>
-      <c r="D216" t="s">
-        <v>3</v>
-      </c>
-      <c r="E216" t="s">
-        <v>124</v>
+    <row r="215">
+      <c r="A215"/>
+      <c r="B215" t="s">
+        <v>644</v>
+      </c>
+      <c r="C215" t="s">
+        <v>645</v>
+      </c>
+      <c r="D215" t="s">
+        <v>18</v>
+      </c>
+      <c r="E215" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>514</v>
+        <v>1</v>
       </c>
       <c r="B217" t="s">
-        <v>609</v>
+        <v>123</v>
       </c>
       <c r="C217" t="s">
-        <v>610</v>
+        <v>2</v>
       </c>
       <c r="D217" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E217" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="218">
-      <c r="A218"/>
+      <c r="A218" t="s">
+        <v>407</v>
+      </c>
       <c r="B218" t="s">
-        <v>611</v>
+        <v>646</v>
       </c>
       <c r="C218" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="D218" t="s">
         <v>18</v>
@@ -27916,10 +27971,10 @@
     <row r="219">
       <c r="A219"/>
       <c r="B219" t="s">
-        <v>613</v>
+        <v>648</v>
       </c>
       <c r="C219" t="s">
-        <v>614</v>
+        <v>649</v>
       </c>
       <c r="D219" t="s">
         <v>18</v>
@@ -27962,13 +28017,13 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>516</v>
+        <v>417</v>
       </c>
       <c r="B223" t="s">
-        <v>615</v>
+        <v>650</v>
       </c>
       <c r="C223" t="s">
-        <v>616</v>
+        <v>651</v>
       </c>
       <c r="D223" t="s">
         <v>18</v>
@@ -27980,10 +28035,10 @@
     <row r="224">
       <c r="A224"/>
       <c r="B224" t="s">
-        <v>617</v>
+        <v>652</v>
       </c>
       <c r="C224" t="s">
-        <v>618</v>
+        <v>653</v>
       </c>
       <c r="D224" t="s">
         <v>18</v>
@@ -27992,43 +28047,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="225">
-      <c r="A225"/>
-      <c r="B225" t="s">
-        <v>619</v>
-      </c>
-      <c r="C225" t="s">
-        <v>620</v>
-      </c>
-      <c r="D225" t="s">
-        <v>18</v>
-      </c>
-      <c r="E225" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="226">
-      <c r="A226"/>
+      <c r="A226" t="s">
+        <v>1</v>
+      </c>
       <c r="B226" t="s">
-        <v>621</v>
+        <v>123</v>
       </c>
       <c r="C226" t="s">
-        <v>622</v>
+        <v>2</v>
       </c>
       <c r="D226" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E226" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="227">
-      <c r="A227"/>
+      <c r="A227" t="s">
+        <v>435</v>
+      </c>
       <c r="B227" t="s">
-        <v>623</v>
+        <v>654</v>
       </c>
       <c r="C227" t="s">
-        <v>624</v>
+        <v>655</v>
       </c>
       <c r="D227" t="s">
         <v>18</v>
@@ -28040,10 +28084,10 @@
     <row r="228">
       <c r="A228"/>
       <c r="B228" t="s">
-        <v>625</v>
+        <v>276</v>
       </c>
       <c r="C228" t="s">
-        <v>626</v>
+        <v>277</v>
       </c>
       <c r="D228" t="s">
         <v>18</v>
@@ -28055,10 +28099,10 @@
     <row r="229">
       <c r="A229"/>
       <c r="B229" t="s">
-        <v>627</v>
+        <v>656</v>
       </c>
       <c r="C229" t="s">
-        <v>628</v>
+        <v>656</v>
       </c>
       <c r="D229" t="s">
         <v>18</v>
@@ -28070,10 +28114,10 @@
     <row r="230">
       <c r="A230"/>
       <c r="B230" t="s">
-        <v>629</v>
+        <v>657</v>
       </c>
       <c r="C230" t="s">
-        <v>630</v>
+        <v>657</v>
       </c>
       <c r="D230" t="s">
         <v>18</v>
@@ -28085,10 +28129,10 @@
     <row r="231">
       <c r="A231"/>
       <c r="B231" t="s">
-        <v>631</v>
+        <v>658</v>
       </c>
       <c r="C231" t="s">
-        <v>632</v>
+        <v>658</v>
       </c>
       <c r="D231" t="s">
         <v>18</v>
@@ -28100,10 +28144,10 @@
     <row r="232">
       <c r="A232"/>
       <c r="B232" t="s">
-        <v>633</v>
+        <v>659</v>
       </c>
       <c r="C232" t="s">
-        <v>634</v>
+        <v>660</v>
       </c>
       <c r="D232" t="s">
         <v>18</v>
@@ -28115,10 +28159,10 @@
     <row r="233">
       <c r="A233"/>
       <c r="B233" t="s">
-        <v>635</v>
+        <v>661</v>
       </c>
       <c r="C233" t="s">
-        <v>636</v>
+        <v>661</v>
       </c>
       <c r="D233" t="s">
         <v>18</v>
@@ -28130,10 +28174,10 @@
     <row r="234">
       <c r="A234"/>
       <c r="B234" t="s">
-        <v>637</v>
+        <v>662</v>
       </c>
       <c r="C234" t="s">
-        <v>638</v>
+        <v>663</v>
       </c>
       <c r="D234" t="s">
         <v>18</v>
@@ -28145,10 +28189,10 @@
     <row r="235">
       <c r="A235"/>
       <c r="B235" t="s">
-        <v>639</v>
+        <v>260</v>
       </c>
       <c r="C235" t="s">
-        <v>640</v>
+        <v>262</v>
       </c>
       <c r="D235" t="s">
         <v>18</v>
@@ -28157,43 +28201,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="236">
-      <c r="A236"/>
-      <c r="B236" t="s">
-        <v>268</v>
-      </c>
-      <c r="C236" t="s">
-        <v>269</v>
-      </c>
-      <c r="D236" t="s">
-        <v>18</v>
-      </c>
-      <c r="E236" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="237">
-      <c r="A237"/>
+      <c r="A237" t="s">
+        <v>1</v>
+      </c>
       <c r="B237" t="s">
-        <v>641</v>
+        <v>123</v>
       </c>
       <c r="C237" t="s">
-        <v>642</v>
+        <v>2</v>
       </c>
       <c r="D237" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E237" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="238">
-      <c r="A238"/>
+      <c r="A238" t="s">
+        <v>470</v>
+      </c>
       <c r="B238" t="s">
-        <v>643</v>
+        <v>664</v>
       </c>
       <c r="C238" t="s">
-        <v>644</v>
+        <v>665</v>
       </c>
       <c r="D238" t="s">
         <v>18</v>
@@ -28205,10 +28238,10 @@
     <row r="239">
       <c r="A239"/>
       <c r="B239" t="s">
-        <v>645</v>
+        <v>666</v>
       </c>
       <c r="C239" t="s">
-        <v>646</v>
+        <v>667</v>
       </c>
       <c r="D239" t="s">
         <v>18</v>
@@ -28217,43 +28250,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="240">
-      <c r="A240"/>
-      <c r="B240" t="s">
-        <v>601</v>
-      </c>
-      <c r="C240" t="s">
-        <v>602</v>
-      </c>
-      <c r="D240" t="s">
-        <v>18</v>
-      </c>
-      <c r="E240" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="241">
-      <c r="A241"/>
+      <c r="A241" t="s">
+        <v>1</v>
+      </c>
       <c r="B241" t="s">
-        <v>647</v>
+        <v>123</v>
       </c>
       <c r="C241" t="s">
-        <v>648</v>
+        <v>2</v>
       </c>
       <c r="D241" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E241" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="242">
-      <c r="A242"/>
+      <c r="A242" t="s">
+        <v>485</v>
+      </c>
       <c r="B242" t="s">
-        <v>649</v>
+        <v>668</v>
       </c>
       <c r="C242" t="s">
-        <v>650</v>
+        <v>669</v>
       </c>
       <c r="D242" t="s">
         <v>18</v>
@@ -28265,10 +28287,10 @@
     <row r="243">
       <c r="A243"/>
       <c r="B243" t="s">
-        <v>651</v>
+        <v>670</v>
       </c>
       <c r="C243" t="s">
-        <v>652</v>
+        <v>671</v>
       </c>
       <c r="D243" t="s">
         <v>18</v>
@@ -28280,10 +28302,10 @@
     <row r="244">
       <c r="A244"/>
       <c r="B244" t="s">
-        <v>653</v>
+        <v>274</v>
       </c>
       <c r="C244" t="s">
-        <v>654</v>
+        <v>672</v>
       </c>
       <c r="D244" t="s">
         <v>18</v>
@@ -28295,10 +28317,10 @@
     <row r="245">
       <c r="A245"/>
       <c r="B245" t="s">
-        <v>655</v>
+        <v>341</v>
       </c>
       <c r="C245" t="s">
-        <v>656</v>
+        <v>342</v>
       </c>
       <c r="D245" t="s">
         <v>18</v>
@@ -28310,10 +28332,10 @@
     <row r="246">
       <c r="A246"/>
       <c r="B246" t="s">
-        <v>657</v>
+        <v>260</v>
       </c>
       <c r="C246" t="s">
-        <v>658</v>
+        <v>262</v>
       </c>
       <c r="D246" t="s">
         <v>18</v>
@@ -28322,43 +28344,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="247">
-      <c r="A247"/>
-      <c r="B247" t="s">
-        <v>659</v>
-      </c>
-      <c r="C247" t="s">
-        <v>660</v>
-      </c>
-      <c r="D247" t="s">
-        <v>18</v>
-      </c>
-      <c r="E247" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="248">
-      <c r="A248"/>
+      <c r="A248" t="s">
+        <v>1</v>
+      </c>
       <c r="B248" t="s">
-        <v>661</v>
+        <v>123</v>
       </c>
       <c r="C248" t="s">
-        <v>662</v>
+        <v>2</v>
       </c>
       <c r="D248" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E248" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="249">
-      <c r="A249"/>
+      <c r="A249" t="s">
+        <v>511</v>
+      </c>
       <c r="B249" t="s">
-        <v>663</v>
+        <v>673</v>
       </c>
       <c r="C249" t="s">
-        <v>664</v>
+        <v>674</v>
       </c>
       <c r="D249" t="s">
         <v>18</v>
@@ -28370,10 +28381,10 @@
     <row r="250">
       <c r="A250"/>
       <c r="B250" t="s">
-        <v>665</v>
+        <v>675</v>
       </c>
       <c r="C250" t="s">
-        <v>666</v>
+        <v>676</v>
       </c>
       <c r="D250" t="s">
         <v>18</v>
@@ -28385,10 +28396,10 @@
     <row r="251">
       <c r="A251"/>
       <c r="B251" t="s">
-        <v>667</v>
+        <v>677</v>
       </c>
       <c r="C251" t="s">
-        <v>668</v>
+        <v>678</v>
       </c>
       <c r="D251" t="s">
         <v>18</v>
@@ -28400,10 +28411,10 @@
     <row r="252">
       <c r="A252"/>
       <c r="B252" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="C252" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="D252" t="s">
         <v>18</v>
@@ -28415,10 +28426,10 @@
     <row r="253">
       <c r="A253"/>
       <c r="B253" t="s">
-        <v>671</v>
+        <v>598</v>
       </c>
       <c r="C253" t="s">
-        <v>672</v>
+        <v>599</v>
       </c>
       <c r="D253" t="s">
         <v>18</v>
@@ -28430,10 +28441,10 @@
     <row r="254">
       <c r="A254"/>
       <c r="B254" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="C254" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="D254" t="s">
         <v>18</v>
@@ -28445,10 +28456,10 @@
     <row r="255">
       <c r="A255"/>
       <c r="B255" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="C255" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="D255" t="s">
         <v>18</v>
@@ -28460,10 +28471,10 @@
     <row r="256">
       <c r="A256"/>
       <c r="B256" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="C256" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="D256" t="s">
         <v>18</v>
@@ -28475,10 +28486,10 @@
     <row r="257">
       <c r="A257"/>
       <c r="B257" t="s">
-        <v>679</v>
+        <v>260</v>
       </c>
       <c r="C257" t="s">
-        <v>680</v>
+        <v>262</v>
       </c>
       <c r="D257" t="s">
         <v>18</v>
@@ -28487,43 +28498,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="258">
-      <c r="A258"/>
-      <c r="B258" t="s">
-        <v>681</v>
-      </c>
-      <c r="C258" t="s">
-        <v>682</v>
-      </c>
-      <c r="D258" t="s">
-        <v>18</v>
-      </c>
-      <c r="E258" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="259">
-      <c r="A259"/>
+      <c r="A259" t="s">
+        <v>1</v>
+      </c>
       <c r="B259" t="s">
-        <v>683</v>
+        <v>123</v>
       </c>
       <c r="C259" t="s">
-        <v>684</v>
+        <v>2</v>
       </c>
       <c r="D259" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E259" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260"/>
+      <c r="A260" t="s">
+        <v>516</v>
+      </c>
       <c r="B260" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C260" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D260" t="s">
         <v>18</v>
@@ -28535,10 +28535,10 @@
     <row r="261">
       <c r="A261"/>
       <c r="B261" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="C261" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="D261" t="s">
         <v>18</v>
@@ -28550,10 +28550,10 @@
     <row r="262">
       <c r="A262"/>
       <c r="B262" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="C262" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="D262" t="s">
         <v>18</v>
@@ -28565,10 +28565,10 @@
     <row r="263">
       <c r="A263"/>
       <c r="B263" t="s">
-        <v>691</v>
+        <v>341</v>
       </c>
       <c r="C263" t="s">
-        <v>692</v>
+        <v>342</v>
       </c>
       <c r="D263" t="s">
         <v>18</v>
@@ -29811,7 +29811,7 @@
         <v>839</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C45" t="s">
         <v>840</v>
@@ -29830,7 +29830,7 @@
         <v>841</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C46" t="s">
         <v>842</v>
@@ -29868,7 +29868,7 @@
         <v>845</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C48" t="s">
         <v>846</v>
@@ -29887,7 +29887,7 @@
         <v>847</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C49" t="s">
         <v>848</v>
@@ -29906,7 +29906,7 @@
         <v>849</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C50" t="s">
         <v>850</v>
@@ -29944,7 +29944,7 @@
         <v>854</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C52" t="s">
         <v>855</v>
@@ -30077,7 +30077,7 @@
         <v>865</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C59" t="s">
         <v>866</v>
@@ -30115,7 +30115,7 @@
         <v>869</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C61" t="s">
         <v>870</v>
@@ -30891,7 +30891,7 @@
         <v>969</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C101" t="s">
         <v>970</v>
@@ -33471,7 +33471,7 @@
         <v>1276</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C51" t="s">
         <v>1277</v>
@@ -33874,13 +33874,13 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B79" t="s">
-        <v>566</v>
+        <v>646</v>
       </c>
       <c r="C79" t="s">
-        <v>567</v>
+        <v>647</v>
       </c>
       <c r="D79" t="s">
         <v>18</v>
@@ -33892,10 +33892,10 @@
     <row r="80">
       <c r="A80"/>
       <c r="B80" t="s">
-        <v>568</v>
+        <v>648</v>
       </c>
       <c r="C80" t="s">
-        <v>569</v>
+        <v>649</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -34525,7 +34525,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>1350</v>
@@ -35136,7 +35136,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>1350</v>

</xml_diff>

<commit_message>
#2728 do not count deleted participants
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7849" uniqueCount="2150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7849" uniqueCount="2152">
   <si>
     <t>Field</t>
   </si>
@@ -6331,7 +6331,13 @@
     <t>publicOwnership</t>
   </si>
   <si>
+    <t>Public ownership</t>
+  </si>
+  <si>
     <t>archived</t>
+  </si>
+  <si>
+    <t>Archived</t>
   </si>
   <si>
     <t>epidCode</t>
@@ -12776,7 +12782,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>584</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>18</v>
@@ -12795,7 +12801,7 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>587</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>18</v>
@@ -12814,7 +12820,7 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>590</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>18</v>
@@ -23223,7 +23229,7 @@
         <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>2098</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>18</v>
@@ -23236,13 +23242,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>133</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>2100</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>18</v>
@@ -24486,13 +24492,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2099</v>
+        <v>2101</v>
       </c>
       <c r="B3" s="20" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>2100</v>
+        <v>2102</v>
       </c>
       <c r="D3" s="20" t="s">
         <v>18</v>
@@ -24505,13 +24511,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2101</v>
+        <v>2103</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>2102</v>
+        <v>2104</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>18</v>
@@ -24524,13 +24530,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>133</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>2100</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>18</v>
@@ -24562,10 +24568,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2103</v>
+        <v>2105</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>2104</v>
+        <v>2106</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
@@ -24649,13 +24655,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2099</v>
+        <v>2101</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>2100</v>
+        <v>2102</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>18</v>
@@ -24668,13 +24674,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2101</v>
+        <v>2103</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>2102</v>
+        <v>2104</v>
       </c>
       <c r="D4" s="21" t="s">
         <v>18</v>
@@ -24706,13 +24712,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B6" s="21" t="s">
         <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>2100</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>18</v>
@@ -24850,13 +24856,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>133</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>2100</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>18</v>
@@ -24937,13 +24943,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2105</v>
+        <v>2107</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>133</v>
       </c>
       <c r="C2" t="s">
-        <v>2106</v>
+        <v>2108</v>
       </c>
       <c r="D2" s="23" t="s">
         <v>18</v>
@@ -24956,13 +24962,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2107</v>
+        <v>2109</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>2108</v>
+        <v>2110</v>
       </c>
       <c r="D3" s="23" t="s">
         <v>18</v>
@@ -25013,7 +25019,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2109</v>
+        <v>2111</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>9</v>
@@ -25057,7 +25063,7 @@
         <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>2110</v>
+        <v>2112</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>18</v>
@@ -25070,11 +25076,11 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2111</v>
+        <v>2113</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" t="s">
-        <v>2112</v>
+        <v>2114</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>18</v>
@@ -25087,10 +25093,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2103</v>
+        <v>2105</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>2104</v>
+        <v>2106</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
@@ -25182,7 +25188,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2113</v>
+        <v>2115</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>58</v>
@@ -25207,7 +25213,7 @@
         <v>615</v>
       </c>
       <c r="C16" t="s">
-        <v>2114</v>
+        <v>2116</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>18</v>
@@ -25220,13 +25226,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2115</v>
+        <v>2117</v>
       </c>
       <c r="B17" s="23" t="s">
         <v>498</v>
       </c>
       <c r="C17" t="s">
-        <v>2116</v>
+        <v>2118</v>
       </c>
       <c r="D17" s="23" t="s">
         <v>18</v>
@@ -25239,16 +25245,16 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2117</v>
+        <v>2119</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>2118</v>
+        <v>2120</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>2119</v>
+        <v>2121</v>
       </c>
       <c r="E18"/>
       <c r="G18" s="23" t="s">
@@ -25258,10 +25264,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2120</v>
+        <v>2122</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>2121</v>
+        <v>2123</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -26153,13 +26159,13 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>2121</v>
+        <v>2123</v>
       </c>
       <c r="B80" t="s">
-        <v>2122</v>
+        <v>2124</v>
       </c>
       <c r="C80" t="s">
-        <v>2123</v>
+        <v>2125</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -26171,10 +26177,10 @@
     <row r="81">
       <c r="A81"/>
       <c r="B81" t="s">
-        <v>2124</v>
+        <v>2126</v>
       </c>
       <c r="C81" t="s">
-        <v>2125</v>
+        <v>2127</v>
       </c>
       <c r="D81" t="s">
         <v>18</v>
@@ -26186,10 +26192,10 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>2126</v>
+        <v>2128</v>
       </c>
       <c r="C82" t="s">
-        <v>2127</v>
+        <v>2129</v>
       </c>
       <c r="D82" t="s">
         <v>18</v>
@@ -26201,10 +26207,10 @@
     <row r="83">
       <c r="A83"/>
       <c r="B83" t="s">
-        <v>2128</v>
+        <v>2130</v>
       </c>
       <c r="C83" t="s">
-        <v>2129</v>
+        <v>2131</v>
       </c>
       <c r="D83" t="s">
         <v>18</v>
@@ -26216,10 +26222,10 @@
     <row r="84">
       <c r="A84"/>
       <c r="B84" t="s">
-        <v>2130</v>
+        <v>2132</v>
       </c>
       <c r="C84" t="s">
-        <v>2131</v>
+        <v>2133</v>
       </c>
       <c r="D84" t="s">
         <v>18</v>
@@ -26231,10 +26237,10 @@
     <row r="85">
       <c r="A85"/>
       <c r="B85" t="s">
-        <v>2132</v>
+        <v>2134</v>
       </c>
       <c r="C85" t="s">
-        <v>2133</v>
+        <v>2135</v>
       </c>
       <c r="D85" t="s">
         <v>18</v>
@@ -26246,10 +26252,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>2134</v>
+        <v>2136</v>
       </c>
       <c r="C86" t="s">
-        <v>2135</v>
+        <v>2137</v>
       </c>
       <c r="D86" t="s">
         <v>18</v>
@@ -26261,10 +26267,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>2136</v>
+        <v>2138</v>
       </c>
       <c r="C87" t="s">
-        <v>2137</v>
+        <v>2139</v>
       </c>
       <c r="D87" t="s">
         <v>18</v>
@@ -26276,10 +26282,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>2138</v>
+        <v>2140</v>
       </c>
       <c r="C88" t="s">
-        <v>2139</v>
+        <v>2141</v>
       </c>
       <c r="D88" t="s">
         <v>18</v>
@@ -26291,10 +26297,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2140</v>
+        <v>2142</v>
       </c>
       <c r="C89" t="s">
-        <v>2141</v>
+        <v>2143</v>
       </c>
       <c r="D89" t="s">
         <v>18</v>
@@ -26306,10 +26312,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>2142</v>
+        <v>2144</v>
       </c>
       <c r="C90" t="s">
-        <v>2143</v>
+        <v>2145</v>
       </c>
       <c r="D90" t="s">
         <v>18</v>
@@ -26321,10 +26327,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>2144</v>
+        <v>2146</v>
       </c>
       <c r="C91" t="s">
-        <v>2145</v>
+        <v>2147</v>
       </c>
       <c r="D91" t="s">
         <v>18</v>
@@ -26336,10 +26342,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>2146</v>
+        <v>2148</v>
       </c>
       <c r="C92" t="s">
-        <v>2147</v>
+        <v>2149</v>
       </c>
       <c r="D92" t="s">
         <v>18</v>
@@ -26365,12 +26371,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>2148</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2149</v>
+        <v>2151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#4773 add missing sample material types
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11215" uniqueCount="2782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11235" uniqueCount="2792">
   <si>
     <t>Field</t>
   </si>
@@ -6789,6 +6789,36 @@
   </si>
   <si>
     <t>Brain tissue</t>
+  </si>
+  <si>
+    <t>ANTERIOR_NARES_SWAB</t>
+  </si>
+  <si>
+    <t>Anterior nares swab</t>
+  </si>
+  <si>
+    <t>OROPHARYNGEAL_ASPIRATE</t>
+  </si>
+  <si>
+    <t>Oropharyngeal aspirate</t>
+  </si>
+  <si>
+    <t>NASOPHARYNGEAL_ASPIRATE</t>
+  </si>
+  <si>
+    <t>Nasopharyngeal aspirate</t>
+  </si>
+  <si>
+    <t>LOWER_RESPIRATORY_SAMPLE</t>
+  </si>
+  <si>
+    <t>Lower respiratory sample</t>
+  </si>
+  <si>
+    <t>PLEURAL_FLUID_SPECIMEN</t>
+  </si>
+  <si>
+    <t>Pleural fluid specimen</t>
   </si>
   <si>
     <t>EXTERNAL</t>
@@ -8618,7 +8648,7 @@
 </file>
 
 <file path=xl/tables/table105.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="105" name="SampleSampleMaterial" displayName="SampleSampleMaterial" ref="A45:E65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="105" name="SampleSampleMaterial" displayName="SampleSampleMaterial" ref="A45:E70">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -8632,7 +8662,7 @@
 </file>
 
 <file path=xl/tables/table106.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="106" name="SampleSamplePurpose" displayName="SampleSamplePurpose" ref="A67:E69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="106" name="SampleSamplePurpose" displayName="SampleSamplePurpose" ref="A72:E74">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -8646,7 +8676,7 @@
 </file>
 
 <file path=xl/tables/table107.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="107" name="SampleSpecimenCondition" displayName="SampleSpecimenCondition" ref="A71:E73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="107" name="SampleSpecimenCondition" displayName="SampleSpecimenCondition" ref="A76:E78">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -8660,7 +8690,7 @@
 </file>
 
 <file path=xl/tables/table108.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="108" name="SampleSampleSource" displayName="SampleSampleSource" ref="A75:E78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="108" name="SampleSampleSource" displayName="SampleSampleSource" ref="A80:E83">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -8674,7 +8704,7 @@
 </file>
 
 <file path=xl/tables/table109.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="109" name="SamplePathogenTestResultType" displayName="SamplePathogenTestResultType" ref="A80:E85">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="109" name="SamplePathogenTestResultType" displayName="SamplePathogenTestResultType" ref="A85:E90">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -8702,7 +8732,7 @@
 </file>
 
 <file path=xl/tables/table110.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="110" name="SampleSamplingReason" displayName="SampleSamplingReason" ref="A87:E101">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="110" name="SampleSamplingReason" displayName="SampleSamplingReason" ref="A92:E106">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -22744,7 +22774,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -23990,10 +24020,10 @@
     <row r="65">
       <c r="A65"/>
       <c r="B65" t="s">
-        <v>179</v>
+        <v>2250</v>
       </c>
       <c r="C65" t="s">
-        <v>180</v>
+        <v>2251</v>
       </c>
       <c r="D65" t="s">
         <v>22</v>
@@ -24002,32 +24032,43 @@
         <v>22</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66"/>
+      <c r="B66" t="s">
+        <v>2252</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2253</v>
+      </c>
+      <c r="D66" t="s">
+        <v>22</v>
+      </c>
+      <c r="E66" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="67">
-      <c r="A67" t="s">
-        <v>1</v>
-      </c>
+      <c r="A67"/>
       <c r="B67" t="s">
-        <v>158</v>
+        <v>2254</v>
       </c>
       <c r="C67" t="s">
-        <v>3</v>
+        <v>2255</v>
       </c>
       <c r="D67" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E67" t="s">
-        <v>168</v>
+        <v>22</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="s">
-        <v>2166</v>
-      </c>
+      <c r="A68"/>
       <c r="B68" t="s">
-        <v>2250</v>
+        <v>2256</v>
       </c>
       <c r="C68" t="s">
-        <v>2251</v>
+        <v>2257</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
@@ -24039,10 +24080,10 @@
     <row r="69">
       <c r="A69"/>
       <c r="B69" t="s">
-        <v>2252</v>
+        <v>2258</v>
       </c>
       <c r="C69" t="s">
-        <v>2253</v>
+        <v>2259</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
@@ -24051,47 +24092,47 @@
         <v>22</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="s">
-        <v>1</v>
-      </c>
-      <c r="B71" t="s">
-        <v>158</v>
-      </c>
-      <c r="C71" t="s">
-        <v>3</v>
-      </c>
-      <c r="D71" t="s">
-        <v>4</v>
-      </c>
-      <c r="E71" t="s">
-        <v>168</v>
+    <row r="70">
+      <c r="A70"/>
+      <c r="B70" t="s">
+        <v>179</v>
+      </c>
+      <c r="C70" t="s">
+        <v>180</v>
+      </c>
+      <c r="D70" t="s">
+        <v>22</v>
+      </c>
+      <c r="E70" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>2178</v>
+        <v>1</v>
       </c>
       <c r="B72" t="s">
-        <v>2254</v>
+        <v>158</v>
       </c>
       <c r="C72" t="s">
-        <v>2255</v>
+        <v>3</v>
       </c>
       <c r="D72" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E72" t="s">
-        <v>22</v>
+        <v>168</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73"/>
+      <c r="A73" t="s">
+        <v>2166</v>
+      </c>
       <c r="B73" t="s">
-        <v>2256</v>
+        <v>2260</v>
       </c>
       <c r="C73" t="s">
-        <v>2257</v>
+        <v>2261</v>
       </c>
       <c r="D73" t="s">
         <v>22</v>
@@ -24100,47 +24141,47 @@
         <v>22</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="s">
-        <v>1</v>
-      </c>
-      <c r="B75" t="s">
-        <v>158</v>
-      </c>
-      <c r="C75" t="s">
-        <v>3</v>
-      </c>
-      <c r="D75" t="s">
-        <v>4</v>
-      </c>
-      <c r="E75" t="s">
-        <v>168</v>
+    <row r="74">
+      <c r="A74"/>
+      <c r="B74" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C74" t="s">
+        <v>2263</v>
+      </c>
+      <c r="D74" t="s">
+        <v>22</v>
+      </c>
+      <c r="E74" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>2184</v>
+        <v>1</v>
       </c>
       <c r="B76" t="s">
-        <v>2258</v>
+        <v>158</v>
       </c>
       <c r="C76" t="s">
-        <v>2259</v>
+        <v>3</v>
       </c>
       <c r="D76" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E76" t="s">
-        <v>22</v>
+        <v>168</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77"/>
+      <c r="A77" t="s">
+        <v>2178</v>
+      </c>
       <c r="B77" t="s">
-        <v>2260</v>
+        <v>2264</v>
       </c>
       <c r="C77" t="s">
-        <v>2261</v>
+        <v>2265</v>
       </c>
       <c r="D77" t="s">
         <v>22</v>
@@ -24152,10 +24193,10 @@
     <row r="78">
       <c r="A78"/>
       <c r="B78" t="s">
-        <v>2262</v>
+        <v>2266</v>
       </c>
       <c r="C78" t="s">
-        <v>2263</v>
+        <v>2267</v>
       </c>
       <c r="D78" t="s">
         <v>22</v>
@@ -24183,13 +24224,13 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>2193</v>
+        <v>2184</v>
       </c>
       <c r="B81" t="s">
-        <v>2264</v>
+        <v>2268</v>
       </c>
       <c r="C81" t="s">
-        <v>2265</v>
+        <v>2269</v>
       </c>
       <c r="D81" t="s">
         <v>22</v>
@@ -24201,10 +24242,10 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>936</v>
+        <v>2270</v>
       </c>
       <c r="C82" t="s">
-        <v>938</v>
+        <v>2271</v>
       </c>
       <c r="D82" t="s">
         <v>22</v>
@@ -24216,10 +24257,10 @@
     <row r="83">
       <c r="A83"/>
       <c r="B83" t="s">
-        <v>2266</v>
+        <v>2272</v>
       </c>
       <c r="C83" t="s">
-        <v>2267</v>
+        <v>2273</v>
       </c>
       <c r="D83" t="s">
         <v>22</v>
@@ -24228,62 +24269,62 @@
         <v>22</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84"/>
-      <c r="B84" t="s">
-        <v>2268</v>
-      </c>
-      <c r="C84" t="s">
-        <v>2269</v>
-      </c>
-      <c r="D84" t="s">
-        <v>22</v>
-      </c>
-      <c r="E84" t="s">
-        <v>22</v>
-      </c>
-    </row>
     <row r="85">
-      <c r="A85"/>
+      <c r="A85" t="s">
+        <v>1</v>
+      </c>
       <c r="B85" t="s">
-        <v>2270</v>
+        <v>158</v>
       </c>
       <c r="C85" t="s">
-        <v>2271</v>
+        <v>3</v>
       </c>
       <c r="D85" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E85" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>2193</v>
+      </c>
+      <c r="B86" t="s">
+        <v>2274</v>
+      </c>
+      <c r="C86" t="s">
+        <v>2275</v>
+      </c>
+      <c r="D86" t="s">
+        <v>22</v>
+      </c>
+      <c r="E86" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="s">
-        <v>1</v>
-      </c>
+      <c r="A87"/>
       <c r="B87" t="s">
-        <v>158</v>
+        <v>936</v>
       </c>
       <c r="C87" t="s">
-        <v>3</v>
+        <v>938</v>
       </c>
       <c r="D87" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E87" t="s">
-        <v>168</v>
+        <v>22</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="s">
-        <v>2208</v>
-      </c>
+      <c r="A88"/>
       <c r="B88" t="s">
-        <v>2272</v>
+        <v>2276</v>
       </c>
       <c r="C88" t="s">
-        <v>2273</v>
+        <v>2277</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -24295,10 +24336,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2274</v>
+        <v>2278</v>
       </c>
       <c r="C89" t="s">
-        <v>2275</v>
+        <v>2279</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -24310,10 +24351,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>919</v>
+        <v>2280</v>
       </c>
       <c r="C90" t="s">
-        <v>643</v>
+        <v>2281</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -24322,43 +24363,32 @@
         <v>22</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91"/>
-      <c r="B91" t="s">
-        <v>2276</v>
-      </c>
-      <c r="C91" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D91" t="s">
-        <v>22</v>
-      </c>
-      <c r="E91" t="s">
-        <v>22</v>
-      </c>
-    </row>
     <row r="92">
-      <c r="A92"/>
+      <c r="A92" t="s">
+        <v>1</v>
+      </c>
       <c r="B92" t="s">
-        <v>2278</v>
+        <v>158</v>
       </c>
       <c r="C92" t="s">
-        <v>2279</v>
+        <v>3</v>
       </c>
       <c r="D92" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E92" t="s">
-        <v>22</v>
+        <v>168</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93"/>
+      <c r="A93" t="s">
+        <v>2208</v>
+      </c>
       <c r="B93" t="s">
-        <v>2280</v>
+        <v>2282</v>
       </c>
       <c r="C93" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="D93" t="s">
         <v>22</v>
@@ -24370,10 +24400,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>2282</v>
+        <v>2284</v>
       </c>
       <c r="C94" t="s">
-        <v>2283</v>
+        <v>2285</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -24385,10 +24415,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
-        <v>2284</v>
+        <v>919</v>
       </c>
       <c r="C95" t="s">
-        <v>2285</v>
+        <v>643</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -24430,10 +24460,10 @@
     <row r="98">
       <c r="A98"/>
       <c r="B98" t="s">
-        <v>1071</v>
+        <v>2290</v>
       </c>
       <c r="C98" t="s">
-        <v>2290</v>
+        <v>2291</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -24445,10 +24475,10 @@
     <row r="99">
       <c r="A99"/>
       <c r="B99" t="s">
-        <v>2291</v>
+        <v>2292</v>
       </c>
       <c r="C99" t="s">
-        <v>791</v>
+        <v>2293</v>
       </c>
       <c r="D99" t="s">
         <v>22</v>
@@ -24460,10 +24490,10 @@
     <row r="100">
       <c r="A100"/>
       <c r="B100" t="s">
-        <v>185</v>
+        <v>2294</v>
       </c>
       <c r="C100" t="s">
-        <v>186</v>
+        <v>2295</v>
       </c>
       <c r="D100" t="s">
         <v>22</v>
@@ -24475,15 +24505,90 @@
     <row r="101">
       <c r="A101"/>
       <c r="B101" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C101" t="s">
+        <v>2297</v>
+      </c>
+      <c r="D101" t="s">
+        <v>22</v>
+      </c>
+      <c r="E101" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102"/>
+      <c r="B102" t="s">
+        <v>2298</v>
+      </c>
+      <c r="C102" t="s">
+        <v>2299</v>
+      </c>
+      <c r="D102" t="s">
+        <v>22</v>
+      </c>
+      <c r="E102" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103"/>
+      <c r="B103" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C103" t="s">
+        <v>2300</v>
+      </c>
+      <c r="D103" t="s">
+        <v>22</v>
+      </c>
+      <c r="E103" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104"/>
+      <c r="B104" t="s">
+        <v>2301</v>
+      </c>
+      <c r="C104" t="s">
+        <v>791</v>
+      </c>
+      <c r="D104" t="s">
+        <v>22</v>
+      </c>
+      <c r="E104" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105"/>
+      <c r="B105" t="s">
+        <v>185</v>
+      </c>
+      <c r="C105" t="s">
+        <v>186</v>
+      </c>
+      <c r="D105" t="s">
+        <v>22</v>
+      </c>
+      <c r="E105" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106"/>
+      <c r="B106" t="s">
         <v>1074</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C106" t="s">
         <v>847</v>
       </c>
-      <c r="D101" t="s">
-        <v>22</v>
-      </c>
-      <c r="E101" t="s">
+      <c r="D106" t="s">
+        <v>22</v>
+      </c>
+      <c r="E106" t="s">
         <v>22</v>
       </c>
     </row>
@@ -24557,7 +24662,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2292</v>
+        <v>2302</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>2187</v>
@@ -24581,17 +24686,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2293</v>
+        <v>2303</v>
       </c>
       <c r="B3" s="16" t="s">
         <v>91</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2294</v>
+        <v>2304</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>2295</v>
+        <v>2305</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -24605,17 +24710,17 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2296</v>
+        <v>2306</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>12</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2297</v>
+        <v>2307</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>2298</v>
+        <v>2308</v>
       </c>
       <c r="F4"/>
       <c r="H4" s="16" t="s">
@@ -24627,14 +24732,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2299</v>
+        <v>2309</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>12</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2300</v>
+        <v>2310</v>
       </c>
       <c r="E5" s="16" t="s">
         <v>22</v>
@@ -24649,17 +24754,17 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2301</v>
+        <v>2311</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>2302</v>
+        <v>2312</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2303</v>
+        <v>2313</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>2304</v>
+        <v>2314</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -24673,7 +24778,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2305</v>
+        <v>2315</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>12</v>
@@ -24682,10 +24787,10 @@
         <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>2306</v>
+        <v>2316</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>2307</v>
+        <v>2317</v>
       </c>
       <c r="F7"/>
       <c r="H7" s="16" t="s">
@@ -24697,17 +24802,17 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2308</v>
+        <v>2318</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>55</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2309</v>
+        <v>2319</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>2310</v>
+        <v>2320</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -24731,7 +24836,7 @@
         <v>230</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>2311</v>
+        <v>2321</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -24757,7 +24862,7 @@
         <v>2170</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>2312</v>
+        <v>2322</v>
       </c>
       <c r="F10"/>
       <c r="H10" s="16" t="s">
@@ -24769,7 +24874,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2313</v>
+        <v>2323</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>626</v>
@@ -24795,17 +24900,17 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2314</v>
+        <v>2324</v>
       </c>
       <c r="B12" s="16" t="s">
         <v>2193</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2315</v>
+        <v>2325</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>2316</v>
+        <v>2326</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -24819,7 +24924,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2317</v>
+        <v>2327</v>
       </c>
       <c r="B13" s="16" t="s">
         <v>12</v>
@@ -24828,10 +24933,10 @@
         <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>2318</v>
+        <v>2328</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>2319</v>
+        <v>2329</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -24845,17 +24950,17 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2320</v>
+        <v>2330</v>
       </c>
       <c r="B14" s="16" t="s">
         <v>140</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2321</v>
+        <v>2331</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>2322</v>
+        <v>2332</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -24869,17 +24974,17 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2323</v>
+        <v>2333</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>140</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2324</v>
+        <v>2334</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>2325</v>
+        <v>2335</v>
       </c>
       <c r="F15"/>
       <c r="H15" s="16" t="s">
@@ -24891,7 +24996,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2326</v>
+        <v>2336</v>
       </c>
       <c r="B16" s="16" t="s">
         <v>12</v>
@@ -24900,10 +25005,10 @@
         <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>2327</v>
+        <v>2337</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>2328</v>
+        <v>2338</v>
       </c>
       <c r="F16"/>
       <c r="H16" s="16" t="s">
@@ -24915,14 +25020,14 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2329</v>
+        <v>2339</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2330</v>
+        <v>2340</v>
       </c>
       <c r="E17" s="16" t="s">
         <v>22</v>
@@ -24961,14 +25066,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2331</v>
+        <v>2341</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>140</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2332</v>
+        <v>2342</v>
       </c>
       <c r="E19" s="16" t="s">
         <v>22</v>
@@ -25913,13 +26018,13 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>2302</v>
+        <v>2312</v>
       </c>
       <c r="B85" t="s">
-        <v>2333</v>
+        <v>2343</v>
       </c>
       <c r="C85" t="s">
-        <v>2334</v>
+        <v>2344</v>
       </c>
       <c r="D85" t="s">
         <v>22</v>
@@ -25931,10 +26036,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>2335</v>
+        <v>2345</v>
       </c>
       <c r="C86" t="s">
-        <v>2336</v>
+        <v>2346</v>
       </c>
       <c r="D86" t="s">
         <v>22</v>
@@ -25946,10 +26051,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>2337</v>
+        <v>2347</v>
       </c>
       <c r="C87" t="s">
-        <v>2338</v>
+        <v>2348</v>
       </c>
       <c r="D87" t="s">
         <v>22</v>
@@ -25961,10 +26066,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>2339</v>
+        <v>2349</v>
       </c>
       <c r="C88" t="s">
-        <v>2340</v>
+        <v>2350</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -25976,10 +26081,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2341</v>
+        <v>2351</v>
       </c>
       <c r="C89" t="s">
-        <v>2342</v>
+        <v>2352</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -25991,7 +26096,7 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>2343</v>
+        <v>2353</v>
       </c>
       <c r="C90" t="s">
         <v>1087</v>
@@ -26006,10 +26111,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>2344</v>
+        <v>2354</v>
       </c>
       <c r="C91" t="s">
-        <v>2345</v>
+        <v>2355</v>
       </c>
       <c r="D91" t="s">
         <v>22</v>
@@ -26021,10 +26126,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>2346</v>
+        <v>2356</v>
       </c>
       <c r="C92" t="s">
-        <v>2347</v>
+        <v>2357</v>
       </c>
       <c r="D92" t="s">
         <v>22</v>
@@ -26036,10 +26141,10 @@
     <row r="93">
       <c r="A93"/>
       <c r="B93" t="s">
-        <v>2348</v>
+        <v>2358</v>
       </c>
       <c r="C93" t="s">
-        <v>2349</v>
+        <v>2359</v>
       </c>
       <c r="D93" t="s">
         <v>22</v>
@@ -26051,10 +26156,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>2350</v>
+        <v>2360</v>
       </c>
       <c r="C94" t="s">
-        <v>2351</v>
+        <v>2361</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -26066,10 +26171,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
-        <v>2352</v>
+        <v>2362</v>
       </c>
       <c r="C95" t="s">
-        <v>2353</v>
+        <v>2363</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -26081,10 +26186,10 @@
     <row r="96">
       <c r="A96"/>
       <c r="B96" t="s">
-        <v>2354</v>
+        <v>2364</v>
       </c>
       <c r="C96" t="s">
-        <v>2355</v>
+        <v>2365</v>
       </c>
       <c r="D96" t="s">
         <v>22</v>
@@ -26096,10 +26201,10 @@
     <row r="97">
       <c r="A97"/>
       <c r="B97" t="s">
-        <v>2356</v>
+        <v>2366</v>
       </c>
       <c r="C97" t="s">
-        <v>2357</v>
+        <v>2367</v>
       </c>
       <c r="D97" t="s">
         <v>22</v>
@@ -26111,10 +26216,10 @@
     <row r="98">
       <c r="A98"/>
       <c r="B98" t="s">
-        <v>2358</v>
+        <v>2368</v>
       </c>
       <c r="C98" t="s">
-        <v>2359</v>
+        <v>2369</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -26126,10 +26231,10 @@
     <row r="99">
       <c r="A99"/>
       <c r="B99" t="s">
-        <v>2360</v>
+        <v>2370</v>
       </c>
       <c r="C99" t="s">
-        <v>2361</v>
+        <v>2371</v>
       </c>
       <c r="D99" t="s">
         <v>22</v>
@@ -26141,10 +26246,10 @@
     <row r="100">
       <c r="A100"/>
       <c r="B100" t="s">
-        <v>2362</v>
+        <v>2372</v>
       </c>
       <c r="C100" t="s">
-        <v>2363</v>
+        <v>2373</v>
       </c>
       <c r="D100" t="s">
         <v>22</v>
@@ -26156,10 +26261,10 @@
     <row r="101">
       <c r="A101"/>
       <c r="B101" t="s">
-        <v>2364</v>
+        <v>2374</v>
       </c>
       <c r="C101" t="s">
-        <v>2365</v>
+        <v>2375</v>
       </c>
       <c r="D101" t="s">
         <v>22</v>
@@ -26171,10 +26276,10 @@
     <row r="102">
       <c r="A102"/>
       <c r="B102" t="s">
-        <v>2366</v>
+        <v>2376</v>
       </c>
       <c r="C102" t="s">
-        <v>2367</v>
+        <v>2377</v>
       </c>
       <c r="D102" t="s">
         <v>22</v>
@@ -26186,10 +26291,10 @@
     <row r="103">
       <c r="A103"/>
       <c r="B103" t="s">
-        <v>2368</v>
+        <v>2378</v>
       </c>
       <c r="C103" t="s">
-        <v>2369</v>
+        <v>2379</v>
       </c>
       <c r="D103" t="s">
         <v>22</v>
@@ -26201,10 +26306,10 @@
     <row r="104">
       <c r="A104"/>
       <c r="B104" t="s">
-        <v>2370</v>
+        <v>2380</v>
       </c>
       <c r="C104" t="s">
-        <v>2371</v>
+        <v>2381</v>
       </c>
       <c r="D104" t="s">
         <v>22</v>
@@ -26250,10 +26355,10 @@
         <v>2193</v>
       </c>
       <c r="B108" t="s">
-        <v>2264</v>
+        <v>2274</v>
       </c>
       <c r="C108" t="s">
-        <v>2265</v>
+        <v>2275</v>
       </c>
       <c r="D108" t="s">
         <v>22</v>
@@ -26280,10 +26385,10 @@
     <row r="110">
       <c r="A110"/>
       <c r="B110" t="s">
-        <v>2266</v>
+        <v>2276</v>
       </c>
       <c r="C110" t="s">
-        <v>2267</v>
+        <v>2277</v>
       </c>
       <c r="D110" t="s">
         <v>22</v>
@@ -26295,10 +26400,10 @@
     <row r="111">
       <c r="A111"/>
       <c r="B111" t="s">
-        <v>2268</v>
+        <v>2278</v>
       </c>
       <c r="C111" t="s">
-        <v>2269</v>
+        <v>2279</v>
       </c>
       <c r="D111" t="s">
         <v>22</v>
@@ -26310,10 +26415,10 @@
     <row r="112">
       <c r="A112"/>
       <c r="B112" t="s">
-        <v>2270</v>
+        <v>2280</v>
       </c>
       <c r="C112" t="s">
-        <v>2271</v>
+        <v>2281</v>
       </c>
       <c r="D112" t="s">
         <v>22</v>
@@ -26389,7 +26494,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2292</v>
+        <v>2302</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>2187</v>
@@ -26411,14 +26516,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2308</v>
+        <v>2318</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>55</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2309</v>
+        <v>2319</v>
       </c>
       <c r="E3" s="17" t="s">
         <v>22</v>
@@ -26433,14 +26538,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2372</v>
+        <v>2382</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>2373</v>
+        <v>2383</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2374</v>
+        <v>2384</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>22</v>
@@ -26455,14 +26560,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2375</v>
+        <v>2385</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>2373</v>
+        <v>2383</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2376</v>
+        <v>2386</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>22</v>
@@ -26477,14 +26582,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2377</v>
+        <v>2387</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>2373</v>
+        <v>2383</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2378</v>
+        <v>2388</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>22</v>
@@ -26499,14 +26604,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2379</v>
+        <v>2389</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2380</v>
+        <v>2390</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>22</v>
@@ -26521,14 +26626,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2381</v>
+        <v>2391</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2382</v>
+        <v>2392</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>22</v>
@@ -26543,14 +26648,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2383</v>
+        <v>2393</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2384</v>
+        <v>2394</v>
       </c>
       <c r="E9" s="17" t="s">
         <v>22</v>
@@ -26565,14 +26670,14 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2385</v>
+        <v>2395</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>2386</v>
+        <v>2396</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>22</v>
@@ -26587,14 +26692,14 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2387</v>
+        <v>2397</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>2388</v>
+        <v>2398</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>22</v>
@@ -26609,14 +26714,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2389</v>
+        <v>2399</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2390</v>
+        <v>2400</v>
       </c>
       <c r="E12" s="17" t="s">
         <v>22</v>
@@ -26631,14 +26736,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2391</v>
+        <v>2401</v>
       </c>
       <c r="B13" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2392</v>
+        <v>2402</v>
       </c>
       <c r="E13" s="17" t="s">
         <v>22</v>
@@ -26653,14 +26758,14 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2393</v>
+        <v>2403</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2394</v>
+        <v>2404</v>
       </c>
       <c r="E14" s="17" t="s">
         <v>22</v>
@@ -26675,14 +26780,14 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2395</v>
+        <v>2405</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2396</v>
+        <v>2406</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>22</v>
@@ -26697,14 +26802,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2397</v>
+        <v>2407</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2398</v>
+        <v>2408</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>22</v>
@@ -26719,14 +26824,14 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2399</v>
+        <v>2409</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2400</v>
+        <v>2410</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>22</v>
@@ -26741,14 +26846,14 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2401</v>
+        <v>2411</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>2402</v>
+        <v>2412</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>22</v>
@@ -26763,14 +26868,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2403</v>
+        <v>2413</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2404</v>
+        <v>2414</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>22</v>
@@ -26785,14 +26890,14 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2405</v>
+        <v>2415</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>2406</v>
+        <v>2416</v>
       </c>
       <c r="E20" s="17" t="s">
         <v>22</v>
@@ -26807,14 +26912,14 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>2407</v>
+        <v>2417</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>2408</v>
+        <v>2418</v>
       </c>
       <c r="E21" s="17" t="s">
         <v>22</v>
@@ -26829,14 +26934,14 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>2409</v>
+        <v>2419</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="s">
-        <v>2410</v>
+        <v>2420</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>22</v>
@@ -26851,14 +26956,14 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>2411</v>
+        <v>2421</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>12</v>
       </c>
       <c r="C23"/>
       <c r="D23" t="s">
-        <v>2412</v>
+        <v>2422</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>22</v>
@@ -26890,13 +26995,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>2373</v>
+        <v>2383</v>
       </c>
       <c r="B26" t="s">
-        <v>2268</v>
+        <v>2278</v>
       </c>
       <c r="C26" t="s">
-        <v>2269</v>
+        <v>2279</v>
       </c>
       <c r="D26" t="s">
         <v>22</v>
@@ -26908,10 +27013,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>2266</v>
+        <v>2276</v>
       </c>
       <c r="C27" t="s">
-        <v>2267</v>
+        <v>2277</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -26923,10 +27028,10 @@
     <row r="28">
       <c r="A28"/>
       <c r="B28" t="s">
-        <v>2264</v>
+        <v>2274</v>
       </c>
       <c r="C28" t="s">
-        <v>2265</v>
+        <v>2275</v>
       </c>
       <c r="D28" t="s">
         <v>22</v>
@@ -26999,14 +27104,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2413</v>
+        <v>2423</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>2414</v>
+        <v>2424</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2415</v>
+        <v>2425</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>22</v>
@@ -27045,14 +27150,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2416</v>
+        <v>2426</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>2417</v>
+        <v>2427</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2418</v>
+        <v>2428</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>22</v>
@@ -27067,7 +27172,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2419</v>
+        <v>2429</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>1690</v>
@@ -27089,17 +27194,17 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2420</v>
+        <v>2430</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>2421</v>
+        <v>2431</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2422</v>
+        <v>2432</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>2423</v>
+        <v>2433</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -27113,14 +27218,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2424</v>
+        <v>2434</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>2425</v>
+        <v>2435</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2426</v>
+        <v>2436</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>22</v>
@@ -27135,14 +27240,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2427</v>
+        <v>2437</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>55</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2428</v>
+        <v>2438</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>22</v>
@@ -27159,14 +27264,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2429</v>
+        <v>2439</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>55</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2430</v>
+        <v>2440</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>22</v>
@@ -27181,14 +27286,14 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2431</v>
+        <v>2441</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>2432</v>
+        <v>2442</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>2433</v>
+        <v>2443</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>22</v>
@@ -27203,14 +27308,14 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2434</v>
+        <v>2444</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>55</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>2435</v>
+        <v>2445</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>22</v>
@@ -27225,14 +27330,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2436</v>
+        <v>2446</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>55</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2437</v>
+        <v>2447</v>
       </c>
       <c r="E12" s="18" t="s">
         <v>22</v>
@@ -27247,14 +27352,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2438</v>
+        <v>2448</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>626</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2439</v>
+        <v>2449</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>22</v>
@@ -27269,14 +27374,14 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2440</v>
+        <v>2450</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2441</v>
+        <v>2451</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>22</v>
@@ -27291,14 +27396,14 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2442</v>
+        <v>2452</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>626</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2443</v>
+        <v>2453</v>
       </c>
       <c r="E15" s="18" t="s">
         <v>22</v>
@@ -27315,14 +27420,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2444</v>
+        <v>2454</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2445</v>
+        <v>2455</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>22</v>
@@ -27337,7 +27442,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2446</v>
+        <v>2456</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>42</v>
@@ -27359,7 +27464,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2447</v>
+        <v>2457</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>42</v>
@@ -27381,7 +27486,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2448</v>
+        <v>2458</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>42</v>
@@ -27420,13 +27525,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>2414</v>
+        <v>2424</v>
       </c>
       <c r="B22" t="s">
-        <v>2449</v>
+        <v>2459</v>
       </c>
       <c r="C22" t="s">
-        <v>2450</v>
+        <v>2460</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -27438,10 +27543,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>2451</v>
+        <v>2461</v>
       </c>
       <c r="C23" t="s">
-        <v>2452</v>
+        <v>2462</v>
       </c>
       <c r="D23" t="s">
         <v>22</v>
@@ -27453,10 +27558,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>2453</v>
+        <v>2463</v>
       </c>
       <c r="C24" t="s">
-        <v>2454</v>
+        <v>2464</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -27468,10 +27573,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>2455</v>
+        <v>2465</v>
       </c>
       <c r="C25" t="s">
-        <v>2456</v>
+        <v>2466</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -27499,13 +27604,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2421</v>
+        <v>2431</v>
       </c>
       <c r="B28" t="s">
-        <v>2457</v>
+        <v>2467</v>
       </c>
       <c r="C28" t="s">
-        <v>2458</v>
+        <v>2468</v>
       </c>
       <c r="D28" t="s">
         <v>22</v>
@@ -27517,10 +27622,10 @@
     <row r="29">
       <c r="A29"/>
       <c r="B29" t="s">
-        <v>2459</v>
+        <v>2469</v>
       </c>
       <c r="C29" t="s">
-        <v>2460</v>
+        <v>2470</v>
       </c>
       <c r="D29" t="s">
         <v>22</v>
@@ -27532,10 +27637,10 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>2461</v>
+        <v>2471</v>
       </c>
       <c r="C30" t="s">
-        <v>2462</v>
+        <v>2472</v>
       </c>
       <c r="D30" t="s">
         <v>22</v>
@@ -27547,10 +27652,10 @@
     <row r="31">
       <c r="A31"/>
       <c r="B31" t="s">
-        <v>2463</v>
+        <v>2473</v>
       </c>
       <c r="C31" t="s">
-        <v>2464</v>
+        <v>2474</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -27562,10 +27667,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>2465</v>
+        <v>2475</v>
       </c>
       <c r="C32" t="s">
-        <v>2466</v>
+        <v>2476</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -27580,7 +27685,7 @@
         <v>917</v>
       </c>
       <c r="C33" t="s">
-        <v>2467</v>
+        <v>2477</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -27592,10 +27697,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>2468</v>
+        <v>2478</v>
       </c>
       <c r="C34" t="s">
-        <v>2469</v>
+        <v>2479</v>
       </c>
       <c r="D34" t="s">
         <v>22</v>
@@ -27607,10 +27712,10 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>2470</v>
+        <v>2480</v>
       </c>
       <c r="C35" t="s">
-        <v>2471</v>
+        <v>2481</v>
       </c>
       <c r="D35" t="s">
         <v>22</v>
@@ -27622,10 +27727,10 @@
     <row r="36">
       <c r="A36"/>
       <c r="B36" t="s">
-        <v>2472</v>
+        <v>2482</v>
       </c>
       <c r="C36" t="s">
-        <v>2473</v>
+        <v>2483</v>
       </c>
       <c r="D36" t="s">
         <v>22</v>
@@ -27637,10 +27742,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>2474</v>
+        <v>2484</v>
       </c>
       <c r="C37" t="s">
-        <v>2475</v>
+        <v>2485</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -27652,10 +27757,10 @@
     <row r="38">
       <c r="A38"/>
       <c r="B38" t="s">
-        <v>2476</v>
+        <v>2486</v>
       </c>
       <c r="C38" t="s">
-        <v>2477</v>
+        <v>2487</v>
       </c>
       <c r="D38" t="s">
         <v>22</v>
@@ -27667,10 +27772,10 @@
     <row r="39">
       <c r="A39"/>
       <c r="B39" t="s">
-        <v>2478</v>
+        <v>2488</v>
       </c>
       <c r="C39" t="s">
-        <v>2479</v>
+        <v>2489</v>
       </c>
       <c r="D39" t="s">
         <v>22</v>
@@ -27682,10 +27787,10 @@
     <row r="40">
       <c r="A40"/>
       <c r="B40" t="s">
-        <v>2480</v>
+        <v>2490</v>
       </c>
       <c r="C40" t="s">
-        <v>2481</v>
+        <v>2491</v>
       </c>
       <c r="D40" t="s">
         <v>22</v>
@@ -27697,10 +27802,10 @@
     <row r="41">
       <c r="A41"/>
       <c r="B41" t="s">
-        <v>2482</v>
+        <v>2492</v>
       </c>
       <c r="C41" t="s">
-        <v>2483</v>
+        <v>2493</v>
       </c>
       <c r="D41" t="s">
         <v>22</v>
@@ -27712,10 +27817,10 @@
     <row r="42">
       <c r="A42"/>
       <c r="B42" t="s">
-        <v>2484</v>
+        <v>2494</v>
       </c>
       <c r="C42" t="s">
-        <v>2485</v>
+        <v>2495</v>
       </c>
       <c r="D42" t="s">
         <v>22</v>
@@ -27727,10 +27832,10 @@
     <row r="43">
       <c r="A43"/>
       <c r="B43" t="s">
-        <v>2486</v>
+        <v>2496</v>
       </c>
       <c r="C43" t="s">
-        <v>2487</v>
+        <v>2497</v>
       </c>
       <c r="D43" t="s">
         <v>22</v>
@@ -27742,10 +27847,10 @@
     <row r="44">
       <c r="A44"/>
       <c r="B44" t="s">
-        <v>2488</v>
+        <v>2498</v>
       </c>
       <c r="C44" t="s">
-        <v>2489</v>
+        <v>2499</v>
       </c>
       <c r="D44" t="s">
         <v>22</v>
@@ -27757,10 +27862,10 @@
     <row r="45">
       <c r="A45"/>
       <c r="B45" t="s">
-        <v>2490</v>
+        <v>2500</v>
       </c>
       <c r="C45" t="s">
-        <v>2491</v>
+        <v>2501</v>
       </c>
       <c r="D45" t="s">
         <v>22</v>
@@ -27772,10 +27877,10 @@
     <row r="46">
       <c r="A46"/>
       <c r="B46" t="s">
-        <v>2492</v>
+        <v>2502</v>
       </c>
       <c r="C46" t="s">
-        <v>2493</v>
+        <v>2503</v>
       </c>
       <c r="D46" t="s">
         <v>22</v>
@@ -27790,7 +27895,7 @@
         <v>179</v>
       </c>
       <c r="C47" t="s">
-        <v>2494</v>
+        <v>2504</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
@@ -27802,10 +27907,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>2495</v>
+        <v>2505</v>
       </c>
       <c r="C48" t="s">
-        <v>2496</v>
+        <v>2506</v>
       </c>
       <c r="D48" t="s">
         <v>22</v>
@@ -27817,10 +27922,10 @@
     <row r="49">
       <c r="A49"/>
       <c r="B49" t="s">
-        <v>2497</v>
+        <v>2507</v>
       </c>
       <c r="C49" t="s">
-        <v>2498</v>
+        <v>2508</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -27832,10 +27937,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>2499</v>
+        <v>2509</v>
       </c>
       <c r="C50" t="s">
-        <v>2500</v>
+        <v>2510</v>
       </c>
       <c r="D50" t="s">
         <v>22</v>
@@ -27863,13 +27968,13 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>2425</v>
+        <v>2435</v>
       </c>
       <c r="B53" t="s">
-        <v>2501</v>
+        <v>2511</v>
       </c>
       <c r="C53" t="s">
-        <v>2502</v>
+        <v>2512</v>
       </c>
       <c r="D53" t="s">
         <v>22</v>
@@ -27881,10 +27986,10 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>2503</v>
+        <v>2513</v>
       </c>
       <c r="C54" t="s">
-        <v>2504</v>
+        <v>2514</v>
       </c>
       <c r="D54" t="s">
         <v>22</v>
@@ -27896,10 +28001,10 @@
     <row r="55">
       <c r="A55"/>
       <c r="B55" t="s">
-        <v>2505</v>
+        <v>2515</v>
       </c>
       <c r="C55" t="s">
-        <v>2506</v>
+        <v>2516</v>
       </c>
       <c r="D55" t="s">
         <v>22</v>
@@ -27927,13 +28032,13 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>2432</v>
+        <v>2442</v>
       </c>
       <c r="B58" t="s">
         <v>936</v>
       </c>
       <c r="C58" t="s">
-        <v>2507</v>
+        <v>2517</v>
       </c>
       <c r="D58" t="s">
         <v>22</v>
@@ -27948,7 +28053,7 @@
         <v>939</v>
       </c>
       <c r="C59" t="s">
-        <v>2508</v>
+        <v>2518</v>
       </c>
       <c r="D59" t="s">
         <v>22</v>
@@ -27960,10 +28065,10 @@
     <row r="60">
       <c r="A60"/>
       <c r="B60" t="s">
-        <v>2509</v>
+        <v>2519</v>
       </c>
       <c r="C60" t="s">
-        <v>2510</v>
+        <v>2520</v>
       </c>
       <c r="D60" t="s">
         <v>22</v>
@@ -27975,10 +28080,10 @@
     <row r="61">
       <c r="A61"/>
       <c r="B61" t="s">
-        <v>2511</v>
+        <v>2521</v>
       </c>
       <c r="C61" t="s">
-        <v>2512</v>
+        <v>2522</v>
       </c>
       <c r="D61" t="s">
         <v>22</v>
@@ -28054,10 +28159,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2513</v>
+        <v>2523</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>2417</v>
+        <v>2427</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
@@ -28076,17 +28181,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2514</v>
+        <v>2524</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>2515</v>
+        <v>2525</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2516</v>
+        <v>2526</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>2517</v>
+        <v>2527</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -28100,14 +28205,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2518</v>
+        <v>2528</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>2519</v>
+        <v>2529</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2520</v>
+        <v>2530</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>22</v>
@@ -28122,10 +28227,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2521</v>
+        <v>2531</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>2522</v>
+        <v>2532</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
@@ -28144,14 +28249,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2523</v>
+        <v>2533</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>55</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2524</v>
+        <v>2534</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>22</v>
@@ -28166,14 +28271,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2525</v>
+        <v>2535</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>55</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2526</v>
+        <v>2536</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>22</v>
@@ -28188,14 +28293,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2527</v>
+        <v>2537</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>2528</v>
+        <v>2538</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2529</v>
+        <v>2539</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>22</v>
@@ -28254,14 +28359,14 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2530</v>
+        <v>2540</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>2531</v>
+        <v>2541</v>
       </c>
       <c r="E11" s="19" t="s">
         <v>22</v>
@@ -28276,7 +28381,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2532</v>
+        <v>2542</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>12</v>
@@ -28286,7 +28391,7 @@
         <v>4</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>2533</v>
+        <v>2543</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -28300,14 +28405,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2534</v>
+        <v>2544</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>651</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2535</v>
+        <v>2545</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>22</v>
@@ -28329,10 +28434,10 @@
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2536</v>
+        <v>2546</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>2537</v>
+        <v>2547</v>
       </c>
       <c r="F14"/>
       <c r="H14" s="19" t="s">
@@ -28351,10 +28456,10 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2538</v>
+        <v>2548</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>2539</v>
+        <v>2549</v>
       </c>
       <c r="F15"/>
       <c r="H15" s="19" t="s">
@@ -28414,14 +28519,14 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2540</v>
+        <v>2550</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>55</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>2541</v>
+        <v>2551</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>22</v>
@@ -28436,14 +28541,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2542</v>
+        <v>2552</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2543</v>
+        <v>2553</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>22</v>
@@ -28458,7 +28563,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2544</v>
+        <v>2554</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>115</v>
@@ -28490,7 +28595,7 @@
         <v>1625</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>2545</v>
+        <v>2555</v>
       </c>
       <c r="F21"/>
       <c r="H21" s="19" t="s">
@@ -28570,14 +28675,14 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>2546</v>
+        <v>2556</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>55</v>
       </c>
       <c r="C25"/>
       <c r="D25" t="s">
-        <v>2547</v>
+        <v>2557</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>22</v>
@@ -28614,14 +28719,14 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>2548</v>
+        <v>2558</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>2549</v>
+        <v>2559</v>
       </c>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>2550</v>
+        <v>2560</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>22</v>
@@ -28636,14 +28741,14 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2551</v>
+        <v>2561</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>2552</v>
+        <v>2562</v>
       </c>
       <c r="C28"/>
       <c r="D28" t="s">
-        <v>2553</v>
+        <v>2563</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>22</v>
@@ -28658,14 +28763,14 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>2554</v>
+        <v>2564</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>2555</v>
+        <v>2565</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>22</v>
@@ -28680,17 +28785,17 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>2556</v>
+        <v>2566</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>2557</v>
+        <v>2567</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>2558</v>
+        <v>2568</v>
       </c>
       <c r="F30"/>
       <c r="H30" s="19" t="s">
@@ -28702,17 +28807,17 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2559</v>
+        <v>2569</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>2560</v>
+        <v>2570</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>2561</v>
+        <v>2571</v>
       </c>
       <c r="F31"/>
       <c r="H31" s="19" t="s">
@@ -28724,17 +28829,17 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>2562</v>
+        <v>2572</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C32"/>
       <c r="D32" t="s">
-        <v>2563</v>
+        <v>2573</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>2564</v>
+        <v>2574</v>
       </c>
       <c r="F32"/>
       <c r="H32" s="19" t="s">
@@ -28746,17 +28851,17 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>2565</v>
+        <v>2575</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C33"/>
       <c r="D33" t="s">
-        <v>2566</v>
+        <v>2576</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>2567</v>
+        <v>2577</v>
       </c>
       <c r="F33"/>
       <c r="H33" s="19" t="s">
@@ -28768,17 +28873,17 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>2568</v>
+        <v>2578</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C34"/>
       <c r="D34" t="s">
-        <v>2569</v>
+        <v>2579</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>2570</v>
+        <v>2580</v>
       </c>
       <c r="F34"/>
       <c r="H34" s="19" t="s">
@@ -28790,17 +28895,17 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>2571</v>
+        <v>2581</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>2572</v>
+        <v>2582</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>2573</v>
+        <v>2583</v>
       </c>
       <c r="F35"/>
       <c r="H35" s="19" t="s">
@@ -28812,17 +28917,17 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2574</v>
+        <v>2584</v>
       </c>
       <c r="B36" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C36"/>
       <c r="D36" t="s">
-        <v>2575</v>
+        <v>2585</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>2576</v>
+        <v>2586</v>
       </c>
       <c r="F36"/>
       <c r="H36" s="19" t="s">
@@ -28878,7 +28983,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>2577</v>
+        <v>2587</v>
       </c>
       <c r="B39" s="19" t="s">
         <v>626</v>
@@ -28887,7 +28992,7 @@
         <v>66</v>
       </c>
       <c r="D39" t="s">
-        <v>2578</v>
+        <v>2588</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>22</v>
@@ -28902,14 +29007,14 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>2579</v>
+        <v>2589</v>
       </c>
       <c r="B40" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C40"/>
       <c r="D40" t="s">
-        <v>2580</v>
+        <v>2590</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>22</v>
@@ -28990,14 +29095,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>2581</v>
+        <v>2591</v>
       </c>
       <c r="B44" s="19" t="s">
         <v>651</v>
       </c>
       <c r="C44"/>
       <c r="D44" t="s">
-        <v>2582</v>
+        <v>2592</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>22</v>
@@ -29012,14 +29117,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>2583</v>
+        <v>2593</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>2584</v>
+        <v>2594</v>
       </c>
       <c r="C45"/>
       <c r="D45" t="s">
-        <v>2585</v>
+        <v>2595</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>22</v>
@@ -29034,17 +29139,17 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>2586</v>
+        <v>2596</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>2587</v>
+        <v>2597</v>
       </c>
       <c r="C46"/>
       <c r="D46" t="s">
-        <v>2588</v>
+        <v>2598</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>2589</v>
+        <v>2599</v>
       </c>
       <c r="F46"/>
       <c r="H46" s="19" t="s">
@@ -29058,14 +29163,14 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>2590</v>
+        <v>2600</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>2591</v>
+        <v>2601</v>
       </c>
       <c r="C47"/>
       <c r="D47" t="s">
-        <v>2592</v>
+        <v>2602</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>22</v>
@@ -29082,14 +29187,14 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>2593</v>
+        <v>2603</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>2594</v>
+        <v>2604</v>
       </c>
       <c r="C48"/>
       <c r="D48" t="s">
-        <v>2595</v>
+        <v>2605</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>22</v>
@@ -29106,14 +29211,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>2596</v>
+        <v>2606</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>2597</v>
+        <v>2607</v>
       </c>
       <c r="C49"/>
       <c r="D49" t="s">
-        <v>2598</v>
+        <v>2608</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>22</v>
@@ -29174,14 +29279,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>2599</v>
+        <v>2609</v>
       </c>
       <c r="B52" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>2600</v>
+        <v>2610</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>22</v>
@@ -29215,13 +29320,13 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>2515</v>
+        <v>2525</v>
       </c>
       <c r="B55" t="s">
-        <v>2601</v>
+        <v>2611</v>
       </c>
       <c r="C55" t="s">
-        <v>2602</v>
+        <v>2612</v>
       </c>
       <c r="D55" t="s">
         <v>22</v>
@@ -29233,10 +29338,10 @@
     <row r="56">
       <c r="A56"/>
       <c r="B56" t="s">
-        <v>2453</v>
+        <v>2463</v>
       </c>
       <c r="C56" t="s">
-        <v>2454</v>
+        <v>2464</v>
       </c>
       <c r="D56" t="s">
         <v>22</v>
@@ -29263,10 +29368,10 @@
     <row r="58">
       <c r="A58"/>
       <c r="B58" t="s">
-        <v>2603</v>
+        <v>2613</v>
       </c>
       <c r="C58" t="s">
-        <v>2604</v>
+        <v>2614</v>
       </c>
       <c r="D58" t="s">
         <v>22</v>
@@ -29309,13 +29414,13 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>2519</v>
+        <v>2529</v>
       </c>
       <c r="B62" t="s">
-        <v>2505</v>
+        <v>2515</v>
       </c>
       <c r="C62" t="s">
-        <v>2605</v>
+        <v>2615</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -29327,10 +29432,10 @@
     <row r="63">
       <c r="A63"/>
       <c r="B63" t="s">
-        <v>2606</v>
+        <v>2616</v>
       </c>
       <c r="C63" t="s">
-        <v>2607</v>
+        <v>2617</v>
       </c>
       <c r="D63" t="s">
         <v>22</v>
@@ -29342,10 +29447,10 @@
     <row r="64">
       <c r="A64"/>
       <c r="B64" t="s">
-        <v>2501</v>
+        <v>2511</v>
       </c>
       <c r="C64" t="s">
-        <v>2608</v>
+        <v>2618</v>
       </c>
       <c r="D64" t="s">
         <v>22</v>
@@ -29388,7 +29493,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>2522</v>
+        <v>2532</v>
       </c>
       <c r="B68" t="s">
         <v>936</v>
@@ -29406,10 +29511,10 @@
     <row r="69">
       <c r="A69"/>
       <c r="B69" t="s">
-        <v>2609</v>
+        <v>2619</v>
       </c>
       <c r="C69" t="s">
-        <v>2610</v>
+        <v>2620</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
@@ -29467,7 +29572,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>2528</v>
+        <v>2538</v>
       </c>
       <c r="B74" t="s">
         <v>936</v>
@@ -29485,7 +29590,7 @@
     <row r="75">
       <c r="A75"/>
       <c r="B75" t="s">
-        <v>2609</v>
+        <v>2619</v>
       </c>
       <c r="C75" t="s">
         <v>1046</v>
@@ -29515,10 +29620,10 @@
     <row r="77">
       <c r="A77"/>
       <c r="B77" t="s">
-        <v>2611</v>
+        <v>2621</v>
       </c>
       <c r="C77" t="s">
-        <v>2612</v>
+        <v>2622</v>
       </c>
       <c r="D77" t="s">
         <v>22</v>
@@ -29967,13 +30072,13 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>2549</v>
+        <v>2559</v>
       </c>
       <c r="B111" t="s">
-        <v>2613</v>
+        <v>2623</v>
       </c>
       <c r="C111" t="s">
-        <v>2614</v>
+        <v>2624</v>
       </c>
       <c r="D111" t="s">
         <v>22</v>
@@ -29985,10 +30090,10 @@
     <row r="112">
       <c r="A112"/>
       <c r="B112" t="s">
-        <v>2615</v>
+        <v>2625</v>
       </c>
       <c r="C112" t="s">
-        <v>2616</v>
+        <v>2626</v>
       </c>
       <c r="D112" t="s">
         <v>22</v>
@@ -30000,10 +30105,10 @@
     <row r="113">
       <c r="A113"/>
       <c r="B113" t="s">
-        <v>2617</v>
+        <v>2627</v>
       </c>
       <c r="C113" t="s">
-        <v>2618</v>
+        <v>2628</v>
       </c>
       <c r="D113" t="s">
         <v>22</v>
@@ -30015,10 +30120,10 @@
     <row r="114">
       <c r="A114"/>
       <c r="B114" t="s">
-        <v>2619</v>
+        <v>2629</v>
       </c>
       <c r="C114" t="s">
-        <v>2620</v>
+        <v>2630</v>
       </c>
       <c r="D114" t="s">
         <v>22</v>
@@ -30030,10 +30135,10 @@
     <row r="115">
       <c r="A115"/>
       <c r="B115" t="s">
-        <v>2621</v>
+        <v>2631</v>
       </c>
       <c r="C115" t="s">
-        <v>2622</v>
+        <v>2632</v>
       </c>
       <c r="D115" t="s">
         <v>22</v>
@@ -30061,13 +30166,13 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>2552</v>
+        <v>2562</v>
       </c>
       <c r="B118" t="s">
-        <v>2623</v>
+        <v>2633</v>
       </c>
       <c r="C118" t="s">
-        <v>2624</v>
+        <v>2634</v>
       </c>
       <c r="D118" t="s">
         <v>22</v>
@@ -30079,10 +30184,10 @@
     <row r="119">
       <c r="A119"/>
       <c r="B119" t="s">
-        <v>2625</v>
+        <v>2635</v>
       </c>
       <c r="C119" t="s">
-        <v>2626</v>
+        <v>2636</v>
       </c>
       <c r="D119" t="s">
         <v>22</v>
@@ -30094,10 +30199,10 @@
     <row r="120">
       <c r="A120"/>
       <c r="B120" t="s">
-        <v>2627</v>
+        <v>2637</v>
       </c>
       <c r="C120" t="s">
-        <v>2628</v>
+        <v>2638</v>
       </c>
       <c r="D120" t="s">
         <v>22</v>
@@ -30109,10 +30214,10 @@
     <row r="121">
       <c r="A121"/>
       <c r="B121" t="s">
-        <v>2629</v>
+        <v>2639</v>
       </c>
       <c r="C121" t="s">
-        <v>2630</v>
+        <v>2640</v>
       </c>
       <c r="D121" t="s">
         <v>22</v>
@@ -30124,10 +30229,10 @@
     <row r="122">
       <c r="A122"/>
       <c r="B122" t="s">
-        <v>2631</v>
+        <v>2641</v>
       </c>
       <c r="C122" t="s">
-        <v>2632</v>
+        <v>2642</v>
       </c>
       <c r="D122" t="s">
         <v>22</v>
@@ -31029,13 +31134,13 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>2584</v>
+        <v>2594</v>
       </c>
       <c r="B184" t="s">
-        <v>2633</v>
+        <v>2643</v>
       </c>
       <c r="C184" t="s">
-        <v>2634</v>
+        <v>2644</v>
       </c>
       <c r="D184" t="s">
         <v>22</v>
@@ -31047,10 +31152,10 @@
     <row r="185">
       <c r="A185"/>
       <c r="B185" t="s">
-        <v>2260</v>
+        <v>2270</v>
       </c>
       <c r="C185" t="s">
-        <v>2635</v>
+        <v>2645</v>
       </c>
       <c r="D185" t="s">
         <v>22</v>
@@ -31062,10 +31167,10 @@
     <row r="186">
       <c r="A186"/>
       <c r="B186" t="s">
-        <v>2262</v>
+        <v>2272</v>
       </c>
       <c r="C186" t="s">
-        <v>2636</v>
+        <v>2646</v>
       </c>
       <c r="D186" t="s">
         <v>22</v>
@@ -31077,10 +31182,10 @@
     <row r="187">
       <c r="A187"/>
       <c r="B187" t="s">
-        <v>2637</v>
+        <v>2647</v>
       </c>
       <c r="C187" t="s">
-        <v>2638</v>
+        <v>2648</v>
       </c>
       <c r="D187" t="s">
         <v>22</v>
@@ -31092,10 +31197,10 @@
     <row r="188">
       <c r="A188"/>
       <c r="B188" t="s">
-        <v>2639</v>
+        <v>2649</v>
       </c>
       <c r="C188" t="s">
-        <v>2640</v>
+        <v>2650</v>
       </c>
       <c r="D188" t="s">
         <v>22</v>
@@ -31138,7 +31243,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>2587</v>
+        <v>2597</v>
       </c>
       <c r="B192" t="s">
         <v>893</v>
@@ -31217,13 +31322,13 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>2591</v>
+        <v>2601</v>
       </c>
       <c r="B198" t="s">
-        <v>2641</v>
+        <v>2651</v>
       </c>
       <c r="C198" t="s">
-        <v>2642</v>
+        <v>2652</v>
       </c>
       <c r="D198" t="s">
         <v>22</v>
@@ -31235,10 +31340,10 @@
     <row r="199">
       <c r="A199"/>
       <c r="B199" t="s">
-        <v>2643</v>
+        <v>2653</v>
       </c>
       <c r="C199" t="s">
-        <v>2644</v>
+        <v>2654</v>
       </c>
       <c r="D199" t="s">
         <v>22</v>
@@ -31250,10 +31355,10 @@
     <row r="200">
       <c r="A200"/>
       <c r="B200" t="s">
-        <v>2645</v>
+        <v>2655</v>
       </c>
       <c r="C200" t="s">
-        <v>2646</v>
+        <v>2656</v>
       </c>
       <c r="D200" t="s">
         <v>22</v>
@@ -31265,10 +31370,10 @@
     <row r="201">
       <c r="A201"/>
       <c r="B201" t="s">
-        <v>2647</v>
+        <v>2657</v>
       </c>
       <c r="C201" t="s">
-        <v>2648</v>
+        <v>2658</v>
       </c>
       <c r="D201" t="s">
         <v>22</v>
@@ -31280,10 +31385,10 @@
     <row r="202">
       <c r="A202"/>
       <c r="B202" t="s">
-        <v>2649</v>
+        <v>2659</v>
       </c>
       <c r="C202" t="s">
-        <v>2650</v>
+        <v>2660</v>
       </c>
       <c r="D202" t="s">
         <v>22</v>
@@ -31295,10 +31400,10 @@
     <row r="203">
       <c r="A203"/>
       <c r="B203" t="s">
-        <v>2651</v>
+        <v>2661</v>
       </c>
       <c r="C203" t="s">
-        <v>2652</v>
+        <v>2662</v>
       </c>
       <c r="D203" t="s">
         <v>22</v>
@@ -31341,13 +31446,13 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>2594</v>
+        <v>2604</v>
       </c>
       <c r="B207" t="s">
-        <v>2653</v>
+        <v>2663</v>
       </c>
       <c r="C207" t="s">
-        <v>2654</v>
+        <v>2664</v>
       </c>
       <c r="D207" t="s">
         <v>22</v>
@@ -31359,10 +31464,10 @@
     <row r="208">
       <c r="A208"/>
       <c r="B208" t="s">
-        <v>2655</v>
+        <v>2665</v>
       </c>
       <c r="C208" t="s">
-        <v>2656</v>
+        <v>2666</v>
       </c>
       <c r="D208" t="s">
         <v>22</v>
@@ -31374,10 +31479,10 @@
     <row r="209">
       <c r="A209"/>
       <c r="B209" t="s">
-        <v>2657</v>
+        <v>2667</v>
       </c>
       <c r="C209" t="s">
-        <v>2658</v>
+        <v>2668</v>
       </c>
       <c r="D209" t="s">
         <v>22</v>
@@ -31389,10 +31494,10 @@
     <row r="210">
       <c r="A210"/>
       <c r="B210" t="s">
-        <v>2659</v>
+        <v>2669</v>
       </c>
       <c r="C210" t="s">
-        <v>2660</v>
+        <v>2670</v>
       </c>
       <c r="D210" t="s">
         <v>22</v>
@@ -31404,10 +31509,10 @@
     <row r="211">
       <c r="A211"/>
       <c r="B211" t="s">
-        <v>2661</v>
+        <v>2671</v>
       </c>
       <c r="C211" t="s">
-        <v>2662</v>
+        <v>2672</v>
       </c>
       <c r="D211" t="s">
         <v>22</v>
@@ -31450,13 +31555,13 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>2597</v>
+        <v>2607</v>
       </c>
       <c r="B215" t="s">
-        <v>2663</v>
+        <v>2673</v>
       </c>
       <c r="C215" t="s">
-        <v>2664</v>
+        <v>2674</v>
       </c>
       <c r="D215" t="s">
         <v>22</v>
@@ -31468,10 +31573,10 @@
     <row r="216">
       <c r="A216"/>
       <c r="B216" t="s">
-        <v>2665</v>
+        <v>2675</v>
       </c>
       <c r="C216" t="s">
-        <v>2666</v>
+        <v>2676</v>
       </c>
       <c r="D216" t="s">
         <v>22</v>
@@ -31483,10 +31588,10 @@
     <row r="217">
       <c r="A217"/>
       <c r="B217" t="s">
-        <v>2667</v>
+        <v>2677</v>
       </c>
       <c r="C217" t="s">
-        <v>2668</v>
+        <v>2678</v>
       </c>
       <c r="D217" t="s">
         <v>22</v>
@@ -31498,10 +31603,10 @@
     <row r="218">
       <c r="A218"/>
       <c r="B218" t="s">
-        <v>2669</v>
+        <v>2679</v>
       </c>
       <c r="C218" t="s">
-        <v>2670</v>
+        <v>2680</v>
       </c>
       <c r="D218" t="s">
         <v>22</v>
@@ -31513,10 +31618,10 @@
     <row r="219">
       <c r="A219"/>
       <c r="B219" t="s">
-        <v>2671</v>
+        <v>2681</v>
       </c>
       <c r="C219" t="s">
-        <v>2672</v>
+        <v>2682</v>
       </c>
       <c r="D219" t="s">
         <v>22</v>
@@ -33294,14 +33399,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2416</v>
+        <v>2426</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>2417</v>
+        <v>2427</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2454</v>
+        <v>2464</v>
       </c>
       <c r="E3" s="20" t="s">
         <v>22</v>
@@ -33321,11 +33426,11 @@
         <v>617</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>2673</v>
+        <v>2683</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2673</v>
+        <v>2683</v>
       </c>
       <c r="E4" s="20" t="s">
         <v>22</v>
@@ -33342,7 +33447,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2674</v>
+        <v>2684</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>12</v>
@@ -33351,7 +33456,7 @@
         <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>2675</v>
+        <v>2685</v>
       </c>
       <c r="E5" s="20" t="s">
         <v>22</v>
@@ -33476,7 +33581,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2676</v>
+        <v>2686</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>140</v>
@@ -33559,14 +33664,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2677</v>
+        <v>2687</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>2678</v>
+        <v>2688</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2679</v>
+        <v>2689</v>
       </c>
       <c r="E2" s="21" t="s">
         <v>22</v>
@@ -33583,14 +33688,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2416</v>
+        <v>2426</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>2417</v>
+        <v>2427</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2418</v>
+        <v>2428</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>22</v>
@@ -33605,14 +33710,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2680</v>
+        <v>2690</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>2681</v>
+        <v>2691</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2682</v>
+        <v>2692</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>22</v>
@@ -33627,14 +33732,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2424</v>
+        <v>2434</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>2683</v>
+        <v>2693</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2426</v>
+        <v>2436</v>
       </c>
       <c r="E5" s="21" t="s">
         <v>22</v>
@@ -33649,7 +33754,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2684</v>
+        <v>2694</v>
       </c>
       <c r="B6" s="21" t="s">
         <v>55</v>
@@ -33673,14 +33778,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2685</v>
+        <v>2695</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>2686</v>
+        <v>2696</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2687</v>
+        <v>2697</v>
       </c>
       <c r="E7" s="21" t="s">
         <v>22</v>
@@ -33695,7 +33800,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2434</v>
+        <v>2444</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>55</v>
@@ -33717,14 +33822,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2438</v>
+        <v>2448</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>626</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2439</v>
+        <v>2449</v>
       </c>
       <c r="E9" s="21" t="s">
         <v>22</v>
@@ -33739,14 +33844,14 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2688</v>
+        <v>2698</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>12</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>2531</v>
+        <v>2541</v>
       </c>
       <c r="E10" s="21" t="s">
         <v>22</v>
@@ -33783,14 +33888,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2689</v>
+        <v>2699</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>12</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2445</v>
+        <v>2455</v>
       </c>
       <c r="E12" s="21" t="s">
         <v>22</v>
@@ -33805,14 +33910,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2690</v>
+        <v>2700</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>626</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2691</v>
+        <v>2701</v>
       </c>
       <c r="E13" s="21" t="s">
         <v>22</v>
@@ -33844,13 +33949,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2678</v>
+        <v>2688</v>
       </c>
       <c r="B16" t="s">
-        <v>2453</v>
+        <v>2463</v>
       </c>
       <c r="C16" t="s">
-        <v>2454</v>
+        <v>2464</v>
       </c>
       <c r="D16" t="s">
         <v>22</v>
@@ -33878,13 +33983,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2681</v>
+        <v>2691</v>
       </c>
       <c r="B19" t="s">
-        <v>2692</v>
+        <v>2702</v>
       </c>
       <c r="C19" t="s">
-        <v>2693</v>
+        <v>2703</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -33896,10 +34001,10 @@
     <row r="20">
       <c r="A20"/>
       <c r="B20" t="s">
-        <v>2468</v>
+        <v>2478</v>
       </c>
       <c r="C20" t="s">
-        <v>2694</v>
+        <v>2704</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -33911,10 +34016,10 @@
     <row r="21">
       <c r="A21"/>
       <c r="B21" t="s">
-        <v>2695</v>
+        <v>2705</v>
       </c>
       <c r="C21" t="s">
-        <v>2696</v>
+        <v>2706</v>
       </c>
       <c r="D21" t="s">
         <v>22</v>
@@ -33926,10 +34031,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>2472</v>
+        <v>2482</v>
       </c>
       <c r="C22" t="s">
-        <v>2697</v>
+        <v>2707</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -33941,10 +34046,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>2698</v>
+        <v>2708</v>
       </c>
       <c r="C23" t="s">
-        <v>2699</v>
+        <v>2709</v>
       </c>
       <c r="D23" t="s">
         <v>22</v>
@@ -33956,10 +34061,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>2700</v>
+        <v>2710</v>
       </c>
       <c r="C24" t="s">
-        <v>2701</v>
+        <v>2711</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -33971,10 +34076,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>2702</v>
+        <v>2712</v>
       </c>
       <c r="C25" t="s">
-        <v>2703</v>
+        <v>2713</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -33986,10 +34091,10 @@
     <row r="26">
       <c r="A26"/>
       <c r="B26" t="s">
-        <v>2704</v>
+        <v>2714</v>
       </c>
       <c r="C26" t="s">
-        <v>2705</v>
+        <v>2715</v>
       </c>
       <c r="D26" t="s">
         <v>22</v>
@@ -34001,10 +34106,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>2706</v>
+        <v>2716</v>
       </c>
       <c r="C27" t="s">
-        <v>2707</v>
+        <v>2717</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -34047,13 +34152,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2683</v>
+        <v>2693</v>
       </c>
       <c r="B31" t="s">
-        <v>2501</v>
+        <v>2511</v>
       </c>
       <c r="C31" t="s">
-        <v>2502</v>
+        <v>2512</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -34065,10 +34170,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>2503</v>
+        <v>2513</v>
       </c>
       <c r="C32" t="s">
-        <v>2504</v>
+        <v>2514</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -34080,10 +34185,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>2505</v>
+        <v>2515</v>
       </c>
       <c r="C33" t="s">
-        <v>2506</v>
+        <v>2516</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -34111,7 +34216,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2686</v>
+        <v>2696</v>
       </c>
       <c r="B36" t="s">
         <v>936</v>
@@ -34129,10 +34234,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>2708</v>
+        <v>2718</v>
       </c>
       <c r="C37" t="s">
-        <v>2709</v>
+        <v>2719</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -34223,14 +34328,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2710</v>
+        <v>2720</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2711</v>
+        <v>2721</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>22</v>
@@ -34450,7 +34555,7 @@
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2712</v>
+        <v>2722</v>
       </c>
       <c r="E12" s="22" t="s">
         <v>22</v>
@@ -34472,7 +34577,7 @@
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2713</v>
+        <v>2723</v>
       </c>
       <c r="E13" s="22" t="s">
         <v>22</v>
@@ -34487,7 +34592,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2714</v>
+        <v>2724</v>
       </c>
       <c r="B14" s="22" t="s">
         <v>69</v>
@@ -34509,14 +34614,14 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2715</v>
+        <v>2725</v>
       </c>
       <c r="B15" s="22" t="s">
         <v>140</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2716</v>
+        <v>2726</v>
       </c>
       <c r="E15" s="22" t="s">
         <v>22</v>
@@ -34531,14 +34636,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2717</v>
+        <v>2727</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>140</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2718</v>
+        <v>2728</v>
       </c>
       <c r="E16" s="22" t="s">
         <v>22</v>
@@ -35621,14 +35726,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2719</v>
+        <v>2729</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2720</v>
+        <v>2730</v>
       </c>
       <c r="E2" s="23" t="s">
         <v>22</v>
@@ -35665,14 +35770,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>12</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2722</v>
+        <v>2732</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>22</v>
@@ -35687,14 +35792,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2723</v>
+        <v>2733</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>12</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2724</v>
+        <v>2734</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>22</v>
@@ -35709,14 +35814,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2717</v>
+        <v>2727</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>140</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2718</v>
+        <v>2728</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>22</v>
@@ -35792,14 +35897,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2710</v>
+        <v>2720</v>
       </c>
       <c r="B2" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2711</v>
+        <v>2721</v>
       </c>
       <c r="E2" s="24" t="s">
         <v>22</v>
@@ -35814,14 +35919,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2725</v>
+        <v>2735</v>
       </c>
       <c r="B3" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2726</v>
+        <v>2736</v>
       </c>
       <c r="E3" s="24" t="s">
         <v>22</v>
@@ -35836,14 +35941,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2727</v>
+        <v>2737</v>
       </c>
       <c r="B4" s="24" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2728</v>
+        <v>2738</v>
       </c>
       <c r="E4" s="24" t="s">
         <v>22</v>
@@ -35858,14 +35963,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2717</v>
+        <v>2727</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>140</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2718</v>
+        <v>2728</v>
       </c>
       <c r="E5" s="24" t="s">
         <v>22</v>
@@ -35902,10 +36007,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2729</v>
+        <v>2739</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>2730</v>
+        <v>2740</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
@@ -35985,14 +36090,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2710</v>
+        <v>2720</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2711</v>
+        <v>2721</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>22</v>
@@ -36007,14 +36112,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2725</v>
+        <v>2735</v>
       </c>
       <c r="B3" s="25" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2726</v>
+        <v>2736</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>22</v>
@@ -36029,14 +36134,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2727</v>
+        <v>2737</v>
       </c>
       <c r="B4" s="25" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2728</v>
+        <v>2738</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>22</v>
@@ -36073,14 +36178,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2717</v>
+        <v>2727</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>140</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2718</v>
+        <v>2728</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>22</v>
@@ -36178,14 +36283,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2710</v>
+        <v>2720</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2711</v>
+        <v>2721</v>
       </c>
       <c r="E2" s="26" t="s">
         <v>22</v>
@@ -36244,14 +36349,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2717</v>
+        <v>2727</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>140</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2718</v>
+        <v>2728</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>22</v>
@@ -36349,14 +36454,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2731</v>
+        <v>2741</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>140</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2732</v>
+        <v>2742</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>22</v>
@@ -36371,14 +36476,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2733</v>
+        <v>2743</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2734</v>
+        <v>2744</v>
       </c>
       <c r="E3" s="27" t="s">
         <v>22</v>
@@ -36437,14 +36542,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2735</v>
+        <v>2745</v>
       </c>
       <c r="B6" s="27" t="s">
         <v>12</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2566</v>
+        <v>2576</v>
       </c>
       <c r="E6" s="27" t="s">
         <v>22</v>
@@ -36488,7 +36593,7 @@
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2736</v>
+        <v>2746</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>22</v>
@@ -36503,12 +36608,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2737</v>
+        <v>2747</v>
       </c>
       <c r="B9" s="27"/>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2738</v>
+        <v>2748</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>22</v>
@@ -36611,7 +36716,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2739</v>
+        <v>2749</v>
       </c>
       <c r="B14" s="27" t="s">
         <v>72</v>
@@ -36640,7 +36745,7 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2740</v>
+        <v>2750</v>
       </c>
       <c r="E15" s="27" t="s">
         <v>22</v>
@@ -36655,14 +36760,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2741</v>
+        <v>2751</v>
       </c>
       <c r="B16" s="27" t="s">
         <v>626</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2742</v>
+        <v>2752</v>
       </c>
       <c r="E16" s="27" t="s">
         <v>22</v>
@@ -36677,17 +36782,17 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2743</v>
+        <v>2753</v>
       </c>
       <c r="B17" s="27" t="s">
         <v>91</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2744</v>
+        <v>2754</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>2745</v>
+        <v>2755</v>
       </c>
       <c r="F17"/>
       <c r="H17" s="27" t="s">
@@ -36699,10 +36804,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2746</v>
+        <v>2756</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>2747</v>
+        <v>2757</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
@@ -36721,14 +36826,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2748</v>
+        <v>2758</v>
       </c>
       <c r="B19" s="27" t="s">
         <v>140</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2749</v>
+        <v>2759</v>
       </c>
       <c r="E19" s="27" t="s">
         <v>22</v>
@@ -37671,13 +37776,13 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>2747</v>
+        <v>2757</v>
       </c>
       <c r="B85" t="s">
-        <v>2750</v>
+        <v>2760</v>
       </c>
       <c r="C85" t="s">
-        <v>2751</v>
+        <v>2761</v>
       </c>
       <c r="D85" t="s">
         <v>22</v>
@@ -37689,10 +37794,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>2752</v>
+        <v>2762</v>
       </c>
       <c r="C86" t="s">
-        <v>2753</v>
+        <v>2763</v>
       </c>
       <c r="D86" t="s">
         <v>22</v>
@@ -37704,10 +37809,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>2754</v>
+        <v>2764</v>
       </c>
       <c r="C87" t="s">
-        <v>2755</v>
+        <v>2765</v>
       </c>
       <c r="D87" t="s">
         <v>22</v>
@@ -37719,10 +37824,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>2756</v>
+        <v>2766</v>
       </c>
       <c r="C88" t="s">
-        <v>2757</v>
+        <v>2767</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -37734,10 +37839,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2758</v>
+        <v>2768</v>
       </c>
       <c r="C89" t="s">
-        <v>2759</v>
+        <v>2769</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -37749,10 +37854,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>2760</v>
+        <v>2770</v>
       </c>
       <c r="C90" t="s">
-        <v>2761</v>
+        <v>2771</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -37764,10 +37869,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>2762</v>
+        <v>2772</v>
       </c>
       <c r="C91" t="s">
-        <v>2763</v>
+        <v>2773</v>
       </c>
       <c r="D91" t="s">
         <v>22</v>
@@ -37779,10 +37884,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>2764</v>
+        <v>2774</v>
       </c>
       <c r="C92" t="s">
-        <v>2765</v>
+        <v>2775</v>
       </c>
       <c r="D92" t="s">
         <v>22</v>
@@ -37794,10 +37899,10 @@
     <row r="93">
       <c r="A93"/>
       <c r="B93" t="s">
-        <v>2766</v>
+        <v>2776</v>
       </c>
       <c r="C93" t="s">
-        <v>2767</v>
+        <v>2777</v>
       </c>
       <c r="D93" t="s">
         <v>22</v>
@@ -37809,10 +37914,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>2768</v>
+        <v>2778</v>
       </c>
       <c r="C94" t="s">
-        <v>2769</v>
+        <v>2779</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -37824,10 +37929,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
-        <v>2770</v>
+        <v>2780</v>
       </c>
       <c r="C95" t="s">
-        <v>2771</v>
+        <v>2781</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -37839,10 +37944,10 @@
     <row r="96">
       <c r="A96"/>
       <c r="B96" t="s">
-        <v>2772</v>
+        <v>2782</v>
       </c>
       <c r="C96" t="s">
-        <v>2773</v>
+        <v>2783</v>
       </c>
       <c r="D96" t="s">
         <v>22</v>
@@ -37854,10 +37959,10 @@
     <row r="97">
       <c r="A97"/>
       <c r="B97" t="s">
-        <v>2774</v>
+        <v>2784</v>
       </c>
       <c r="C97" t="s">
-        <v>2775</v>
+        <v>2785</v>
       </c>
       <c r="D97" t="s">
         <v>22</v>
@@ -37869,10 +37974,10 @@
     <row r="98">
       <c r="A98"/>
       <c r="B98" t="s">
-        <v>2776</v>
+        <v>2786</v>
       </c>
       <c r="C98" t="s">
-        <v>2777</v>
+        <v>2787</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -37884,10 +37989,10 @@
     <row r="99">
       <c r="A99"/>
       <c r="B99" t="s">
-        <v>2778</v>
+        <v>2788</v>
       </c>
       <c r="C99" t="s">
-        <v>2779</v>
+        <v>2789</v>
       </c>
       <c r="D99" t="s">
         <v>22</v>
@@ -37914,12 +38019,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>2780</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2781</v>
+        <v>2791</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#5644 / #4694 - move jurisdiction check to database for cases
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12051" uniqueCount="2866">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12067" uniqueCount="2874">
   <si>
     <t>Field</t>
   </si>
@@ -7679,6 +7679,18 @@
     <t>contact tracing</t>
   </si>
   <si>
+    <t>CONTACT_MANAGEMENT</t>
+  </si>
+  <si>
+    <t>contact management</t>
+  </si>
+  <si>
+    <t>SOURCECASE_TRACING</t>
+  </si>
+  <si>
+    <t>source case tracing</t>
+  </si>
+  <si>
     <t>SAMPLE_COLLECTION</t>
   </si>
   <si>
@@ -7745,6 +7757,18 @@
     <t>quarantine place</t>
   </si>
   <si>
+    <t>QUARANTINE_MANAGEMENT</t>
+  </si>
+  <si>
+    <t>quarantine management</t>
+  </si>
+  <si>
+    <t>QUARANTINE_ORDER_SEND</t>
+  </si>
+  <si>
+    <t>send quarantine order</t>
+  </si>
+  <si>
     <t>VACCINATION_ACTIVITIES</t>
   </si>
   <si>
@@ -8639,7 +8663,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.60.0-SNAPSHOT</t>
+    <t>1.0.0</t>
   </si>
 </sst>
 </file>
@@ -9387,7 +9411,7 @@
 </file>
 
 <file path=xl/tables/table136.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="TaskTaskType" displayName="TaskTaskType" ref="A27:E50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="TaskTaskType" displayName="TaskTaskType" ref="A27:E54">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -9401,7 +9425,7 @@
 </file>
 
 <file path=xl/tables/table137.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="TaskTaskPriority" displayName="TaskTaskPriority" ref="A52:E55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="TaskTaskPriority" displayName="TaskTaskPriority" ref="A56:E59">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -9415,7 +9439,7 @@
 </file>
 
 <file path=xl/tables/table138.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TaskTaskStatus" displayName="TaskTaskStatus" ref="A57:E61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TaskTaskStatus" displayName="TaskTaskStatus" ref="A61:E65">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -31926,7 +31950,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -32767,10 +32791,10 @@
     <row r="47">
       <c r="A47"/>
       <c r="B47" t="s">
-        <v>173</v>
+        <v>2571</v>
       </c>
       <c r="C47" t="s">
-        <v>2571</v>
+        <v>2572</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
@@ -32782,10 +32806,10 @@
     <row r="48">
       <c r="A48"/>
       <c r="B48" t="s">
-        <v>2572</v>
+        <v>2573</v>
       </c>
       <c r="C48" t="s">
-        <v>2573</v>
+        <v>2574</v>
       </c>
       <c r="D48" t="s">
         <v>22</v>
@@ -32797,10 +32821,10 @@
     <row r="49">
       <c r="A49"/>
       <c r="B49" t="s">
-        <v>2574</v>
+        <v>2575</v>
       </c>
       <c r="C49" t="s">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -32812,10 +32836,10 @@
     <row r="50">
       <c r="A50"/>
       <c r="B50" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="C50" t="s">
-        <v>2577</v>
+        <v>2578</v>
       </c>
       <c r="D50" t="s">
         <v>22</v>
@@ -32824,32 +32848,43 @@
         <v>22</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51"/>
+      <c r="B51" t="s">
+        <v>173</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2579</v>
+      </c>
+      <c r="D51" t="s">
+        <v>22</v>
+      </c>
+      <c r="E51" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="52">
-      <c r="A52" t="s">
-        <v>1</v>
-      </c>
+      <c r="A52"/>
       <c r="B52" t="s">
-        <v>152</v>
+        <v>2580</v>
       </c>
       <c r="C52" t="s">
-        <v>3</v>
+        <v>2581</v>
       </c>
       <c r="D52" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E52" t="s">
-        <v>162</v>
+        <v>22</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="s">
-        <v>2502</v>
-      </c>
+      <c r="A53"/>
       <c r="B53" t="s">
-        <v>2578</v>
+        <v>2582</v>
       </c>
       <c r="C53" t="s">
-        <v>2579</v>
+        <v>2583</v>
       </c>
       <c r="D53" t="s">
         <v>22</v>
@@ -32861,10 +32896,10 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>2580</v>
+        <v>2584</v>
       </c>
       <c r="C54" t="s">
-        <v>2581</v>
+        <v>2585</v>
       </c>
       <c r="D54" t="s">
         <v>22</v>
@@ -32873,47 +32908,47 @@
         <v>22</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55"/>
-      <c r="B55" t="s">
-        <v>2582</v>
-      </c>
-      <c r="C55" t="s">
-        <v>2583</v>
-      </c>
-      <c r="D55" t="s">
-        <v>22</v>
-      </c>
-      <c r="E55" t="s">
-        <v>22</v>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>1</v>
+      </c>
+      <c r="B56" t="s">
+        <v>152</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>4</v>
+      </c>
+      <c r="E56" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>1</v>
+        <v>2502</v>
       </c>
       <c r="B57" t="s">
-        <v>152</v>
+        <v>2586</v>
       </c>
       <c r="C57" t="s">
-        <v>3</v>
+        <v>2587</v>
       </c>
       <c r="D57" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E57" t="s">
-        <v>162</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="s">
-        <v>2509</v>
-      </c>
+      <c r="A58"/>
       <c r="B58" t="s">
-        <v>981</v>
+        <v>2588</v>
       </c>
       <c r="C58" t="s">
-        <v>2584</v>
+        <v>2589</v>
       </c>
       <c r="D58" t="s">
         <v>22</v>
@@ -32925,45 +32960,94 @@
     <row r="59">
       <c r="A59"/>
       <c r="B59" t="s">
+        <v>2590</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2591</v>
+      </c>
+      <c r="D59" t="s">
+        <v>22</v>
+      </c>
+      <c r="E59" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>1</v>
+      </c>
+      <c r="B61" t="s">
+        <v>152</v>
+      </c>
+      <c r="C61" t="s">
+        <v>3</v>
+      </c>
+      <c r="D61" t="s">
+        <v>4</v>
+      </c>
+      <c r="E61" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B62" t="s">
+        <v>981</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2592</v>
+      </c>
+      <c r="D62" t="s">
+        <v>22</v>
+      </c>
+      <c r="E62" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63"/>
+      <c r="B63" t="s">
         <v>984</v>
       </c>
-      <c r="C59" t="s">
-        <v>2585</v>
-      </c>
-      <c r="D59" t="s">
-        <v>22</v>
-      </c>
-      <c r="E59" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60"/>
-      <c r="B60" t="s">
-        <v>2586</v>
-      </c>
-      <c r="C60" t="s">
-        <v>2587</v>
-      </c>
-      <c r="D60" t="s">
-        <v>22</v>
-      </c>
-      <c r="E60" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61"/>
-      <c r="B61" t="s">
-        <v>2588</v>
-      </c>
-      <c r="C61" t="s">
-        <v>2589</v>
-      </c>
-      <c r="D61" t="s">
-        <v>22</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="C63" t="s">
+        <v>2593</v>
+      </c>
+      <c r="D63" t="s">
+        <v>22</v>
+      </c>
+      <c r="E63" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64"/>
+      <c r="B64" t="s">
+        <v>2594</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2595</v>
+      </c>
+      <c r="D64" t="s">
+        <v>22</v>
+      </c>
+      <c r="E64" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65"/>
+      <c r="B65" t="s">
+        <v>2596</v>
+      </c>
+      <c r="C65" t="s">
+        <v>2597</v>
+      </c>
+      <c r="D65" t="s">
+        <v>22</v>
+      </c>
+      <c r="E65" t="s">
         <v>22</v>
       </c>
     </row>
@@ -33034,7 +33118,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2590</v>
+        <v>2598</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>2494</v>
@@ -33056,17 +33140,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2591</v>
+        <v>2599</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>2592</v>
+        <v>2600</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2593</v>
+        <v>2601</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>2594</v>
+        <v>2602</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -33080,14 +33164,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2595</v>
+        <v>2603</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>2596</v>
+        <v>2604</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2597</v>
+        <v>2605</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>22</v>
@@ -33102,10 +33186,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2598</v>
+        <v>2606</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>2599</v>
+        <v>2607</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
@@ -33124,14 +33208,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2600</v>
+        <v>2608</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2601</v>
+        <v>2609</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>22</v>
@@ -33146,14 +33230,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2602</v>
+        <v>2610</v>
       </c>
       <c r="B7" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2603</v>
+        <v>2611</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>22</v>
@@ -33168,14 +33252,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2604</v>
+        <v>2612</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>2605</v>
+        <v>2613</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2606</v>
+        <v>2614</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>22</v>
@@ -33234,14 +33318,14 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2607</v>
+        <v>2615</v>
       </c>
       <c r="B11" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>2608</v>
+        <v>2616</v>
       </c>
       <c r="E11" s="22" t="s">
         <v>22</v>
@@ -33256,7 +33340,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2609</v>
+        <v>2617</v>
       </c>
       <c r="B12" s="22" t="s">
         <v>12</v>
@@ -33266,7 +33350,7 @@
         <v>4</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>2610</v>
+        <v>2618</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -33280,14 +33364,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2611</v>
+        <v>2619</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>687</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2612</v>
+        <v>2620</v>
       </c>
       <c r="E13" s="22" t="s">
         <v>22</v>
@@ -33309,10 +33393,10 @@
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2613</v>
+        <v>2621</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>2614</v>
+        <v>2622</v>
       </c>
       <c r="F14"/>
       <c r="H14" s="22" t="s">
@@ -33331,10 +33415,10 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2615</v>
+        <v>2623</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>2616</v>
+        <v>2624</v>
       </c>
       <c r="F15"/>
       <c r="H15" s="22" t="s">
@@ -33394,14 +33478,14 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2617</v>
+        <v>2625</v>
       </c>
       <c r="B18" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>2618</v>
+        <v>2626</v>
       </c>
       <c r="E18" s="22" t="s">
         <v>22</v>
@@ -33416,14 +33500,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2619</v>
+        <v>2627</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2620</v>
+        <v>2628</v>
       </c>
       <c r="E19" s="22" t="s">
         <v>22</v>
@@ -33438,7 +33522,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2621</v>
+        <v>2629</v>
       </c>
       <c r="B20" s="22" t="s">
         <v>110</v>
@@ -33470,7 +33554,7 @@
         <v>1139</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>2622</v>
+        <v>2630</v>
       </c>
       <c r="F21"/>
       <c r="H21" s="22" t="s">
@@ -33550,14 +33634,14 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>2623</v>
+        <v>2631</v>
       </c>
       <c r="B25" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C25"/>
       <c r="D25" t="s">
-        <v>2624</v>
+        <v>2632</v>
       </c>
       <c r="E25" s="22" t="s">
         <v>22</v>
@@ -33594,14 +33678,14 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>2625</v>
+        <v>2633</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>2626</v>
+        <v>2634</v>
       </c>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>2627</v>
+        <v>2635</v>
       </c>
       <c r="E27" s="22" t="s">
         <v>22</v>
@@ -33616,14 +33700,14 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2628</v>
+        <v>2636</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>2629</v>
+        <v>2637</v>
       </c>
       <c r="C28"/>
       <c r="D28" t="s">
-        <v>2630</v>
+        <v>2638</v>
       </c>
       <c r="E28" s="22" t="s">
         <v>22</v>
@@ -33638,14 +33722,14 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>2631</v>
+        <v>2639</v>
       </c>
       <c r="B29" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>2632</v>
+        <v>2640</v>
       </c>
       <c r="E29" s="22" t="s">
         <v>22</v>
@@ -33660,17 +33744,17 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>2633</v>
+        <v>2641</v>
       </c>
       <c r="B30" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>2634</v>
+        <v>2642</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>2635</v>
+        <v>2643</v>
       </c>
       <c r="F30"/>
       <c r="H30" s="22" t="s">
@@ -33682,17 +33766,17 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2636</v>
+        <v>2644</v>
       </c>
       <c r="B31" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>2637</v>
+        <v>2645</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>2638</v>
+        <v>2646</v>
       </c>
       <c r="F31"/>
       <c r="H31" s="22" t="s">
@@ -33704,17 +33788,17 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>2639</v>
+        <v>2647</v>
       </c>
       <c r="B32" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C32"/>
       <c r="D32" t="s">
-        <v>2640</v>
+        <v>2648</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>2641</v>
+        <v>2649</v>
       </c>
       <c r="F32"/>
       <c r="H32" s="22" t="s">
@@ -33726,7 +33810,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>2642</v>
+        <v>2650</v>
       </c>
       <c r="B33" s="22" t="s">
         <v>12</v>
@@ -33736,7 +33820,7 @@
         <v>562</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>2643</v>
+        <v>2651</v>
       </c>
       <c r="F33"/>
       <c r="H33" s="22" t="s">
@@ -33748,17 +33832,17 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>2644</v>
+        <v>2652</v>
       </c>
       <c r="B34" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C34"/>
       <c r="D34" t="s">
-        <v>2645</v>
+        <v>2653</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>2646</v>
+        <v>2654</v>
       </c>
       <c r="F34"/>
       <c r="H34" s="22" t="s">
@@ -33770,17 +33854,17 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>2647</v>
+        <v>2655</v>
       </c>
       <c r="B35" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>2648</v>
+        <v>2656</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>2649</v>
+        <v>2657</v>
       </c>
       <c r="F35"/>
       <c r="H35" s="22" t="s">
@@ -33792,17 +33876,17 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2650</v>
+        <v>2658</v>
       </c>
       <c r="B36" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C36"/>
       <c r="D36" t="s">
-        <v>2651</v>
+        <v>2659</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>2652</v>
+        <v>2660</v>
       </c>
       <c r="F36"/>
       <c r="H36" s="22" t="s">
@@ -33858,7 +33942,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>2653</v>
+        <v>2661</v>
       </c>
       <c r="B39" s="22" t="s">
         <v>662</v>
@@ -33882,14 +33966,14 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>2654</v>
+        <v>2662</v>
       </c>
       <c r="B40" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C40"/>
       <c r="D40" t="s">
-        <v>2655</v>
+        <v>2663</v>
       </c>
       <c r="E40" s="22" t="s">
         <v>22</v>
@@ -33970,14 +34054,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>2656</v>
+        <v>2664</v>
       </c>
       <c r="B44" s="22" t="s">
         <v>687</v>
       </c>
       <c r="C44"/>
       <c r="D44" t="s">
-        <v>2657</v>
+        <v>2665</v>
       </c>
       <c r="E44" s="22" t="s">
         <v>22</v>
@@ -33992,14 +34076,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>2658</v>
+        <v>2666</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>2659</v>
+        <v>2667</v>
       </c>
       <c r="C45"/>
       <c r="D45" t="s">
-        <v>2660</v>
+        <v>2668</v>
       </c>
       <c r="E45" s="22" t="s">
         <v>22</v>
@@ -34014,17 +34098,17 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>2661</v>
+        <v>2669</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>2662</v>
+        <v>2670</v>
       </c>
       <c r="C46"/>
       <c r="D46" t="s">
-        <v>2663</v>
+        <v>2671</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>2664</v>
+        <v>2672</v>
       </c>
       <c r="F46"/>
       <c r="H46" s="22" t="s">
@@ -34038,14 +34122,14 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>2665</v>
+        <v>2673</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>2666</v>
+        <v>2674</v>
       </c>
       <c r="C47"/>
       <c r="D47" t="s">
-        <v>2667</v>
+        <v>2675</v>
       </c>
       <c r="E47" s="22" t="s">
         <v>22</v>
@@ -34062,14 +34146,14 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>2668</v>
+        <v>2676</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>2669</v>
+        <v>2677</v>
       </c>
       <c r="C48"/>
       <c r="D48" t="s">
-        <v>2670</v>
+        <v>2678</v>
       </c>
       <c r="E48" s="22" t="s">
         <v>22</v>
@@ -34086,14 +34170,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>2671</v>
+        <v>2679</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>2672</v>
+        <v>2680</v>
       </c>
       <c r="C49"/>
       <c r="D49" t="s">
-        <v>2673</v>
+        <v>2681</v>
       </c>
       <c r="E49" s="22" t="s">
         <v>22</v>
@@ -34110,14 +34194,14 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>2674</v>
+        <v>2682</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>687</v>
       </c>
       <c r="C50"/>
       <c r="D50" t="s">
-        <v>2675</v>
+        <v>2683</v>
       </c>
       <c r="E50" s="22" t="s">
         <v>22</v>
@@ -34134,7 +34218,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>2676</v>
+        <v>2684</v>
       </c>
       <c r="B51" s="22"/>
       <c r="C51"/>
@@ -34156,14 +34240,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>2677</v>
+        <v>2685</v>
       </c>
       <c r="B52" s="22" t="s">
         <v>687</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>2678</v>
+        <v>2686</v>
       </c>
       <c r="E52" s="22" t="s">
         <v>22</v>
@@ -34180,7 +34264,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>2679</v>
+        <v>2687</v>
       </c>
       <c r="B53" s="22"/>
       <c r="C53"/>
@@ -34246,14 +34330,14 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>2680</v>
+        <v>2688</v>
       </c>
       <c r="B56" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C56"/>
       <c r="D56" t="s">
-        <v>2681</v>
+        <v>2689</v>
       </c>
       <c r="E56" s="22" t="s">
         <v>22</v>
@@ -34287,13 +34371,13 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>2592</v>
+        <v>2600</v>
       </c>
       <c r="B59" t="s">
-        <v>2682</v>
+        <v>2690</v>
       </c>
       <c r="C59" t="s">
-        <v>2683</v>
+        <v>2691</v>
       </c>
       <c r="D59" t="s">
         <v>22</v>
@@ -34335,10 +34419,10 @@
     <row r="62">
       <c r="A62"/>
       <c r="B62" t="s">
-        <v>2684</v>
+        <v>2692</v>
       </c>
       <c r="C62" t="s">
-        <v>2685</v>
+        <v>2693</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -34381,13 +34465,13 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>2596</v>
+        <v>2604</v>
       </c>
       <c r="B66" t="s">
-        <v>2582</v>
+        <v>2590</v>
       </c>
       <c r="C66" t="s">
-        <v>2686</v>
+        <v>2694</v>
       </c>
       <c r="D66" t="s">
         <v>22</v>
@@ -34399,10 +34483,10 @@
     <row r="67">
       <c r="A67"/>
       <c r="B67" t="s">
-        <v>2687</v>
+        <v>2695</v>
       </c>
       <c r="C67" t="s">
-        <v>2688</v>
+        <v>2696</v>
       </c>
       <c r="D67" t="s">
         <v>22</v>
@@ -34414,10 +34498,10 @@
     <row r="68">
       <c r="A68"/>
       <c r="B68" t="s">
-        <v>2578</v>
+        <v>2586</v>
       </c>
       <c r="C68" t="s">
-        <v>2689</v>
+        <v>2697</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
@@ -34460,7 +34544,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>2599</v>
+        <v>2607</v>
       </c>
       <c r="B72" t="s">
         <v>981</v>
@@ -34478,10 +34562,10 @@
     <row r="73">
       <c r="A73"/>
       <c r="B73" t="s">
-        <v>2690</v>
+        <v>2698</v>
       </c>
       <c r="C73" t="s">
-        <v>2691</v>
+        <v>2699</v>
       </c>
       <c r="D73" t="s">
         <v>22</v>
@@ -34539,7 +34623,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>2605</v>
+        <v>2613</v>
       </c>
       <c r="B78" t="s">
         <v>981</v>
@@ -34557,7 +34641,7 @@
     <row r="79">
       <c r="A79"/>
       <c r="B79" t="s">
-        <v>2690</v>
+        <v>2698</v>
       </c>
       <c r="C79" t="s">
         <v>1091</v>
@@ -34587,10 +34671,10 @@
     <row r="81">
       <c r="A81"/>
       <c r="B81" t="s">
-        <v>2692</v>
+        <v>2700</v>
       </c>
       <c r="C81" t="s">
-        <v>2693</v>
+        <v>2701</v>
       </c>
       <c r="D81" t="s">
         <v>22</v>
@@ -35084,13 +35168,13 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>2626</v>
+        <v>2634</v>
       </c>
       <c r="B118" t="s">
-        <v>2694</v>
+        <v>2702</v>
       </c>
       <c r="C118" t="s">
-        <v>2695</v>
+        <v>2703</v>
       </c>
       <c r="D118" t="s">
         <v>22</v>
@@ -35102,10 +35186,10 @@
     <row r="119">
       <c r="A119"/>
       <c r="B119" t="s">
-        <v>2696</v>
+        <v>2704</v>
       </c>
       <c r="C119" t="s">
-        <v>2697</v>
+        <v>2705</v>
       </c>
       <c r="D119" t="s">
         <v>22</v>
@@ -35117,10 +35201,10 @@
     <row r="120">
       <c r="A120"/>
       <c r="B120" t="s">
-        <v>2698</v>
+        <v>2706</v>
       </c>
       <c r="C120" t="s">
-        <v>2699</v>
+        <v>2707</v>
       </c>
       <c r="D120" t="s">
         <v>22</v>
@@ -35132,10 +35216,10 @@
     <row r="121">
       <c r="A121"/>
       <c r="B121" t="s">
-        <v>2700</v>
+        <v>2708</v>
       </c>
       <c r="C121" t="s">
-        <v>2701</v>
+        <v>2709</v>
       </c>
       <c r="D121" t="s">
         <v>22</v>
@@ -35147,10 +35231,10 @@
     <row r="122">
       <c r="A122"/>
       <c r="B122" t="s">
-        <v>2702</v>
+        <v>2710</v>
       </c>
       <c r="C122" t="s">
-        <v>2703</v>
+        <v>2711</v>
       </c>
       <c r="D122" t="s">
         <v>22</v>
@@ -35178,13 +35262,13 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>2629</v>
+        <v>2637</v>
       </c>
       <c r="B125" t="s">
-        <v>2704</v>
+        <v>2712</v>
       </c>
       <c r="C125" t="s">
-        <v>2705</v>
+        <v>2713</v>
       </c>
       <c r="D125" t="s">
         <v>22</v>
@@ -35196,10 +35280,10 @@
     <row r="126">
       <c r="A126"/>
       <c r="B126" t="s">
-        <v>2706</v>
+        <v>2714</v>
       </c>
       <c r="C126" t="s">
-        <v>2707</v>
+        <v>2715</v>
       </c>
       <c r="D126" t="s">
         <v>22</v>
@@ -35211,10 +35295,10 @@
     <row r="127">
       <c r="A127"/>
       <c r="B127" t="s">
-        <v>2708</v>
+        <v>2716</v>
       </c>
       <c r="C127" t="s">
-        <v>2709</v>
+        <v>2717</v>
       </c>
       <c r="D127" t="s">
         <v>22</v>
@@ -35226,10 +35310,10 @@
     <row r="128">
       <c r="A128"/>
       <c r="B128" t="s">
-        <v>2710</v>
+        <v>2718</v>
       </c>
       <c r="C128" t="s">
-        <v>2711</v>
+        <v>2719</v>
       </c>
       <c r="D128" t="s">
         <v>22</v>
@@ -35241,10 +35325,10 @@
     <row r="129">
       <c r="A129"/>
       <c r="B129" t="s">
-        <v>2712</v>
+        <v>2720</v>
       </c>
       <c r="C129" t="s">
-        <v>2713</v>
+        <v>2721</v>
       </c>
       <c r="D129" t="s">
         <v>22</v>
@@ -36146,13 +36230,13 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>2659</v>
+        <v>2667</v>
       </c>
       <c r="B191" t="s">
-        <v>2714</v>
+        <v>2722</v>
       </c>
       <c r="C191" t="s">
-        <v>2715</v>
+        <v>2723</v>
       </c>
       <c r="D191" t="s">
         <v>22</v>
@@ -36167,7 +36251,7 @@
         <v>2328</v>
       </c>
       <c r="C192" t="s">
-        <v>2716</v>
+        <v>2724</v>
       </c>
       <c r="D192" t="s">
         <v>22</v>
@@ -36182,7 +36266,7 @@
         <v>2330</v>
       </c>
       <c r="C193" t="s">
-        <v>2717</v>
+        <v>2725</v>
       </c>
       <c r="D193" t="s">
         <v>22</v>
@@ -36194,10 +36278,10 @@
     <row r="194">
       <c r="A194"/>
       <c r="B194" t="s">
-        <v>2718</v>
+        <v>2726</v>
       </c>
       <c r="C194" t="s">
-        <v>2719</v>
+        <v>2727</v>
       </c>
       <c r="D194" t="s">
         <v>22</v>
@@ -36209,10 +36293,10 @@
     <row r="195">
       <c r="A195"/>
       <c r="B195" t="s">
-        <v>2720</v>
+        <v>2728</v>
       </c>
       <c r="C195" t="s">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="D195" t="s">
         <v>22</v>
@@ -36255,7 +36339,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>2662</v>
+        <v>2670</v>
       </c>
       <c r="B199" t="s">
         <v>934</v>
@@ -36334,13 +36418,13 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>2666</v>
+        <v>2674</v>
       </c>
       <c r="B205" t="s">
-        <v>2722</v>
+        <v>2730</v>
       </c>
       <c r="C205" t="s">
-        <v>2723</v>
+        <v>2731</v>
       </c>
       <c r="D205" t="s">
         <v>22</v>
@@ -36352,10 +36436,10 @@
     <row r="206">
       <c r="A206"/>
       <c r="B206" t="s">
-        <v>2724</v>
+        <v>2732</v>
       </c>
       <c r="C206" t="s">
-        <v>2725</v>
+        <v>2733</v>
       </c>
       <c r="D206" t="s">
         <v>22</v>
@@ -36367,10 +36451,10 @@
     <row r="207">
       <c r="A207"/>
       <c r="B207" t="s">
-        <v>2726</v>
+        <v>2734</v>
       </c>
       <c r="C207" t="s">
-        <v>2727</v>
+        <v>2735</v>
       </c>
       <c r="D207" t="s">
         <v>22</v>
@@ -36382,10 +36466,10 @@
     <row r="208">
       <c r="A208"/>
       <c r="B208" t="s">
-        <v>2728</v>
+        <v>2736</v>
       </c>
       <c r="C208" t="s">
-        <v>2729</v>
+        <v>2737</v>
       </c>
       <c r="D208" t="s">
         <v>22</v>
@@ -36397,10 +36481,10 @@
     <row r="209">
       <c r="A209"/>
       <c r="B209" t="s">
-        <v>2730</v>
+        <v>2738</v>
       </c>
       <c r="C209" t="s">
-        <v>2731</v>
+        <v>2739</v>
       </c>
       <c r="D209" t="s">
         <v>22</v>
@@ -36412,10 +36496,10 @@
     <row r="210">
       <c r="A210"/>
       <c r="B210" t="s">
-        <v>2732</v>
+        <v>2740</v>
       </c>
       <c r="C210" t="s">
-        <v>2733</v>
+        <v>2741</v>
       </c>
       <c r="D210" t="s">
         <v>22</v>
@@ -36458,13 +36542,13 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>2669</v>
+        <v>2677</v>
       </c>
       <c r="B214" t="s">
-        <v>2734</v>
+        <v>2742</v>
       </c>
       <c r="C214" t="s">
-        <v>2735</v>
+        <v>2743</v>
       </c>
       <c r="D214" t="s">
         <v>22</v>
@@ -36476,10 +36560,10 @@
     <row r="215">
       <c r="A215"/>
       <c r="B215" t="s">
-        <v>2736</v>
+        <v>2744</v>
       </c>
       <c r="C215" t="s">
-        <v>2737</v>
+        <v>2745</v>
       </c>
       <c r="D215" t="s">
         <v>22</v>
@@ -36491,10 +36575,10 @@
     <row r="216">
       <c r="A216"/>
       <c r="B216" t="s">
-        <v>2738</v>
+        <v>2746</v>
       </c>
       <c r="C216" t="s">
-        <v>2739</v>
+        <v>2747</v>
       </c>
       <c r="D216" t="s">
         <v>22</v>
@@ -36506,10 +36590,10 @@
     <row r="217">
       <c r="A217"/>
       <c r="B217" t="s">
-        <v>2740</v>
+        <v>2748</v>
       </c>
       <c r="C217" t="s">
-        <v>2741</v>
+        <v>2749</v>
       </c>
       <c r="D217" t="s">
         <v>22</v>
@@ -36521,10 +36605,10 @@
     <row r="218">
       <c r="A218"/>
       <c r="B218" t="s">
-        <v>2742</v>
+        <v>2750</v>
       </c>
       <c r="C218" t="s">
-        <v>2743</v>
+        <v>2751</v>
       </c>
       <c r="D218" t="s">
         <v>22</v>
@@ -36567,13 +36651,13 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>2672</v>
+        <v>2680</v>
       </c>
       <c r="B222" t="s">
-        <v>2744</v>
+        <v>2752</v>
       </c>
       <c r="C222" t="s">
-        <v>2745</v>
+        <v>2753</v>
       </c>
       <c r="D222" t="s">
         <v>22</v>
@@ -36585,10 +36669,10 @@
     <row r="223">
       <c r="A223"/>
       <c r="B223" t="s">
-        <v>2746</v>
+        <v>2754</v>
       </c>
       <c r="C223" t="s">
-        <v>2747</v>
+        <v>2755</v>
       </c>
       <c r="D223" t="s">
         <v>22</v>
@@ -36600,10 +36684,10 @@
     <row r="224">
       <c r="A224"/>
       <c r="B224" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="C224" t="s">
-        <v>2749</v>
+        <v>2757</v>
       </c>
       <c r="D224" t="s">
         <v>22</v>
@@ -36615,10 +36699,10 @@
     <row r="225">
       <c r="A225"/>
       <c r="B225" t="s">
-        <v>2750</v>
+        <v>2758</v>
       </c>
       <c r="C225" t="s">
-        <v>2751</v>
+        <v>2759</v>
       </c>
       <c r="D225" t="s">
         <v>22</v>
@@ -36630,10 +36714,10 @@
     <row r="226">
       <c r="A226"/>
       <c r="B226" t="s">
-        <v>2752</v>
+        <v>2760</v>
       </c>
       <c r="C226" t="s">
-        <v>2753</v>
+        <v>2761</v>
       </c>
       <c r="D226" t="s">
         <v>22</v>
@@ -36791,7 +36875,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2754</v>
+        <v>2762</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>12</v>
@@ -36800,7 +36884,7 @@
         <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>2755</v>
+        <v>2763</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>22</v>
@@ -37008,14 +37092,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2756</v>
+        <v>2764</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>2757</v>
+        <v>2765</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2758</v>
+        <v>2766</v>
       </c>
       <c r="E2" s="24" t="s">
         <v>22</v>
@@ -37054,14 +37138,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2759</v>
+        <v>2767</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>2760</v>
+        <v>2768</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2761</v>
+        <v>2769</v>
       </c>
       <c r="E4" s="24" t="s">
         <v>22</v>
@@ -37079,7 +37163,7 @@
         <v>2501</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>2762</v>
+        <v>2770</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
@@ -37098,7 +37182,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2763</v>
+        <v>2771</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>55</v>
@@ -37122,14 +37206,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2764</v>
+        <v>2772</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>2765</v>
+        <v>2773</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2766</v>
+        <v>2774</v>
       </c>
       <c r="E7" s="24" t="s">
         <v>22</v>
@@ -37188,14 +37272,14 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2767</v>
+        <v>2775</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>2608</v>
+        <v>2616</v>
       </c>
       <c r="E10" s="24" t="s">
         <v>22</v>
@@ -37232,7 +37316,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2768</v>
+        <v>2776</v>
       </c>
       <c r="B12" s="24" t="s">
         <v>12</v>
@@ -37254,14 +37338,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2769</v>
+        <v>2777</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>662</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2770</v>
+        <v>2778</v>
       </c>
       <c r="E13" s="24" t="s">
         <v>22</v>
@@ -37293,7 +37377,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2757</v>
+        <v>2765</v>
       </c>
       <c r="B16" t="s">
         <v>2530</v>
@@ -37327,13 +37411,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2760</v>
+        <v>2768</v>
       </c>
       <c r="B19" t="s">
-        <v>2771</v>
+        <v>2779</v>
       </c>
       <c r="C19" t="s">
-        <v>2772</v>
+        <v>2780</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -37345,10 +37429,10 @@
     <row r="20">
       <c r="A20"/>
       <c r="B20" t="s">
-        <v>2545</v>
+        <v>2549</v>
       </c>
       <c r="C20" t="s">
-        <v>2773</v>
+        <v>2781</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -37360,10 +37444,10 @@
     <row r="21">
       <c r="A21"/>
       <c r="B21" t="s">
-        <v>2774</v>
+        <v>2782</v>
       </c>
       <c r="C21" t="s">
-        <v>2775</v>
+        <v>2783</v>
       </c>
       <c r="D21" t="s">
         <v>22</v>
@@ -37375,10 +37459,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>2549</v>
+        <v>2553</v>
       </c>
       <c r="C22" t="s">
-        <v>2776</v>
+        <v>2784</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -37390,10 +37474,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>2777</v>
+        <v>2785</v>
       </c>
       <c r="C23" t="s">
-        <v>2778</v>
+        <v>2786</v>
       </c>
       <c r="D23" t="s">
         <v>22</v>
@@ -37405,10 +37489,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>2779</v>
+        <v>2787</v>
       </c>
       <c r="C24" t="s">
-        <v>2780</v>
+        <v>2788</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -37420,10 +37504,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>2781</v>
+        <v>2789</v>
       </c>
       <c r="C25" t="s">
-        <v>2782</v>
+        <v>2790</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -37435,10 +37519,10 @@
     <row r="26">
       <c r="A26"/>
       <c r="B26" t="s">
-        <v>2783</v>
+        <v>2791</v>
       </c>
       <c r="C26" t="s">
-        <v>2784</v>
+        <v>2792</v>
       </c>
       <c r="D26" t="s">
         <v>22</v>
@@ -37450,10 +37534,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>2785</v>
+        <v>2793</v>
       </c>
       <c r="C27" t="s">
-        <v>2786</v>
+        <v>2794</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -37496,13 +37580,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2762</v>
+        <v>2770</v>
       </c>
       <c r="B31" t="s">
-        <v>2578</v>
+        <v>2586</v>
       </c>
       <c r="C31" t="s">
-        <v>2579</v>
+        <v>2587</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -37514,10 +37598,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>2580</v>
+        <v>2588</v>
       </c>
       <c r="C32" t="s">
-        <v>2581</v>
+        <v>2589</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -37529,10 +37613,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>2582</v>
+        <v>2590</v>
       </c>
       <c r="C33" t="s">
-        <v>2583</v>
+        <v>2591</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -37560,7 +37644,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2765</v>
+        <v>2773</v>
       </c>
       <c r="B36" t="s">
         <v>981</v>
@@ -37578,10 +37662,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>2787</v>
+        <v>2795</v>
       </c>
       <c r="C37" t="s">
-        <v>2788</v>
+        <v>2796</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -37672,14 +37756,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2789</v>
+        <v>2797</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2790</v>
+        <v>2798</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>22</v>
@@ -37987,7 +38071,7 @@
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2791</v>
+        <v>2799</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>22</v>
@@ -38009,7 +38093,7 @@
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2792</v>
+        <v>2800</v>
       </c>
       <c r="E17" s="25" t="s">
         <v>22</v>
@@ -38024,7 +38108,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2793</v>
+        <v>2801</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>69</v>
@@ -38046,14 +38130,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2794</v>
+        <v>2802</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>132</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2795</v>
+        <v>2803</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>22</v>
@@ -38068,14 +38152,14 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>132</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>2797</v>
+        <v>2805</v>
       </c>
       <c r="E20" s="25" t="s">
         <v>22</v>
@@ -39158,14 +39242,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2798</v>
+        <v>2806</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2799</v>
+        <v>2807</v>
       </c>
       <c r="E2" s="26" t="s">
         <v>22</v>
@@ -39202,14 +39286,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2800</v>
+        <v>2808</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2801</v>
+        <v>2809</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>22</v>
@@ -39224,14 +39308,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2802</v>
+        <v>2810</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2803</v>
+        <v>2811</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>22</v>
@@ -39246,14 +39330,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>132</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2797</v>
+        <v>2805</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>22</v>
@@ -39351,14 +39435,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2789</v>
+        <v>2797</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2790</v>
+        <v>2798</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>22</v>
@@ -39373,14 +39457,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2804</v>
+        <v>2812</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2805</v>
+        <v>2813</v>
       </c>
       <c r="E3" s="27" t="s">
         <v>22</v>
@@ -39395,14 +39479,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2806</v>
+        <v>2814</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2807</v>
+        <v>2815</v>
       </c>
       <c r="E4" s="27" t="s">
         <v>22</v>
@@ -39417,14 +39501,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>132</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2797</v>
+        <v>2805</v>
       </c>
       <c r="E5" s="27" t="s">
         <v>22</v>
@@ -39461,14 +39545,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2808</v>
+        <v>2816</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>2809</v>
+        <v>2817</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2810</v>
+        <v>2818</v>
       </c>
       <c r="E7" s="27" t="s">
         <v>22</v>
@@ -39566,14 +39650,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2789</v>
+        <v>2797</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2790</v>
+        <v>2798</v>
       </c>
       <c r="E2" s="28" t="s">
         <v>22</v>
@@ -39588,14 +39672,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2804</v>
+        <v>2812</v>
       </c>
       <c r="B3" s="28" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2805</v>
+        <v>2813</v>
       </c>
       <c r="E3" s="28" t="s">
         <v>22</v>
@@ -39610,14 +39694,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2806</v>
+        <v>2814</v>
       </c>
       <c r="B4" s="28" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2807</v>
+        <v>2815</v>
       </c>
       <c r="E4" s="28" t="s">
         <v>22</v>
@@ -39654,14 +39738,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="B6" s="28" t="s">
         <v>132</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2797</v>
+        <v>2805</v>
       </c>
       <c r="E6" s="28" t="s">
         <v>22</v>
@@ -39759,14 +39843,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2789</v>
+        <v>2797</v>
       </c>
       <c r="B2" s="29" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2790</v>
+        <v>2798</v>
       </c>
       <c r="E2" s="29" t="s">
         <v>22</v>
@@ -39781,7 +39865,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2806</v>
+        <v>2814</v>
       </c>
       <c r="B3" s="29" t="s">
         <v>42</v>
@@ -39847,14 +39931,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2796</v>
+        <v>2804</v>
       </c>
       <c r="B6" s="29" t="s">
         <v>132</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2797</v>
+        <v>2805</v>
       </c>
       <c r="E6" s="29" t="s">
         <v>22</v>
@@ -41752,14 +41836,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2811</v>
+        <v>2819</v>
       </c>
       <c r="B2" s="30" t="s">
         <v>132</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2812</v>
+        <v>2820</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>22</v>
@@ -41774,14 +41858,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2813</v>
+        <v>2821</v>
       </c>
       <c r="B3" s="30" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2814</v>
+        <v>2822</v>
       </c>
       <c r="E3" s="30" t="s">
         <v>22</v>
@@ -41840,7 +41924,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2815</v>
+        <v>2823</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>12</v>
@@ -41862,14 +41946,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2816</v>
+        <v>2824</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>12</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2817</v>
+        <v>2825</v>
       </c>
       <c r="E7" s="30" t="s">
         <v>22</v>
@@ -41891,7 +41975,7 @@
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2818</v>
+        <v>2826</v>
       </c>
       <c r="E8" s="30" t="s">
         <v>22</v>
@@ -41906,12 +41990,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2819</v>
+        <v>2827</v>
       </c>
       <c r="B9" s="30"/>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2820</v>
+        <v>2828</v>
       </c>
       <c r="E9" s="30" t="s">
         <v>22</v>
@@ -42014,7 +42098,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2821</v>
+        <v>2829</v>
       </c>
       <c r="B14" s="30" t="s">
         <v>72</v>
@@ -42043,7 +42127,7 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2822</v>
+        <v>2830</v>
       </c>
       <c r="E15" s="30" t="s">
         <v>22</v>
@@ -42058,14 +42142,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2823</v>
+        <v>2831</v>
       </c>
       <c r="B16" s="30" t="s">
         <v>662</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2824</v>
+        <v>2832</v>
       </c>
       <c r="E16" s="30" t="s">
         <v>22</v>
@@ -42080,17 +42164,17 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2825</v>
+        <v>2833</v>
       </c>
       <c r="B17" s="30" t="s">
         <v>91</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2826</v>
+        <v>2834</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>2827</v>
+        <v>2835</v>
       </c>
       <c r="F17"/>
       <c r="H17" s="30" t="s">
@@ -42102,10 +42186,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2828</v>
+        <v>2836</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>2829</v>
+        <v>2837</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
@@ -42124,14 +42208,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2830</v>
+        <v>2838</v>
       </c>
       <c r="B19" s="30" t="s">
         <v>132</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2831</v>
+        <v>2839</v>
       </c>
       <c r="E19" s="30" t="s">
         <v>22</v>
@@ -43074,13 +43158,13 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>2829</v>
+        <v>2837</v>
       </c>
       <c r="B85" t="s">
-        <v>2832</v>
+        <v>2840</v>
       </c>
       <c r="C85" t="s">
-        <v>2833</v>
+        <v>2841</v>
       </c>
       <c r="D85" t="s">
         <v>22</v>
@@ -43092,10 +43176,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>2834</v>
+        <v>2842</v>
       </c>
       <c r="C86" t="s">
-        <v>2835</v>
+        <v>2843</v>
       </c>
       <c r="D86" t="s">
         <v>22</v>
@@ -43107,10 +43191,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>2836</v>
+        <v>2844</v>
       </c>
       <c r="C87" t="s">
-        <v>2837</v>
+        <v>2845</v>
       </c>
       <c r="D87" t="s">
         <v>22</v>
@@ -43122,10 +43206,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>2838</v>
+        <v>2846</v>
       </c>
       <c r="C88" t="s">
-        <v>2839</v>
+        <v>2847</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -43137,10 +43221,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2840</v>
+        <v>2848</v>
       </c>
       <c r="C89" t="s">
-        <v>2841</v>
+        <v>2849</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -43152,10 +43236,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>2842</v>
+        <v>2850</v>
       </c>
       <c r="C90" t="s">
-        <v>2843</v>
+        <v>2851</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -43167,10 +43251,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>2844</v>
+        <v>2852</v>
       </c>
       <c r="C91" t="s">
-        <v>2845</v>
+        <v>2853</v>
       </c>
       <c r="D91" t="s">
         <v>22</v>
@@ -43182,10 +43266,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>2846</v>
+        <v>2854</v>
       </c>
       <c r="C92" t="s">
-        <v>2847</v>
+        <v>2855</v>
       </c>
       <c r="D92" t="s">
         <v>22</v>
@@ -43197,10 +43281,10 @@
     <row r="93">
       <c r="A93"/>
       <c r="B93" t="s">
-        <v>2848</v>
+        <v>2856</v>
       </c>
       <c r="C93" t="s">
-        <v>2849</v>
+        <v>2857</v>
       </c>
       <c r="D93" t="s">
         <v>22</v>
@@ -43212,10 +43296,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>2850</v>
+        <v>2858</v>
       </c>
       <c r="C94" t="s">
-        <v>2851</v>
+        <v>2859</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -43227,10 +43311,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
-        <v>2852</v>
+        <v>2860</v>
       </c>
       <c r="C95" t="s">
-        <v>2853</v>
+        <v>2861</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -43242,10 +43326,10 @@
     <row r="96">
       <c r="A96"/>
       <c r="B96" t="s">
-        <v>2854</v>
+        <v>2862</v>
       </c>
       <c r="C96" t="s">
-        <v>2855</v>
+        <v>2863</v>
       </c>
       <c r="D96" t="s">
         <v>22</v>
@@ -43257,10 +43341,10 @@
     <row r="97">
       <c r="A97"/>
       <c r="B97" t="s">
-        <v>2856</v>
+        <v>2864</v>
       </c>
       <c r="C97" t="s">
-        <v>2857</v>
+        <v>2865</v>
       </c>
       <c r="D97" t="s">
         <v>22</v>
@@ -43272,10 +43356,10 @@
     <row r="98">
       <c r="A98"/>
       <c r="B98" t="s">
-        <v>2858</v>
+        <v>2866</v>
       </c>
       <c r="C98" t="s">
-        <v>2859</v>
+        <v>2867</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -43287,10 +43371,10 @@
     <row r="99">
       <c r="A99"/>
       <c r="B99" t="s">
-        <v>2860</v>
+        <v>2868</v>
       </c>
       <c r="C99" t="s">
-        <v>2861</v>
+        <v>2869</v>
       </c>
       <c r="D99" t="s">
         <v>22</v>
@@ -43302,10 +43386,10 @@
     <row r="100">
       <c r="A100"/>
       <c r="B100" t="s">
-        <v>2862</v>
+        <v>2870</v>
       </c>
       <c r="C100" t="s">
-        <v>2863</v>
+        <v>2871</v>
       </c>
       <c r="D100" t="s">
         <v>22</v>
@@ -43332,12 +43416,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>2864</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2865</v>
+        <v>2873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[#6688] extract etcd client and create producer
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_Data_Dictionary.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12784" uniqueCount="2929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12793" uniqueCount="2933">
   <si>
     <t>Field</t>
   </si>
@@ -7617,6 +7617,15 @@
     <t>contact</t>
   </si>
   <si>
+    <t>travelEntry</t>
+  </si>
+  <si>
+    <t>TravelEntryReference</t>
+  </si>
+  <si>
+    <t>Travel entry</t>
+  </si>
+  <si>
     <t>taskType</t>
   </si>
   <si>
@@ -7726,6 +7735,9 @@
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>TRAVEL_ENTRY</t>
   </si>
   <si>
     <t>ACTIVE_SEARCH_FOR_OTHER_CASES</t>
@@ -9578,7 +9590,7 @@
 </file>
 
 <file path=xl/tables/table135.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="135" name="Task" displayName="Task" ref="A1:K19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="135" name="Task" displayName="Task" ref="A1:K20">
   <autoFilter/>
   <tableColumns count="11">
     <tableColumn id="1" name="Field"/>
@@ -9598,7 +9610,7 @@
 </file>
 
 <file path=xl/tables/table136.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="TaskTaskContext" displayName="TaskTaskContext" ref="A21:E25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="TaskTaskContext" displayName="TaskTaskContext" ref="A22:E27">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -9612,7 +9624,7 @@
 </file>
 
 <file path=xl/tables/table137.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="TaskTaskType" displayName="TaskTaskType" ref="A27:E54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="TaskTaskType" displayName="TaskTaskType" ref="A29:E56">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -9626,7 +9638,7 @@
 </file>
 
 <file path=xl/tables/table138.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TaskTaskPriority" displayName="TaskTaskPriority" ref="A56:E59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TaskTaskPriority" displayName="TaskTaskPriority" ref="A58:E61">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -9640,7 +9652,7 @@
 </file>
 
 <file path=xl/tables/table139.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="139" name="TaskTaskStatus" displayName="TaskTaskStatus" ref="A61:E65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="139" name="TaskTaskStatus" displayName="TaskTaskStatus" ref="A63:E67">
   <autoFilter/>
   <tableColumns count="5">
     <tableColumn id="1" name="Type"/>
@@ -32353,7 +32365,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -32506,11 +32518,9 @@
         <v>2525</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>2526</v>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F6"/>
       <c r="H6" s="21" t="s">
         <v>16</v>
       </c>
@@ -32520,19 +32530,21 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>2527</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>2528</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
+        <v>2528</v>
+      </c>
+      <c r="E7" s="21" t="s">
         <v>2529</v>
       </c>
-      <c r="E7" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7"/>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
       <c r="H7" s="21" t="s">
         <v>16</v>
       </c>
@@ -32545,18 +32557,16 @@
         <v>2530</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>55</v>
+        <v>2531</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="E8" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
+      <c r="F8"/>
       <c r="H8" s="21" t="s">
         <v>16</v>
       </c>
@@ -32566,19 +32576,21 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>55</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="E9" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F9"/>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
       <c r="H9" s="21" t="s">
         <v>16</v>
       </c>
@@ -32588,10 +32600,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2534</v>
+        <v>2535</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>2535</v>
+        <v>55</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
@@ -32613,11 +32625,11 @@
         <v>2537</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>55</v>
+        <v>2538</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>2538</v>
+        <v>2539</v>
       </c>
       <c r="E11" s="21" t="s">
         <v>22</v>
@@ -32632,14 +32644,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2539</v>
+        <v>2540</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>55</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2540</v>
+        <v>2541</v>
       </c>
       <c r="E12" s="21" t="s">
         <v>22</v>
@@ -32654,14 +32666,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>666</v>
+        <v>55</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="E13" s="21" t="s">
         <v>22</v>
@@ -32676,14 +32688,14 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>12</v>
+        <v>666</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="E14" s="21" t="s">
         <v>22</v>
@@ -32698,21 +32710,19 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>666</v>
+        <v>12</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
       <c r="E15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
+      <c r="F15"/>
       <c r="H15" s="21" t="s">
         <v>16</v>
       </c>
@@ -32722,19 +32732,21 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>12</v>
+        <v>666</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
       <c r="E16" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F16"/>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
       <c r="H16" s="21" t="s">
         <v>16</v>
       </c>
@@ -32744,14 +32756,14 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>2551</v>
       </c>
       <c r="E17" s="21" t="s">
         <v>22</v>
@@ -32766,7 +32778,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2550</v>
+        <v>2552</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>42</v>
@@ -32788,7 +32800,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
       <c r="B19" s="21" t="s">
         <v>42</v>
@@ -32808,47 +32820,54 @@
       <c r="J19"/>
       <c r="K19"/>
     </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>156</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>4</v>
-      </c>
-      <c r="E21" t="s">
-        <v>166</v>
-      </c>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>2554</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20"/>
+      <c r="H20" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
         <v>2517</v>
       </c>
-      <c r="B22" t="s">
-        <v>2552</v>
-      </c>
-      <c r="C22" t="s">
-        <v>2553</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23"/>
       <c r="B23" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
       <c r="C23" t="s">
-        <v>2555</v>
+        <v>2556</v>
       </c>
       <c r="D23" t="s">
         <v>22</v>
@@ -32860,10 +32879,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>2556</v>
+        <v>2557</v>
       </c>
       <c r="C24" t="s">
-        <v>2557</v>
+        <v>2558</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -32875,10 +32894,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>2558</v>
+        <v>2559</v>
       </c>
       <c r="C25" t="s">
-        <v>2559</v>
+        <v>2560</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -32887,57 +32906,57 @@
         <v>22</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26"/>
+      <c r="B26" t="s">
+        <v>2561</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2562</v>
+      </c>
+      <c r="D26" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="27">
-      <c r="A27" t="s">
+      <c r="A27"/>
+      <c r="B27" t="s">
+        <v>2563</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2525</v>
+      </c>
+      <c r="D27" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
         <v>1</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B29" t="s">
         <v>156</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C29" t="s">
         <v>3</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D29" t="s">
         <v>4</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E29" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>2524</v>
-      </c>
-      <c r="B28" t="s">
-        <v>2560</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2561</v>
-      </c>
-      <c r="D28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29"/>
-      <c r="B29" t="s">
-        <v>2562</v>
-      </c>
-      <c r="C29" t="s">
-        <v>2563</v>
-      </c>
-      <c r="D29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" t="s">
-        <v>22</v>
-      </c>
-    </row>
     <row r="30">
-      <c r="A30"/>
+      <c r="A30" t="s">
+        <v>2527</v>
+      </c>
       <c r="B30" t="s">
         <v>2564</v>
       </c>
@@ -32984,10 +33003,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>965</v>
+        <v>2570</v>
       </c>
       <c r="C33" t="s">
-        <v>2570</v>
+        <v>2571</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -32999,10 +33018,10 @@
     <row r="34">
       <c r="A34"/>
       <c r="B34" t="s">
-        <v>2571</v>
+        <v>2572</v>
       </c>
       <c r="C34" t="s">
-        <v>2572</v>
+        <v>2573</v>
       </c>
       <c r="D34" t="s">
         <v>22</v>
@@ -33014,7 +33033,7 @@
     <row r="35">
       <c r="A35"/>
       <c r="B35" t="s">
-        <v>2573</v>
+        <v>965</v>
       </c>
       <c r="C35" t="s">
         <v>2574</v>
@@ -33254,10 +33273,10 @@
     <row r="51">
       <c r="A51"/>
       <c r="B51" t="s">
-        <v>177</v>
+        <v>2605</v>
       </c>
       <c r="C51" t="s">
-        <v>2605</v>
+        <v>2606</v>
       </c>
       <c r="D51" t="s">
         <v>22</v>
@@ -33269,10 +33288,10 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>2606</v>
+        <v>2607</v>
       </c>
       <c r="C52" t="s">
-        <v>2607</v>
+        <v>2608</v>
       </c>
       <c r="D52" t="s">
         <v>22</v>
@@ -33284,7 +33303,7 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>2608</v>
+        <v>177</v>
       </c>
       <c r="C53" t="s">
         <v>2609</v>
@@ -33311,57 +33330,57 @@
         <v>22</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55"/>
+      <c r="B55" t="s">
+        <v>2612</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2613</v>
+      </c>
+      <c r="D55" t="s">
+        <v>22</v>
+      </c>
+      <c r="E55" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="56">
-      <c r="A56" t="s">
+      <c r="A56"/>
+      <c r="B56" t="s">
+        <v>2614</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2615</v>
+      </c>
+      <c r="D56" t="s">
+        <v>22</v>
+      </c>
+      <c r="E56" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
         <v>1</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B58" t="s">
         <v>156</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C58" t="s">
         <v>3</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D58" t="s">
         <v>4</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E58" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="s">
-        <v>2528</v>
-      </c>
-      <c r="B57" t="s">
-        <v>2612</v>
-      </c>
-      <c r="C57" t="s">
-        <v>2613</v>
-      </c>
-      <c r="D57" t="s">
-        <v>22</v>
-      </c>
-      <c r="E57" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58"/>
-      <c r="B58" t="s">
-        <v>2614</v>
-      </c>
-      <c r="C58" t="s">
-        <v>2615</v>
-      </c>
-      <c r="D58" t="s">
-        <v>22</v>
-      </c>
-      <c r="E58" t="s">
-        <v>22</v>
-      </c>
-    </row>
     <row r="59">
-      <c r="A59"/>
+      <c r="A59" t="s">
+        <v>2531</v>
+      </c>
       <c r="B59" t="s">
         <v>2616</v>
       </c>
@@ -33375,62 +33394,62 @@
         <v>22</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60"/>
+      <c r="B60" t="s">
+        <v>2618</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2619</v>
+      </c>
+      <c r="D60" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="61">
-      <c r="A61" t="s">
+      <c r="A61"/>
+      <c r="B61" t="s">
+        <v>2620</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2621</v>
+      </c>
+      <c r="D61" t="s">
+        <v>22</v>
+      </c>
+      <c r="E61" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
         <v>1</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B63" t="s">
         <v>156</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C63" t="s">
         <v>3</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D63" t="s">
         <v>4</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E63" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="s">
-        <v>2535</v>
-      </c>
-      <c r="B62" t="s">
+    <row r="64">
+      <c r="A64" t="s">
+        <v>2538</v>
+      </c>
+      <c r="B64" t="s">
         <v>988</v>
       </c>
-      <c r="C62" t="s">
-        <v>2618</v>
-      </c>
-      <c r="D62" t="s">
-        <v>22</v>
-      </c>
-      <c r="E62" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63"/>
-      <c r="B63" t="s">
-        <v>991</v>
-      </c>
-      <c r="C63" t="s">
-        <v>2619</v>
-      </c>
-      <c r="D63" t="s">
-        <v>22</v>
-      </c>
-      <c r="E63" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64"/>
-      <c r="B64" t="s">
-        <v>2620</v>
-      </c>
       <c r="C64" t="s">
-        <v>2621</v>
+        <v>2622</v>
       </c>
       <c r="D64" t="s">
         <v>22</v>
@@ -33442,7 +33461,7 @@
     <row r="65">
       <c r="A65"/>
       <c r="B65" t="s">
-        <v>2622</v>
+        <v>991</v>
       </c>
       <c r="C65" t="s">
         <v>2623</v>
@@ -33451,6 +33470,36 @@
         <v>22</v>
       </c>
       <c r="E65" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66"/>
+      <c r="B66" t="s">
+        <v>2624</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2625</v>
+      </c>
+      <c r="D66" t="s">
+        <v>22</v>
+      </c>
+      <c r="E66" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67"/>
+      <c r="B67" t="s">
+        <v>2626</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2627</v>
+      </c>
+      <c r="D67" t="s">
+        <v>22</v>
+      </c>
+      <c r="E67" t="s">
         <v>22</v>
       </c>
     </row>
@@ -33521,7 +33570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2624</v>
+        <v>2628</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>2520</v>
@@ -33543,17 +33592,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2625</v>
+        <v>2629</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>2626</v>
+        <v>2630</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2627</v>
+        <v>2631</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>2628</v>
+        <v>2632</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -33567,14 +33616,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2629</v>
+        <v>2633</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>2630</v>
+        <v>2634</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2631</v>
+        <v>2635</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>22</v>
@@ -33589,12 +33638,12 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2632</v>
+        <v>2636</v>
       </c>
       <c r="B5" s="22"/>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2633</v>
+        <v>2637</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>22</v>
@@ -33609,10 +33658,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2634</v>
+        <v>2638</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>2635</v>
+        <v>2639</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
@@ -33631,14 +33680,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2636</v>
+        <v>2640</v>
       </c>
       <c r="B7" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2637</v>
+        <v>2641</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>22</v>
@@ -33653,14 +33702,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2638</v>
+        <v>2642</v>
       </c>
       <c r="B8" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2639</v>
+        <v>2643</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>22</v>
@@ -33675,14 +33724,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2640</v>
+        <v>2644</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>2641</v>
+        <v>2645</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2642</v>
+        <v>2646</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>22</v>
@@ -33741,14 +33790,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2643</v>
+        <v>2647</v>
       </c>
       <c r="B12" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2644</v>
+        <v>2648</v>
       </c>
       <c r="E12" s="22" t="s">
         <v>22</v>
@@ -33763,7 +33812,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2645</v>
+        <v>2649</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>12</v>
@@ -33773,7 +33822,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>2646</v>
+        <v>2650</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -33787,14 +33836,14 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2647</v>
+        <v>2651</v>
       </c>
       <c r="B14" s="22" t="s">
         <v>691</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>2648</v>
+        <v>2652</v>
       </c>
       <c r="E14" s="22" t="s">
         <v>22</v>
@@ -33816,10 +33865,10 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2649</v>
+        <v>2653</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>2650</v>
+        <v>2654</v>
       </c>
       <c r="F15"/>
       <c r="H15" s="22" t="s">
@@ -33838,10 +33887,10 @@
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2651</v>
+        <v>2655</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>2652</v>
+        <v>2656</v>
       </c>
       <c r="F16"/>
       <c r="H16" s="22" t="s">
@@ -33901,14 +33950,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2653</v>
+        <v>2657</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2654</v>
+        <v>2658</v>
       </c>
       <c r="E19" s="22" t="s">
         <v>22</v>
@@ -33923,14 +33972,14 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2655</v>
+        <v>2659</v>
       </c>
       <c r="B20" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>2656</v>
+        <v>2660</v>
       </c>
       <c r="E20" s="22" t="s">
         <v>22</v>
@@ -33945,7 +33994,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>2657</v>
+        <v>2661</v>
       </c>
       <c r="B21" s="22" t="s">
         <v>110</v>
@@ -33977,7 +34026,7 @@
         <v>1158</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>2658</v>
+        <v>2662</v>
       </c>
       <c r="F22"/>
       <c r="H22" s="22" t="s">
@@ -34057,14 +34106,14 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>2659</v>
+        <v>2663</v>
       </c>
       <c r="B26" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C26"/>
       <c r="D26" t="s">
-        <v>2660</v>
+        <v>2664</v>
       </c>
       <c r="E26" s="22" t="s">
         <v>22</v>
@@ -34101,14 +34150,14 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2661</v>
+        <v>2665</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>2662</v>
+        <v>2666</v>
       </c>
       <c r="C28"/>
       <c r="D28" t="s">
-        <v>2663</v>
+        <v>2667</v>
       </c>
       <c r="E28" s="22" t="s">
         <v>22</v>
@@ -34123,14 +34172,14 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>2664</v>
+        <v>2668</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>2665</v>
+        <v>2669</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>2666</v>
+        <v>2670</v>
       </c>
       <c r="E29" s="22" t="s">
         <v>22</v>
@@ -34145,14 +34194,14 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>2667</v>
+        <v>2671</v>
       </c>
       <c r="B30" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>2668</v>
+        <v>2672</v>
       </c>
       <c r="E30" s="22" t="s">
         <v>22</v>
@@ -34167,17 +34216,17 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2669</v>
+        <v>2673</v>
       </c>
       <c r="B31" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>2670</v>
+        <v>2674</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>2671</v>
+        <v>2675</v>
       </c>
       <c r="F31"/>
       <c r="H31" s="22" t="s">
@@ -34189,17 +34238,17 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>2672</v>
+        <v>2676</v>
       </c>
       <c r="B32" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C32"/>
       <c r="D32" t="s">
-        <v>2673</v>
+        <v>2677</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>2674</v>
+        <v>2678</v>
       </c>
       <c r="F32"/>
       <c r="H32" s="22" t="s">
@@ -34211,17 +34260,17 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>2675</v>
+        <v>2679</v>
       </c>
       <c r="B33" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C33"/>
       <c r="D33" t="s">
-        <v>2676</v>
+        <v>2680</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>2677</v>
+        <v>2681</v>
       </c>
       <c r="F33"/>
       <c r="H33" s="22" t="s">
@@ -34233,7 +34282,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>2678</v>
+        <v>2682</v>
       </c>
       <c r="B34" s="22" t="s">
         <v>12</v>
@@ -34243,7 +34292,7 @@
         <v>566</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>2679</v>
+        <v>2683</v>
       </c>
       <c r="F34"/>
       <c r="H34" s="22" t="s">
@@ -34255,17 +34304,17 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>2680</v>
+        <v>2684</v>
       </c>
       <c r="B35" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>2681</v>
+        <v>2685</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>2682</v>
+        <v>2686</v>
       </c>
       <c r="F35"/>
       <c r="H35" s="22" t="s">
@@ -34277,17 +34326,17 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2683</v>
+        <v>2687</v>
       </c>
       <c r="B36" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C36"/>
       <c r="D36" t="s">
-        <v>2684</v>
+        <v>2688</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>2685</v>
+        <v>2689</v>
       </c>
       <c r="F36"/>
       <c r="H36" s="22" t="s">
@@ -34299,17 +34348,17 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>2686</v>
+        <v>2690</v>
       </c>
       <c r="B37" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C37"/>
       <c r="D37" t="s">
-        <v>2687</v>
+        <v>2691</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>2688</v>
+        <v>2692</v>
       </c>
       <c r="F37"/>
       <c r="H37" s="22" t="s">
@@ -34385,7 +34434,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>2689</v>
+        <v>2693</v>
       </c>
       <c r="B41" s="22" t="s">
         <v>666</v>
@@ -34409,14 +34458,14 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>2690</v>
+        <v>2694</v>
       </c>
       <c r="B42" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C42"/>
       <c r="D42" t="s">
-        <v>2691</v>
+        <v>2695</v>
       </c>
       <c r="E42" s="22" t="s">
         <v>22</v>
@@ -34497,14 +34546,14 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>2692</v>
+        <v>2696</v>
       </c>
       <c r="B46" s="22" t="s">
         <v>691</v>
       </c>
       <c r="C46"/>
       <c r="D46" t="s">
-        <v>2693</v>
+        <v>2697</v>
       </c>
       <c r="E46" s="22" t="s">
         <v>22</v>
@@ -34519,14 +34568,14 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>2694</v>
+        <v>2698</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>2695</v>
+        <v>2699</v>
       </c>
       <c r="C47"/>
       <c r="D47" t="s">
-        <v>2696</v>
+        <v>2700</v>
       </c>
       <c r="E47" s="22" t="s">
         <v>22</v>
@@ -34541,17 +34590,17 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>2697</v>
+        <v>2701</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>2698</v>
+        <v>2702</v>
       </c>
       <c r="C48"/>
       <c r="D48" t="s">
-        <v>2699</v>
+        <v>2703</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>2700</v>
+        <v>2704</v>
       </c>
       <c r="F48"/>
       <c r="H48" s="22" t="s">
@@ -34565,14 +34614,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>2701</v>
+        <v>2705</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>2702</v>
+        <v>2706</v>
       </c>
       <c r="C49"/>
       <c r="D49" t="s">
-        <v>2703</v>
+        <v>2707</v>
       </c>
       <c r="E49" s="22" t="s">
         <v>22</v>
@@ -34589,14 +34638,14 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>2704</v>
+        <v>2708</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>2705</v>
+        <v>2709</v>
       </c>
       <c r="C50"/>
       <c r="D50" t="s">
-        <v>2706</v>
+        <v>2710</v>
       </c>
       <c r="E50" s="22" t="s">
         <v>22</v>
@@ -34613,14 +34662,14 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>2707</v>
+        <v>2711</v>
       </c>
       <c r="B51" s="22" t="s">
-        <v>2708</v>
+        <v>2712</v>
       </c>
       <c r="C51"/>
       <c r="D51" t="s">
-        <v>2709</v>
+        <v>2713</v>
       </c>
       <c r="E51" s="22" t="s">
         <v>22</v>
@@ -34637,14 +34686,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>2710</v>
+        <v>2714</v>
       </c>
       <c r="B52" s="22" t="s">
         <v>691</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>2711</v>
+        <v>2715</v>
       </c>
       <c r="E52" s="22" t="s">
         <v>22</v>
@@ -34661,7 +34710,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>2712</v>
+        <v>2716</v>
       </c>
       <c r="B53" s="22"/>
       <c r="C53"/>
@@ -34683,14 +34732,14 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>2713</v>
+        <v>2717</v>
       </c>
       <c r="B54" s="22" t="s">
         <v>691</v>
       </c>
       <c r="C54"/>
       <c r="D54" t="s">
-        <v>2714</v>
+        <v>2718</v>
       </c>
       <c r="E54" s="22" t="s">
         <v>22</v>
@@ -34707,7 +34756,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>2715</v>
+        <v>2719</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55"/>
@@ -34797,14 +34846,14 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>2716</v>
+        <v>2720</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>2717</v>
+        <v>2721</v>
       </c>
       <c r="C59"/>
       <c r="D59" t="s">
-        <v>2718</v>
+        <v>2722</v>
       </c>
       <c r="E59" s="22" t="s">
         <v>22</v>
@@ -34836,13 +34885,13 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>2626</v>
+        <v>2630</v>
       </c>
       <c r="B62" t="s">
-        <v>2719</v>
+        <v>2723</v>
       </c>
       <c r="C62" t="s">
-        <v>2720</v>
+        <v>2724</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -34854,10 +34903,10 @@
     <row r="63">
       <c r="A63"/>
       <c r="B63" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="C63" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="D63" t="s">
         <v>22</v>
@@ -34884,10 +34933,10 @@
     <row r="65">
       <c r="A65"/>
       <c r="B65" t="s">
-        <v>2721</v>
+        <v>2725</v>
       </c>
       <c r="C65" t="s">
-        <v>2722</v>
+        <v>2726</v>
       </c>
       <c r="D65" t="s">
         <v>22</v>
@@ -34930,13 +34979,13 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>2630</v>
+        <v>2634</v>
       </c>
       <c r="B69" t="s">
-        <v>2616</v>
+        <v>2620</v>
       </c>
       <c r="C69" t="s">
-        <v>2723</v>
+        <v>2727</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
@@ -34948,10 +34997,10 @@
     <row r="70">
       <c r="A70"/>
       <c r="B70" t="s">
-        <v>2724</v>
+        <v>2728</v>
       </c>
       <c r="C70" t="s">
-        <v>2725</v>
+        <v>2729</v>
       </c>
       <c r="D70" t="s">
         <v>22</v>
@@ -34963,10 +35012,10 @@
     <row r="71">
       <c r="A71"/>
       <c r="B71" t="s">
-        <v>2612</v>
+        <v>2616</v>
       </c>
       <c r="C71" t="s">
-        <v>2726</v>
+        <v>2730</v>
       </c>
       <c r="D71" t="s">
         <v>22</v>
@@ -35009,7 +35058,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>2635</v>
+        <v>2639</v>
       </c>
       <c r="B75" t="s">
         <v>988</v>
@@ -35027,10 +35076,10 @@
     <row r="76">
       <c r="A76"/>
       <c r="B76" t="s">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="C76" t="s">
-        <v>2728</v>
+        <v>2732</v>
       </c>
       <c r="D76" t="s">
         <v>22</v>
@@ -35088,7 +35137,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>2641</v>
+        <v>2645</v>
       </c>
       <c r="B81" t="s">
         <v>988</v>
@@ -35106,7 +35155,7 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="C82" t="s">
         <v>1106</v>
@@ -35136,10 +35185,10 @@
     <row r="84">
       <c r="A84"/>
       <c r="B84" t="s">
-        <v>2729</v>
+        <v>2733</v>
       </c>
       <c r="C84" t="s">
-        <v>2730</v>
+        <v>2734</v>
       </c>
       <c r="D84" t="s">
         <v>22</v>
@@ -35633,13 +35682,13 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>2662</v>
+        <v>2666</v>
       </c>
       <c r="B121" t="s">
-        <v>2731</v>
+        <v>2735</v>
       </c>
       <c r="C121" t="s">
-        <v>2732</v>
+        <v>2736</v>
       </c>
       <c r="D121" t="s">
         <v>22</v>
@@ -35651,10 +35700,10 @@
     <row r="122">
       <c r="A122"/>
       <c r="B122" t="s">
-        <v>2733</v>
+        <v>2737</v>
       </c>
       <c r="C122" t="s">
-        <v>2734</v>
+        <v>2738</v>
       </c>
       <c r="D122" t="s">
         <v>22</v>
@@ -35666,10 +35715,10 @@
     <row r="123">
       <c r="A123"/>
       <c r="B123" t="s">
-        <v>2735</v>
+        <v>2739</v>
       </c>
       <c r="C123" t="s">
-        <v>2736</v>
+        <v>2740</v>
       </c>
       <c r="D123" t="s">
         <v>22</v>
@@ -35681,10 +35730,10 @@
     <row r="124">
       <c r="A124"/>
       <c r="B124" t="s">
-        <v>2737</v>
+        <v>2741</v>
       </c>
       <c r="C124" t="s">
-        <v>2738</v>
+        <v>2742</v>
       </c>
       <c r="D124" t="s">
         <v>22</v>
@@ -35696,10 +35745,10 @@
     <row r="125">
       <c r="A125"/>
       <c r="B125" t="s">
-        <v>2739</v>
+        <v>2743</v>
       </c>
       <c r="C125" t="s">
-        <v>2740</v>
+        <v>2744</v>
       </c>
       <c r="D125" t="s">
         <v>22</v>
@@ -35727,13 +35776,13 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>2665</v>
+        <v>2669</v>
       </c>
       <c r="B128" t="s">
-        <v>2741</v>
+        <v>2745</v>
       </c>
       <c r="C128" t="s">
-        <v>2742</v>
+        <v>2746</v>
       </c>
       <c r="D128" t="s">
         <v>22</v>
@@ -35745,10 +35794,10 @@
     <row r="129">
       <c r="A129"/>
       <c r="B129" t="s">
-        <v>2743</v>
+        <v>2747</v>
       </c>
       <c r="C129" t="s">
-        <v>2744</v>
+        <v>2748</v>
       </c>
       <c r="D129" t="s">
         <v>22</v>
@@ -35760,10 +35809,10 @@
     <row r="130">
       <c r="A130"/>
       <c r="B130" t="s">
-        <v>2745</v>
+        <v>2749</v>
       </c>
       <c r="C130" t="s">
-        <v>2746</v>
+        <v>2750</v>
       </c>
       <c r="D130" t="s">
         <v>22</v>
@@ -35775,10 +35824,10 @@
     <row r="131">
       <c r="A131"/>
       <c r="B131" t="s">
-        <v>2747</v>
+        <v>2751</v>
       </c>
       <c r="C131" t="s">
-        <v>2748</v>
+        <v>2752</v>
       </c>
       <c r="D131" t="s">
         <v>22</v>
@@ -35790,10 +35839,10 @@
     <row r="132">
       <c r="A132"/>
       <c r="B132" t="s">
-        <v>2749</v>
+        <v>2753</v>
       </c>
       <c r="C132" t="s">
-        <v>2750</v>
+        <v>2754</v>
       </c>
       <c r="D132" t="s">
         <v>22</v>
@@ -36695,13 +36744,13 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>2695</v>
+        <v>2699</v>
       </c>
       <c r="B194" t="s">
-        <v>2751</v>
+        <v>2755</v>
       </c>
       <c r="C194" t="s">
-        <v>2752</v>
+        <v>2756</v>
       </c>
       <c r="D194" t="s">
         <v>22</v>
@@ -36716,7 +36765,7 @@
         <v>2354</v>
       </c>
       <c r="C195" t="s">
-        <v>2753</v>
+        <v>2757</v>
       </c>
       <c r="D195" t="s">
         <v>22</v>
@@ -36731,7 +36780,7 @@
         <v>2356</v>
       </c>
       <c r="C196" t="s">
-        <v>2754</v>
+        <v>2758</v>
       </c>
       <c r="D196" t="s">
         <v>22</v>
@@ -36743,10 +36792,10 @@
     <row r="197">
       <c r="A197"/>
       <c r="B197" t="s">
-        <v>2755</v>
+        <v>2759</v>
       </c>
       <c r="C197" t="s">
-        <v>2756</v>
+        <v>2760</v>
       </c>
       <c r="D197" t="s">
         <v>22</v>
@@ -36758,10 +36807,10 @@
     <row r="198">
       <c r="A198"/>
       <c r="B198" t="s">
-        <v>2757</v>
+        <v>2761</v>
       </c>
       <c r="C198" t="s">
-        <v>2758</v>
+        <v>2762</v>
       </c>
       <c r="D198" t="s">
         <v>22</v>
@@ -36804,7 +36853,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>2698</v>
+        <v>2702</v>
       </c>
       <c r="B202" t="s">
         <v>941</v>
@@ -36883,13 +36932,13 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>2702</v>
+        <v>2706</v>
       </c>
       <c r="B208" t="s">
-        <v>2759</v>
+        <v>2763</v>
       </c>
       <c r="C208" t="s">
-        <v>2760</v>
+        <v>2764</v>
       </c>
       <c r="D208" t="s">
         <v>22</v>
@@ -36901,10 +36950,10 @@
     <row r="209">
       <c r="A209"/>
       <c r="B209" t="s">
-        <v>2761</v>
+        <v>2765</v>
       </c>
       <c r="C209" t="s">
-        <v>2762</v>
+        <v>2766</v>
       </c>
       <c r="D209" t="s">
         <v>22</v>
@@ -36916,10 +36965,10 @@
     <row r="210">
       <c r="A210"/>
       <c r="B210" t="s">
-        <v>2763</v>
+        <v>2767</v>
       </c>
       <c r="C210" t="s">
-        <v>2764</v>
+        <v>2768</v>
       </c>
       <c r="D210" t="s">
         <v>22</v>
@@ -36931,10 +36980,10 @@
     <row r="211">
       <c r="A211"/>
       <c r="B211" t="s">
-        <v>2765</v>
+        <v>2769</v>
       </c>
       <c r="C211" t="s">
-        <v>2766</v>
+        <v>2770</v>
       </c>
       <c r="D211" t="s">
         <v>22</v>
@@ -36946,10 +36995,10 @@
     <row r="212">
       <c r="A212"/>
       <c r="B212" t="s">
-        <v>2767</v>
+        <v>2771</v>
       </c>
       <c r="C212" t="s">
-        <v>2768</v>
+        <v>2772</v>
       </c>
       <c r="D212" t="s">
         <v>22</v>
@@ -36961,10 +37010,10 @@
     <row r="213">
       <c r="A213"/>
       <c r="B213" t="s">
-        <v>2769</v>
+        <v>2773</v>
       </c>
       <c r="C213" t="s">
-        <v>2770</v>
+        <v>2774</v>
       </c>
       <c r="D213" t="s">
         <v>22</v>
@@ -37007,13 +37056,13 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>2705</v>
+        <v>2709</v>
       </c>
       <c r="B217" t="s">
-        <v>2771</v>
+        <v>2775</v>
       </c>
       <c r="C217" t="s">
-        <v>2772</v>
+        <v>2776</v>
       </c>
       <c r="D217" t="s">
         <v>22</v>
@@ -37025,10 +37074,10 @@
     <row r="218">
       <c r="A218"/>
       <c r="B218" t="s">
-        <v>2773</v>
+        <v>2777</v>
       </c>
       <c r="C218" t="s">
-        <v>2774</v>
+        <v>2778</v>
       </c>
       <c r="D218" t="s">
         <v>22</v>
@@ -37040,10 +37089,10 @@
     <row r="219">
       <c r="A219"/>
       <c r="B219" t="s">
-        <v>2775</v>
+        <v>2779</v>
       </c>
       <c r="C219" t="s">
-        <v>2776</v>
+        <v>2780</v>
       </c>
       <c r="D219" t="s">
         <v>22</v>
@@ -37055,10 +37104,10 @@
     <row r="220">
       <c r="A220"/>
       <c r="B220" t="s">
-        <v>2777</v>
+        <v>2781</v>
       </c>
       <c r="C220" t="s">
-        <v>2778</v>
+        <v>2782</v>
       </c>
       <c r="D220" t="s">
         <v>22</v>
@@ -37070,10 +37119,10 @@
     <row r="221">
       <c r="A221"/>
       <c r="B221" t="s">
-        <v>2779</v>
+        <v>2783</v>
       </c>
       <c r="C221" t="s">
-        <v>2780</v>
+        <v>2784</v>
       </c>
       <c r="D221" t="s">
         <v>22</v>
@@ -37116,13 +37165,13 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>2708</v>
+        <v>2712</v>
       </c>
       <c r="B225" t="s">
-        <v>2781</v>
+        <v>2785</v>
       </c>
       <c r="C225" t="s">
-        <v>2782</v>
+        <v>2786</v>
       </c>
       <c r="D225" t="s">
         <v>22</v>
@@ -37134,10 +37183,10 @@
     <row r="226">
       <c r="A226"/>
       <c r="B226" t="s">
-        <v>2783</v>
+        <v>2787</v>
       </c>
       <c r="C226" t="s">
-        <v>2784</v>
+        <v>2788</v>
       </c>
       <c r="D226" t="s">
         <v>22</v>
@@ -37149,10 +37198,10 @@
     <row r="227">
       <c r="A227"/>
       <c r="B227" t="s">
-        <v>2785</v>
+        <v>2789</v>
       </c>
       <c r="C227" t="s">
-        <v>2786</v>
+        <v>2790</v>
       </c>
       <c r="D227" t="s">
         <v>22</v>
@@ -37164,10 +37213,10 @@
     <row r="228">
       <c r="A228"/>
       <c r="B228" t="s">
-        <v>2787</v>
+        <v>2791</v>
       </c>
       <c r="C228" t="s">
-        <v>2788</v>
+        <v>2792</v>
       </c>
       <c r="D228" t="s">
         <v>22</v>
@@ -37179,10 +37228,10 @@
     <row r="229">
       <c r="A229"/>
       <c r="B229" t="s">
-        <v>2789</v>
+        <v>2793</v>
       </c>
       <c r="C229" t="s">
-        <v>2790</v>
+        <v>2794</v>
       </c>
       <c r="D229" t="s">
         <v>22</v>
@@ -37210,7 +37259,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>2717</v>
+        <v>2721</v>
       </c>
       <c r="B232" t="s">
         <v>183</v>
@@ -37228,10 +37277,10 @@
     <row r="233">
       <c r="A233"/>
       <c r="B233" t="s">
-        <v>2791</v>
+        <v>2795</v>
       </c>
       <c r="C233" t="s">
-        <v>2792</v>
+        <v>2796</v>
       </c>
       <c r="D233" t="s">
         <v>22</v>
@@ -37243,10 +37292,10 @@
     <row r="234">
       <c r="A234"/>
       <c r="B234" t="s">
-        <v>2793</v>
+        <v>2797</v>
       </c>
       <c r="C234" t="s">
-        <v>2794</v>
+        <v>2798</v>
       </c>
       <c r="D234" t="s">
         <v>22</v>
@@ -37364,7 +37413,7 @@
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="E3" s="23" t="s">
         <v>22</v>
@@ -37405,7 +37454,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2795</v>
+        <v>2799</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>12</v>
@@ -37414,7 +37463,7 @@
         <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>2796</v>
+        <v>2800</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>22</v>
@@ -37622,14 +37671,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2797</v>
+        <v>2801</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>2798</v>
+        <v>2802</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2799</v>
+        <v>2803</v>
       </c>
       <c r="E2" s="24" t="s">
         <v>22</v>
@@ -37668,14 +37717,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2800</v>
+        <v>2804</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>2801</v>
+        <v>2805</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2802</v>
+        <v>2806</v>
       </c>
       <c r="E4" s="24" t="s">
         <v>22</v>
@@ -37690,14 +37739,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>2803</v>
+        <v>2807</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="E5" s="24" t="s">
         <v>22</v>
@@ -37712,7 +37761,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2804</v>
+        <v>2808</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>55</v>
@@ -37736,14 +37785,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2805</v>
+        <v>2809</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>2806</v>
+        <v>2810</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2807</v>
+        <v>2811</v>
       </c>
       <c r="E7" s="24" t="s">
         <v>22</v>
@@ -37758,7 +37807,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>55</v>
@@ -37780,14 +37829,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>666</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="E9" s="24" t="s">
         <v>22</v>
@@ -37802,14 +37851,14 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2808</v>
+        <v>2812</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>2644</v>
+        <v>2648</v>
       </c>
       <c r="E10" s="24" t="s">
         <v>22</v>
@@ -37846,14 +37895,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2809</v>
+        <v>2813</v>
       </c>
       <c r="B12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="E12" s="24" t="s">
         <v>22</v>
@@ -37868,14 +37917,14 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2810</v>
+        <v>2814</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>666</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>2811</v>
+        <v>2815</v>
       </c>
       <c r="E13" s="24" t="s">
         <v>22</v>
@@ -37907,13 +37956,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2798</v>
+        <v>2802</v>
       </c>
       <c r="B16" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="C16" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="D16" t="s">
         <v>22</v>
@@ -37941,13 +37990,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2801</v>
+        <v>2805</v>
       </c>
       <c r="B19" t="s">
-        <v>2812</v>
+        <v>2816</v>
       </c>
       <c r="C19" t="s">
-        <v>2813</v>
+        <v>2817</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -37959,10 +38008,10 @@
     <row r="20">
       <c r="A20"/>
       <c r="B20" t="s">
-        <v>2575</v>
+        <v>2579</v>
       </c>
       <c r="C20" t="s">
-        <v>2814</v>
+        <v>2818</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -37974,10 +38023,10 @@
     <row r="21">
       <c r="A21"/>
       <c r="B21" t="s">
-        <v>2815</v>
+        <v>2819</v>
       </c>
       <c r="C21" t="s">
-        <v>2816</v>
+        <v>2820</v>
       </c>
       <c r="D21" t="s">
         <v>22</v>
@@ -37989,10 +38038,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>2579</v>
+        <v>2583</v>
       </c>
       <c r="C22" t="s">
-        <v>2817</v>
+        <v>2821</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -38004,10 +38053,10 @@
     <row r="23">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>2818</v>
+        <v>2822</v>
       </c>
       <c r="C23" t="s">
-        <v>2819</v>
+        <v>2823</v>
       </c>
       <c r="D23" t="s">
         <v>22</v>
@@ -38019,10 +38068,10 @@
     <row r="24">
       <c r="A24"/>
       <c r="B24" t="s">
-        <v>2820</v>
+        <v>2824</v>
       </c>
       <c r="C24" t="s">
-        <v>2821</v>
+        <v>2825</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -38034,10 +38083,10 @@
     <row r="25">
       <c r="A25"/>
       <c r="B25" t="s">
-        <v>2822</v>
+        <v>2826</v>
       </c>
       <c r="C25" t="s">
-        <v>2823</v>
+        <v>2827</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -38049,10 +38098,10 @@
     <row r="26">
       <c r="A26"/>
       <c r="B26" t="s">
-        <v>2824</v>
+        <v>2828</v>
       </c>
       <c r="C26" t="s">
-        <v>2825</v>
+        <v>2829</v>
       </c>
       <c r="D26" t="s">
         <v>22</v>
@@ -38064,10 +38113,10 @@
     <row r="27">
       <c r="A27"/>
       <c r="B27" t="s">
-        <v>2826</v>
+        <v>2830</v>
       </c>
       <c r="C27" t="s">
-        <v>2827</v>
+        <v>2831</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -38110,13 +38159,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>2803</v>
+        <v>2807</v>
       </c>
       <c r="B31" t="s">
-        <v>2612</v>
+        <v>2616</v>
       </c>
       <c r="C31" t="s">
-        <v>2613</v>
+        <v>2617</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -38128,10 +38177,10 @@
     <row r="32">
       <c r="A32"/>
       <c r="B32" t="s">
-        <v>2614</v>
+        <v>2618</v>
       </c>
       <c r="C32" t="s">
-        <v>2615</v>
+        <v>2619</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -38143,10 +38192,10 @@
     <row r="33">
       <c r="A33"/>
       <c r="B33" t="s">
-        <v>2616</v>
+        <v>2620</v>
       </c>
       <c r="C33" t="s">
-        <v>2617</v>
+        <v>2621</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -38174,7 +38223,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>2806</v>
+        <v>2810</v>
       </c>
       <c r="B36" t="s">
         <v>988</v>
@@ -38192,10 +38241,10 @@
     <row r="37">
       <c r="A37"/>
       <c r="B37" t="s">
-        <v>2828</v>
+        <v>2832</v>
       </c>
       <c r="C37" t="s">
-        <v>2829</v>
+        <v>2833</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -38293,7 +38342,7 @@
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2830</v>
+        <v>2834</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>22</v>
@@ -38354,7 +38403,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B5" s="25" t="s">
         <v>134</v>
@@ -38376,7 +38425,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2832</v>
+        <v>2836</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>134</v>
@@ -38530,7 +38579,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2833</v>
+        <v>2837</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>58</v>
@@ -38552,7 +38601,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2834</v>
+        <v>2838</v>
       </c>
       <c r="B14" s="25" t="s">
         <v>62</v>
@@ -38605,7 +38654,7 @@
         <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>2835</v>
+        <v>2839</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>22</v>
@@ -38664,7 +38713,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2836</v>
+        <v>2840</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>134</v>
@@ -38686,7 +38735,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2837</v>
+        <v>2841</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>134</v>
@@ -38708,14 +38757,14 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>2838</v>
+        <v>2842</v>
       </c>
       <c r="B21" s="25" t="s">
         <v>134</v>
       </c>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>2839</v>
+        <v>2843</v>
       </c>
       <c r="E21" s="25" t="s">
         <v>22</v>
@@ -38730,10 +38779,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>2840</v>
+        <v>2844</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>2841</v>
+        <v>2845</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="s">
@@ -40260,14 +40309,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2842</v>
+        <v>2846</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2843</v>
+        <v>2847</v>
       </c>
       <c r="E2" s="26" t="s">
         <v>22</v>
@@ -40304,14 +40353,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>134</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>22</v>
@@ -40387,14 +40436,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2842</v>
+        <v>2846</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2843</v>
+        <v>2847</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>22</v>
@@ -40431,14 +40480,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>134</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E4" s="27" t="s">
         <v>22</v>
@@ -40460,7 +40509,7 @@
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2845</v>
+        <v>2849</v>
       </c>
       <c r="E5" s="27" t="s">
         <v>22</v>
@@ -40536,14 +40585,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2842</v>
+        <v>2846</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2843</v>
+        <v>2847</v>
       </c>
       <c r="E2" s="28" t="s">
         <v>22</v>
@@ -40580,14 +40629,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2846</v>
+        <v>2850</v>
       </c>
       <c r="B4" s="28" t="s">
         <v>12</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2847</v>
+        <v>2851</v>
       </c>
       <c r="E4" s="28" t="s">
         <v>22</v>
@@ -40602,14 +40651,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2848</v>
+        <v>2852</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>12</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2849</v>
+        <v>2853</v>
       </c>
       <c r="E5" s="28" t="s">
         <v>22</v>
@@ -40624,14 +40673,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B6" s="28" t="s">
         <v>134</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E6" s="28" t="s">
         <v>22</v>
@@ -40729,14 +40778,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2850</v>
+        <v>2854</v>
       </c>
       <c r="B2" s="29" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2851</v>
+        <v>2855</v>
       </c>
       <c r="E2" s="29" t="s">
         <v>22</v>
@@ -40751,14 +40800,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2852</v>
+        <v>2856</v>
       </c>
       <c r="B3" s="29" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2853</v>
+        <v>2857</v>
       </c>
       <c r="E3" s="29" t="s">
         <v>22</v>
@@ -40773,14 +40822,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2854</v>
+        <v>2858</v>
       </c>
       <c r="B4" s="29" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2855</v>
+        <v>2859</v>
       </c>
       <c r="E4" s="29" t="s">
         <v>22</v>
@@ -40795,14 +40844,14 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B5" s="29" t="s">
         <v>134</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E5" s="29" t="s">
         <v>22</v>
@@ -40839,14 +40888,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2856</v>
+        <v>2860</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>2857</v>
+        <v>2861</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2858</v>
+        <v>2862</v>
       </c>
       <c r="E7" s="29" t="s">
         <v>22</v>
@@ -42744,14 +42793,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2850</v>
+        <v>2854</v>
       </c>
       <c r="B2" s="30" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2851</v>
+        <v>2855</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>22</v>
@@ -42766,14 +42815,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2852</v>
+        <v>2856</v>
       </c>
       <c r="B3" s="30" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2853</v>
+        <v>2857</v>
       </c>
       <c r="E3" s="30" t="s">
         <v>22</v>
@@ -42788,14 +42837,14 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2854</v>
+        <v>2858</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>42</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>2855</v>
+        <v>2859</v>
       </c>
       <c r="E4" s="30" t="s">
         <v>22</v>
@@ -42832,14 +42881,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>134</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E6" s="30" t="s">
         <v>22</v>
@@ -42937,14 +42986,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2850</v>
+        <v>2854</v>
       </c>
       <c r="B2" s="31" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2851</v>
+        <v>2855</v>
       </c>
       <c r="E2" s="31" t="s">
         <v>22</v>
@@ -42959,7 +43008,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2854</v>
+        <v>2858</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>42</v>
@@ -43025,14 +43074,14 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>134</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>22</v>
@@ -43130,14 +43179,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2850</v>
+        <v>2854</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>12</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2851</v>
+        <v>2855</v>
       </c>
       <c r="E2" s="32" t="s">
         <v>22</v>
@@ -43445,7 +43494,7 @@
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2859</v>
+        <v>2863</v>
       </c>
       <c r="E16" s="32" t="s">
         <v>22</v>
@@ -43467,7 +43516,7 @@
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2860</v>
+        <v>2864</v>
       </c>
       <c r="E17" s="32" t="s">
         <v>22</v>
@@ -43482,7 +43531,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2861</v>
+        <v>2865</v>
       </c>
       <c r="B18" s="32" t="s">
         <v>69</v>
@@ -43504,14 +43553,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2862</v>
+        <v>2866</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>134</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2863</v>
+        <v>2867</v>
       </c>
       <c r="E19" s="32" t="s">
         <v>22</v>
@@ -43526,14 +43575,14 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B20" s="32" t="s">
         <v>134</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E20" s="32" t="s">
         <v>22</v>
@@ -44616,14 +44665,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2864</v>
+        <v>2868</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>2865</v>
+        <v>2869</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2866</v>
+        <v>2870</v>
       </c>
       <c r="E2" s="33" t="s">
         <v>22</v>
@@ -44638,14 +44687,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2850</v>
+        <v>2854</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2851</v>
+        <v>2855</v>
       </c>
       <c r="E3" s="33" t="s">
         <v>22</v>
@@ -44711,7 +44760,7 @@
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>2859</v>
+        <v>2863</v>
       </c>
       <c r="E6" s="33" t="s">
         <v>22</v>
@@ -44733,7 +44782,7 @@
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2860</v>
+        <v>2864</v>
       </c>
       <c r="E7" s="33" t="s">
         <v>22</v>
@@ -44748,14 +44797,14 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2867</v>
+        <v>2871</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>134</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2868</v>
+        <v>2872</v>
       </c>
       <c r="E8" s="33" t="s">
         <v>22</v>
@@ -44770,14 +44819,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2831</v>
+        <v>2835</v>
       </c>
       <c r="B9" s="33" t="s">
         <v>134</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2844</v>
+        <v>2848</v>
       </c>
       <c r="E9" s="33" t="s">
         <v>22</v>
@@ -44831,13 +44880,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2865</v>
+        <v>2869</v>
       </c>
       <c r="B13" t="s">
-        <v>2869</v>
+        <v>2873</v>
       </c>
       <c r="C13" t="s">
-        <v>2870</v>
+        <v>2874</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -44849,10 +44898,10 @@
     <row r="14">
       <c r="A14"/>
       <c r="B14" t="s">
-        <v>2871</v>
+        <v>2875</v>
       </c>
       <c r="C14" t="s">
-        <v>2872</v>
+        <v>2876</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
@@ -44864,10 +44913,10 @@
     <row r="15">
       <c r="A15"/>
       <c r="B15" t="s">
-        <v>2873</v>
+        <v>2877</v>
       </c>
       <c r="C15" t="s">
-        <v>2874</v>
+        <v>2878</v>
       </c>
       <c r="D15" t="s">
         <v>22</v>
@@ -44955,14 +45004,14 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2867</v>
+        <v>2871</v>
       </c>
       <c r="B2" s="34" t="s">
         <v>134</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>2868</v>
+        <v>2872</v>
       </c>
       <c r="E2" s="34" t="s">
         <v>22</v>
@@ -44977,14 +45026,14 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2875</v>
+        <v>2879</v>
       </c>
       <c r="B3" s="34" t="s">
         <v>12</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>2876</v>
+        <v>2880</v>
       </c>
       <c r="E3" s="34" t="s">
         <v>22</v>
@@ -45043,7 +45092,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2877</v>
+        <v>2881</v>
       </c>
       <c r="B6" s="34" t="s">
         <v>12</v>
@@ -45065,14 +45114,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2878</v>
+        <v>2882</v>
       </c>
       <c r="B7" s="34" t="s">
         <v>12</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>2879</v>
+        <v>2883</v>
       </c>
       <c r="E7" s="34" t="s">
         <v>22</v>
@@ -45094,7 +45143,7 @@
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>2880</v>
+        <v>2884</v>
       </c>
       <c r="E8" s="34" t="s">
         <v>22</v>
@@ -45109,14 +45158,14 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2881</v>
+        <v>2885</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>2882</v>
+        <v>2886</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>2883</v>
+        <v>2887</v>
       </c>
       <c r="E9" s="34" t="s">
         <v>22</v>
@@ -45219,7 +45268,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2884</v>
+        <v>2888</v>
       </c>
       <c r="B14" s="34" t="s">
         <v>72</v>
@@ -45248,7 +45297,7 @@
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>2885</v>
+        <v>2889</v>
       </c>
       <c r="E15" s="34" t="s">
         <v>22</v>
@@ -45263,14 +45312,14 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2886</v>
+        <v>2890</v>
       </c>
       <c r="B16" s="34" t="s">
         <v>666</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>2887</v>
+        <v>2891</v>
       </c>
       <c r="E16" s="34" t="s">
         <v>22</v>
@@ -45285,17 +45334,17 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2888</v>
+        <v>2892</v>
       </c>
       <c r="B17" s="34" t="s">
         <v>91</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>2889</v>
+        <v>2893</v>
       </c>
       <c r="E17" s="34" t="s">
-        <v>2890</v>
+        <v>2894</v>
       </c>
       <c r="F17"/>
       <c r="H17" s="34" t="s">
@@ -45307,10 +45356,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2891</v>
+        <v>2895</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>2892</v>
+        <v>2896</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
@@ -45329,14 +45378,14 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>2893</v>
+        <v>2897</v>
       </c>
       <c r="B19" s="34" t="s">
         <v>134</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>2894</v>
+        <v>2898</v>
       </c>
       <c r="E19" s="34" t="s">
         <v>22</v>
@@ -46279,13 +46328,13 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>2892</v>
+        <v>2896</v>
       </c>
       <c r="B85" t="s">
-        <v>2895</v>
+        <v>2899</v>
       </c>
       <c r="C85" t="s">
-        <v>2896</v>
+        <v>2900</v>
       </c>
       <c r="D85" t="s">
         <v>22</v>
@@ -46297,10 +46346,10 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>2897</v>
+        <v>2901</v>
       </c>
       <c r="C86" t="s">
-        <v>2898</v>
+        <v>2902</v>
       </c>
       <c r="D86" t="s">
         <v>22</v>
@@ -46312,10 +46361,10 @@
     <row r="87">
       <c r="A87"/>
       <c r="B87" t="s">
-        <v>2899</v>
+        <v>2903</v>
       </c>
       <c r="C87" t="s">
-        <v>2900</v>
+        <v>2904</v>
       </c>
       <c r="D87" t="s">
         <v>22</v>
@@ -46327,10 +46376,10 @@
     <row r="88">
       <c r="A88"/>
       <c r="B88" t="s">
-        <v>2901</v>
+        <v>2905</v>
       </c>
       <c r="C88" t="s">
-        <v>2902</v>
+        <v>2906</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -46342,10 +46391,10 @@
     <row r="89">
       <c r="A89"/>
       <c r="B89" t="s">
-        <v>2903</v>
+        <v>2907</v>
       </c>
       <c r="C89" t="s">
-        <v>2904</v>
+        <v>2908</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -46357,10 +46406,10 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>2905</v>
+        <v>2909</v>
       </c>
       <c r="C90" t="s">
-        <v>2906</v>
+        <v>2910</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -46372,10 +46421,10 @@
     <row r="91">
       <c r="A91"/>
       <c r="B91" t="s">
-        <v>2907</v>
+        <v>2911</v>
       </c>
       <c r="C91" t="s">
-        <v>2908</v>
+        <v>2912</v>
       </c>
       <c r="D91" t="s">
         <v>22</v>
@@ -46387,10 +46436,10 @@
     <row r="92">
       <c r="A92"/>
       <c r="B92" t="s">
-        <v>2909</v>
+        <v>2913</v>
       </c>
       <c r="C92" t="s">
-        <v>2910</v>
+        <v>2914</v>
       </c>
       <c r="D92" t="s">
         <v>22</v>
@@ -46402,10 +46451,10 @@
     <row r="93">
       <c r="A93"/>
       <c r="B93" t="s">
-        <v>2911</v>
+        <v>2915</v>
       </c>
       <c r="C93" t="s">
-        <v>2912</v>
+        <v>2916</v>
       </c>
       <c r="D93" t="s">
         <v>22</v>
@@ -46417,10 +46466,10 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>2913</v>
+        <v>2917</v>
       </c>
       <c r="C94" t="s">
-        <v>2914</v>
+        <v>2918</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -46432,10 +46481,10 @@
     <row r="95">
       <c r="A95"/>
       <c r="B95" t="s">
-        <v>2915</v>
+        <v>2919</v>
       </c>
       <c r="C95" t="s">
-        <v>2916</v>
+        <v>2920</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -46447,10 +46496,10 @@
     <row r="96">
       <c r="A96"/>
       <c r="B96" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="C96" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="D96" t="s">
         <v>22</v>
@@ -46462,10 +46511,10 @@
     <row r="97">
       <c r="A97"/>
       <c r="B97" t="s">
-        <v>2919</v>
+        <v>2923</v>
       </c>
       <c r="C97" t="s">
-        <v>2920</v>
+        <v>2924</v>
       </c>
       <c r="D97" t="s">
         <v>22</v>
@@ -46477,10 +46526,10 @@
     <row r="98">
       <c r="A98"/>
       <c r="B98" t="s">
-        <v>2921</v>
+        <v>2925</v>
       </c>
       <c r="C98" t="s">
-        <v>2922</v>
+        <v>2926</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -46492,10 +46541,10 @@
     <row r="99">
       <c r="A99"/>
       <c r="B99" t="s">
-        <v>2923</v>
+        <v>2927</v>
       </c>
       <c r="C99" t="s">
-        <v>2924</v>
+        <v>2928</v>
       </c>
       <c r="D99" t="s">
         <v>22</v>
@@ -46507,10 +46556,10 @@
     <row r="100">
       <c r="A100"/>
       <c r="B100" t="s">
-        <v>2925</v>
+        <v>2929</v>
       </c>
       <c r="C100" t="s">
-        <v>2926</v>
+        <v>2930</v>
       </c>
       <c r="D100" t="s">
         <v>22</v>
@@ -46537,12 +46586,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>2927</v>
+        <v>2931</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2928</v>
+        <v>2932</v>
       </c>
     </row>
   </sheetData>

</xml_diff>